<commit_message>
Scrape Wedding Rose Gold
</commit_message>
<xml_diff>
--- a/py_scraper/product_data.xlsx
+++ b/py_scraper/product_data.xlsx
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Ballad-Three-Quarter-Coverage-Lab-Diamond-Ring-(1/4-ct.-tw.)-White-Gold-BE264LC/</t>
+          <t>https://www.brilliantearth.com/Ballad-Three-Quarter-Coverage-Lab-Diamond-Ring-(1/4-ct.-tw.)-Rose-Gold-BE264LC/</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -463,19 +463,19 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/W4/BE264_white_top.jpeg, https://image.brilliantearth.com/media/product_new_images/4B/BE264LC_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/VP/BE5D301-18KW.jpg, https://image.brilliantearth.com/media/product_images/JR/BE264_white_side1.jpg, https://image.brilliantearth.com/media/product_images/DJ/BE264_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/C7/BE264LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/4U/BE264_rose_top.jpeg, https://image.brilliantearth.com/media/product_new_images/B8/BE264LC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/VZ/BE264.jpg, https://image.brilliantearth.com/media/product_images/ZN/BE264_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/EB/BE264LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9181249?v=1739866026</t>
+          <t>embed.imajize.com/1556546?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Nathalie-Emerald-Cut-Lab-Diamond-Ring-Gold-BE2D3425LC/</t>
+          <t>https://www.brilliantearth.com/Nathalie-Emerald-Cut-Lab-Diamond-Ring-Rose-Gold-BE2D3425LC/</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -485,19 +485,19 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/34/BE2D3425LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/FS/BE2D3425LC-18KY_009.jpg, https://image.brilliantearth.com/media/product_images/97/BE2D3425LC_yellow_side.jpg, https://image.brilliantearth.com/media/product_images/HE/BE2D3425LC_yellow_hand_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/63/BE2D3425LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/1N/BE2D3425LC_rose_F_model.JPG, https://image.brilliantearth.com/media/product_images/E3/BE2D3425LC_rose_side.jpg, https://image.brilliantearth.com/media/product_images/8M/BE2D3425LC_rose_hand_ms_zi.png</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>embed.imajize.com/4107213?v=1739866026</t>
+          <t>embed.imajize.com/4250860?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Luxe-Versailles-Lab-Diamond-Open-Ring-(1/2-ct.-tw.)-Gold-BE2D2952LC/</t>
+          <t>https://www.brilliantearth.com/Luxe-Versailles-Lab-Diamond-Open-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D2952LC/</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -507,19 +507,19 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/DE/BE2D2952_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/90/BE2D2952_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/45/BE2D2952_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/ST/BE2D2952_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/97/BE2D2952_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/07/BE2D2952_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/9A/BE2D2952_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/NV/BE2D2952_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9202459?v=1739866026</t>
+          <t>embed.imajize.com/9927334?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Sia-Half-Coverage-Lab-Diamond-Ring-(1/8-ct.-tw.)-Gold-BE2D2118PLC/</t>
+          <t>https://www.brilliantearth.com/Sia-Half-Coverage-Lab-Diamond-Ring-(1/8-ct.-tw.)-Rose-Gold-BE2D2118PLC/</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -529,19 +529,19 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/37/BE2D2118P_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/9C/BE2D2118P-yellow_2.jpg, https://image.brilliantearth.com/media/product_images/J2/BE2D2118P-yellow_4.jpg, https://image.brilliantearth.com/media/product_new_images/C9/BE2D2118P_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B8/BE2D2118P_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/AD/BE2D2118P_rose_top.jpg, https://image.brilliantearth.com/media/product_images/W3/BE2D2118P-rose_2.jpg, https://image.brilliantearth.com/media/product_images/D2/BE2D2118P-rose_4.jpg, https://image.brilliantearth.com/media/product_new_images/89/BE2D2118P_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/91/BE2D2118P_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>embed.imajize.com/7830208?v=1739866026</t>
+          <t>embed.imajize.com/9279779?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Riviera-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Gold-BE2DR100ELC/</t>
+          <t>https://www.brilliantearth.com/Riviera-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2DR100ELC/</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -551,19 +551,19 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/DD/BE2DR100ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/33/BE2DR100ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/C8/BE2DR100ELC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/57/BE2DR100ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/CE/BE2DR100ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/AC/BE2DR100ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>embed.imajize.com/678250798?v=1739866026</t>
+          <t>embed.imajize.com/355738415?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Emerald-Cut-Eternity-Lab-Diamond-Semi-Bezel-Ring-(3-ct.-tw.)-Gold-BE2D013ELC/</t>
+          <t>https://www.brilliantearth.com/Emerald-Cut-Eternity-Lab-Diamond-Semi-Bezel-Ring-(3-ct.-tw.)-Rose-Gold-BE2D013ELC/</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -573,19 +573,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/AF/BE2D013ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/AA/BE2D013ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/4E/BE2D013ELC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/3F/BE2D013ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/47/BE2D013ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/4D/BE2D013ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>embed.imajize.com/770726255?v=1739866026</t>
+          <t>embed.imajize.com/931741329?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Olivetta-Half-Coverage-Lab-Diamond-Ring-White-Gold-BE2D15103LC/</t>
+          <t>https://www.brilliantearth.com/Olivetta-Half-Coverage-Lab-Diamond-Ring-Rose-Gold-BE2D15103LC/</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -595,19 +595,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/ER/BE2D15103_white_top.webp, https://image.brilliantearth.com/media/product_new_images/0C/BE2D15103LC_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/V6/BE2D15103_white_side1.jpg, https://image.brilliantearth.com/media/product_images/OC/BE2D15103_white_ms_zi.webp</t>
+          <t>https://image.brilliantearth.com/media/product_images/M1/BE2D15103_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/96/BE2D15103LC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/OF/BE2D15103_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/SH/BE2D15103_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>embed.imajize.com/1772072?v=1739866026</t>
+          <t>embed.imajize.com/5680233?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Oval-Eternity-Lab-Diamond-Semi-Bezel-Ring-(3-ct.-tw.)-Gold-BE2D014ELC/</t>
+          <t>https://www.brilliantearth.com/Oval-Eternity-Lab-Diamond-Semi-Bezel-Ring-(3-ct.-tw.)-Rose-Gold-BE2D014ELC/</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -617,19 +617,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/72/BE2D014ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/20/BE2D014ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B4/BE2D014ELC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/50/BE2D014ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/DD/BE2D014ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/7E/BE2D014ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>embed.imajize.com/957394268?v=1739866026</t>
+          <t>embed.imajize.com/120577473?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Ellora-Half-Coverage-Lab-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2M2811LC/</t>
+          <t>https://www.brilliantearth.com/Ellora-Half-Coverage-Lab-Diamond-Ring-(7/8-ct.-tw.)-Rose-Gold-BE2M2811LC/</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -639,19 +639,19 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/06/BE2M2811LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/ME/BE2M2811-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/J9/BE2M2811_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/8D/BE2M2811LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/C5/BE2M2811LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/PO/BE2M2811-rose_2.jpg, https://image.brilliantearth.com/media/product_images/QK/BE2M2811_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/90/BE2M2811LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>embed.imajize.com/4810435?v=1739866026</t>
+          <t>embed.imajize.com/2890774?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Versailles-Three-Quarter-Coverage-Lab-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2D621LC/</t>
+          <t>https://www.brilliantearth.com/Versailles-Three-Quarter-Coverage-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D621LC/</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -661,19 +661,19 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/AJ/BE2D621_white_top.jpeg, https://image.brilliantearth.com/media/product_images/Y8/BE2D621-18KW_4.jpg, https://image.brilliantearth.com/media/product_images/O3/BE2D621-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/QJ/BE2D621_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E2/BE2D621LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/HE/BE2D621_rose_top.jpeg, https://image.brilliantearth.com/media/product_images/W8/BE2D621-rose_4.jpg, https://image.brilliantearth.com/media/product_images/B1/BE2D621-rose_2.jpg, https://image.brilliantearth.com/media/product_images/17/BE2D621_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/15/BE2D621LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>embed.imajize.com/2027567?v=1739866026</t>
+          <t>embed.imajize.com/6214237?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Ballad-Eternity-Lab-Diamond-Ring-(1/3-ct.-tw.)-Gold-BE2D1823ELC/</t>
+          <t>https://www.brilliantearth.com/Ballad-Eternity-Lab-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE2D1823ELC/</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -683,19 +683,19 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/03/BE2D1823E_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/QO/BE2D1823E-yellow_2.jpg, https://image.brilliantearth.com/media/product_new_images/C7/BE2D1823E_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/48/BE2D1823E_yellow_side2.jpg, https://image.brilliantearth.com/media/product_new_images/2C/BE2D1823E_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/99/BE2D1823E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/A1/BE2D1823E-rose_2.jpg, https://image.brilliantearth.com/media/product_images/3N/BE2D1823E_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/0A/BE2D1823E_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B6/BE2D1823E_rose_side2.jpg, https://image.brilliantearth.com/media/product_new_images/BF/BE2D1823E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>embed.imajize.com/2870856?v=1739866026</t>
+          <t>embed.imajize.com/6601356?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Ellora-Eternity-Lab-Diamond-Ring-(1-3/4-ct.-tw.)-White-Gold-BE2D2811ETLC/</t>
+          <t>https://www.brilliantearth.com/Ellora-Eternity-Lab-Diamond-Ring-(1-3/4-ct.-tw.)-Rose-Gold-BE2D2811ETLC/</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -705,19 +705,19 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/55/BE2D2811ETLC_white_top.jpg, https://image.brilliantearth.com/media/product_images/CM/BE2M2811ET_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/BT/BE2M2811ET_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3E/BE2D2811ETLC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/F8/BE2D2811ETLC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/DL/BE2M2811ET_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/LE/BE2M2811ET_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/71/BE2D2811ETLC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>embed.imajize.com/6026199?v=1739866026</t>
+          <t>embed.imajize.com/8850104?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Esther-Lab-Diamond-Ring-Gold-BE2D1463LC/</t>
+          <t>https://www.brilliantearth.com/Esther-Lab-Diamond-Ring-Rose-Gold-BE2D1463LC/</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -727,19 +727,19 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/64/BE2D1463LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/D4/BE2D1463LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/0B/BE2D1463LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/D5/BE2D1463LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/JK/BE2D1463LC_rose_harmony.jpg, https://image.brilliantearth.com/media/product_images/0O/BE2D1463LC_rose_harmony1.jpg, https://image.brilliantearth.com/media/product_new_images/B7/BE2D1463LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/PQ/BE2D1463LC_rose_harmony2.jpg, https://image.brilliantearth.com/media/product_new_images/63/BE2D1463LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>embed.imajize.com/739792766?v=1739866026</t>
+          <t>embed.imajize.com/284894784?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Olivetta-Contoured-Lab-Diamond-Ring-(1/2-ct.-tw.)-Gold-BE2D2237LC/</t>
+          <t>https://www.brilliantearth.com/Olivetta-Contoured-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D2237LC/</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -749,19 +749,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/4A/BE2D2237_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/9O/BE2D2237LC_yellow_F_model.jpg, https://image.brilliantearth.com/media/product_images/O4/BE2D2237_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/IU/BE2D2237_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/EX/BE2D2237_rose_top.jpg, https://image.brilliantearth.com/media/product_images/TH/BE2D2237LC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_images/RQ/BE2D2237_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/LB/BE2D2237_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>embed.imajize.com/496020921?v=1739866026</t>
+          <t>embed.imajize.com/804779212?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Adelaide-Curved-Lab-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2D3861LC/</t>
+          <t>https://www.brilliantearth.com/Adelaide-Curved-Lab-Diamond-Ring-(7/8-ct.-tw.)-Rose-Gold-BE2D3861LC/</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -771,19 +771,19 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/DE/BE2D3861LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/56/BE2D3861LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/16/BE2D3861LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/D5/BE2D3861LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/9E/BE2D3861LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/45/BE2D3861LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>embed.imajize.com/375264141?v=1739866026</t>
+          <t>embed.imajize.com/410565416?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Round-Eternity-Lab-Diamond-Semi-Bezel-Ring-(2-1/2-ct.-tw.)-White-Gold-BE2D012ELC/</t>
+          <t>https://www.brilliantearth.com/Round-Eternity-Lab-Diamond-Semi-Bezel-Ring-(2-1/2-ct.-tw.)-Rose-Gold-BE2D012ELC/</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -793,19 +793,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/CE/BE2D012ELC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/8E/BE2D012ELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/5C/BE2D012ELC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/51/BE2D012ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/2E/BE2D012ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/F0/BE2D012ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>embed.imajize.com/929692860?v=1739866026</t>
+          <t>embed.imajize.com/500984684?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Colette-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2D054ELC/</t>
+          <t>https://www.brilliantearth.com/Colette-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2D054ELC/</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -815,19 +815,19 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/B8/BE2D054ELC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/85/BE2D054ELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/51/BE2D054ELC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/C6/BE2D054ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/DF/BE2D054ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/F0/BE2D054ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>embed.imajize.com/418345109?v=1739866026</t>
+          <t>embed.imajize.com/713386690?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Riviera-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Gold-BE2DR200ELC/</t>
+          <t>https://www.brilliantearth.com/Riviera-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2DR200ELC/</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -837,19 +837,19 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/D1/BE2DR200ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/A8/BE2DR200ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/A7/BE2DR200ELC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/54/BE2DR200ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/6G/BE2DMS200E-rose_v2_2.jpg, https://image.brilliantearth.com/media/product_new_images/E7/BE2DR200ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/40/BE2DR200ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>embed.imajize.com/133560316?v=1739866026</t>
+          <t>embed.imajize.com/596280792?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Colette-Lab-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2D052LC/</t>
+          <t>https://www.brilliantearth.com/Colette-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D052LC/</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -859,19 +859,19 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/BB/BE2D052LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/C7/BE2D052LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/58/BE2D052LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/B1/BE2D052LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/69/BE2D052LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3F/BE2D052LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>embed.imajize.com/578251405?v=1739866026</t>
+          <t>embed.imajize.com/722177391?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Nathalie-Oval-Eternity-Lab-Diamond-Ring-White-Gold-BE2D852LC/</t>
+          <t>https://www.brilliantearth.com/Nathalie-Oval-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D852LC/</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -881,19 +881,19 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/52/BE2D852LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/BE/BE2D852LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BD/BE2D852LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/51/BE2D852LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/6E/BE2D852LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/C4/BE2D852LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>embed.imajize.com/542880609?v=1739866026</t>
+          <t>embed.imajize.com/615580059?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Nathalie-Oval-Lab-Diamond-Ring-Gold-BE2D851LC/</t>
+          <t>https://www.brilliantearth.com/Nathalie-Oval-Lab-Diamond-Ring-Rose-Gold-BE2D851LC/</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -903,19 +903,19 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/E3/BE2D851LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/8D/BE2D851LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/18/BE2D851LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/54/BE2D851LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/0C/BE2D851LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/C1/BE2D851LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>embed.imajize.com/927964878?v=1739866026</t>
+          <t>embed.imajize.com/856914360?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Mira-Lab-Diamond-Double-Row-Ring-White-Gold-BE2D0052LC/</t>
+          <t>https://www.brilliantearth.com/Mira-Lab-Diamond-Double-Row-Ring-Rose-Gold-BE2D0052LC/</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -925,19 +925,19 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/78/BE2D0052LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/CF/BE2D0052LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/DB/BE2D0052LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/EA/BE2D0052LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/68/BE2D0052LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/7E/BE2D0052LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>embed.imajize.com/430433959?v=1739866026</t>
+          <t>embed.imajize.com/957618756?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Monaco-Lab-Diamond-Ring-(3/4-ct.-tw.)-Gold-BE2D829LC/</t>
+          <t>https://www.brilliantearth.com/Monaco-Lab-Diamond-Ring-(3/4-ct.-tw.)-Rose-Gold-BE2D829LC/</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -947,19 +947,19 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/X3/BE2D829_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/KW/BE2D829-yellow_2.jpg, https://image.brilliantearth.com/media/product_images/0I/BE2D829_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/F6/BE2D829_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/0Z/BE2D829LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/W2/BE2D829_rose_top_1.jpg, https://image.brilliantearth.com/media/product_images/EF/BE2D829-rose_2.jpg, https://image.brilliantearth.com/media/product_images/3U/BE2D829_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/0Q/BE2D829_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/1F/BE2D829LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>embed.imajize.com/5200097?v=1739866026</t>
+          <t>embed.imajize.com/3380774?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Colette-Lab-Diamond-Ring-(1-ct.-tw.)-White-Gold-BE2D053LC/</t>
+          <t>https://www.brilliantearth.com/Colette-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D053LC/</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -969,19 +969,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/AA/BE2D053LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/10/BE2D053LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/A2/BE2D053LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/6D/BE2D053LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/4F/BE2D053LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/67/BE2D053LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>embed.imajize.com/446348258?v=1739866026</t>
+          <t>embed.imajize.com/168570285?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Luxe-Nathalie-Emerald-Cut-Lab-Diamond-Ring-(2-1/2-ct.-tw.)-Gold-BE2D3438LC/</t>
+          <t>https://www.brilliantearth.com/Luxe-Nathalie-Emerald-Cut-Lab-Diamond-Ring-(2-1/2-ct.-tw.)-Rose-Gold-BE2D3438LC/</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -991,19 +991,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/BC/BE2D3438LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/1E/BE2D3438LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/C3/BE2D3438LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/39/BE2D3438LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/TD/BE2D3438LC_rose_harmony.jpg, https://image.brilliantearth.com/media/product_images/EX/BE2D3438LC_rose_harmony1.jpg, https://image.brilliantearth.com/media/product_new_images/AB/BE2D3438LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/OC/BE2D3438LC_rose_harmony2.jpg, https://image.brilliantearth.com/media/product_new_images/7C/BE2D3438LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>embed.imajize.com/205572370?v=1739866026</t>
+          <t>embed.imajize.com/920162211?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Cannes-Curved-Lab-Diamond-Ring-(1-ct.-tw.)-Gold-BE2D4646LC/</t>
+          <t>https://www.brilliantearth.com/Cannes-Curved-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D4646LC/</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1013,19 +1013,19 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/8C/BE2D4646LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/72/BE2D4646LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/D6/BE2D4646LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/35/BE2D4646LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/F0/BE2D4646LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/2B/BE2D4646LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>embed.imajize.com/721631291?v=1739866026</t>
+          <t>embed.imajize.com/802375650?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Cara-Flush-Set-Eternity-Lab-Diamond-Ring-Gold-BE2D817LC/</t>
+          <t>https://www.brilliantearth.com/Cara-Flush-Set-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D817LC/</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1035,19 +1035,19 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/0C/BE2D817LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/6P/Holiday_Campaign_PDP_Crops-37_PDP_image_square.jpg, https://image.brilliantearth.com/media/product_new_images/DB/BE2D817LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/0A/BE2D817LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/C6/BE2D817LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/13/BE2D817LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/96/BE2D817LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>embed.imajize.com/593967951?v=1739866026</t>
+          <t>embed.imajize.com/404769111?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Tabitha-Channel-Set-Eternity-Lab-Diamond-Ring-(1/3-ct.-tw.)-Gold-BE2D458LC/</t>
+          <t>https://www.brilliantearth.com/Tabitha-Channel-Set-Eternity-Lab-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE2D458LC/</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1057,19 +1057,19 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/89/BE2D458LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/07/BE2D458LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/02/BE2D458LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/E6/BE2D458LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/19/BE2D458LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/D4/BE2D458LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>embed.imajize.com/237009613?v=1739866026</t>
+          <t>embed.imajize.com/510795764?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Grand-Lunette-Lab-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2D064LC/</t>
+          <t>https://www.brilliantearth.com/Grand-Lunette-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D064LC/</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1079,19 +1079,19 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/66/BE2D064_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/79/BE2D064_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/LK/BE1D5320_BE2D064_2.jpg, https://image.brilliantearth.com/media/product_new_images/AF/BE2D064_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/47/BE2D064_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/5D/BE2D064_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/E9/BE2D064_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/B3/BE2D064_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/28/BE2D064_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>embed.imajize.com/7406044?v=1739866026</t>
+          <t>embed.imajize.com/7747553?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Sienna-Three-Quarter-Coverage-Lab-Diamond-Open-Ring-(1/2-ct.-tw.)-Gold-BE2D1398LC/</t>
+          <t>https://www.brilliantearth.com/Sienna-Three-Quarter-Coverage-Lab-Diamond-Open-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D1398LC/</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1101,19 +1101,19 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/B4/BE2D1398_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/XH/BE2D1398-18KW_020.jpg, https://image.brilliantearth.com/media/product_new_images/23/BE2D1398_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/AF/BE2D1398_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/B1/BE2D1398_rose_top.jpg, https://image.brilliantearth.com/media/product_images/XH/BE2D1398-18KW_020.jpg, https://image.brilliantearth.com/media/product_new_images/38/BE2D1398_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/88/BE2D1398_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>embed.imajize.com/831770073?v=1739866026</t>
+          <t>embed.imajize.com/733442080?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Ravenna-Lab-Diamond-Ring-(1-ct.-tw.)-White-Gold-BE2D4072LC/</t>
+          <t>https://www.brilliantearth.com/Ravenna-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D4072LC/</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1123,19 +1123,19 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/BK/BE2D4072LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/97/BE2D4072LC_white_side1.jpg, https://image.brilliantearth.com/media/product_images/QP/BE2D4072LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/3B/BE2D4072LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/TA/BE2D4072LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/28/BE2D4072LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>embed.imajize.com/466352047?v=1739866026</t>
+          <t>embed.imajize.com/774945554?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Petite-Adelaide-Curved-Lab-Diamond-Ring-(1/2-ct.-tw.)-Gold-BE2D8444LC/</t>
+          <t>https://www.brilliantearth.com/Petite-Adelaide-Curved-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D8444LC/</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1145,19 +1145,19 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/6C/BE2D8444LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/A8/BE2D8444LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BA/BE2D8444LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/0E/BE2D8444LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/3B/BE2D8444LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/FD/BE2D8444LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>embed.imajize.com/539556404?v=1739866026</t>
+          <t>embed.imajize.com/836984222?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Versailles-Half-Coverage-Lab-Diamond-Ring-(3/8-ct.-tw.)-White-Gold-BE2D7890LC/</t>
+          <t>https://www.brilliantearth.com/Versailles-Half-Coverage-Lab-Diamond-Ring-(3/8-ct.-tw.)-Rose-Gold-BE2D7890LC/</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1167,19 +1167,19 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/26/BE2D7890_white_top.jpg, https://image.brilliantearth.com/media/product_images/JR/BE2D1791.jpeg, https://image.brilliantearth.com/media/product_images/9F/BE2D1791_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/45/BE2D7890_white_side1.jpg, https://image.brilliantearth.com/media/product_images/PH/BE2D1791_white_hand_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/UQ/BE2D7890_rose_top.jpg, https://image.brilliantearth.com/media/product_images/A8/BE2D1791_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/9N/BE2D1791.jpg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7890_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/5B/BE2D7890_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8754045?v=1739866026</t>
+          <t>embed.imajize.com/6107544?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Elowen-Lab-Diamond-Ring-(1-ct.-tw.)-Gold-BE2D6381LC/</t>
+          <t>https://www.brilliantearth.com/Elowen-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D6381LC/</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1189,19 +1189,19 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/54/BE2D6381LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/CD/BE2D6381LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/8C/BE2D6381LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/E1/BE2D6381LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/7F/BE2D6381LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/A5/BE2D6381LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>embed.imajize.com/646591857?v=1739866026</t>
+          <t>embed.imajize.com/311015678?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Zadie-Channel-Set-Lab-Diamond-Contour-Ring-(1/4-ct.-tw.)-Gold-BE2D3689LC/</t>
+          <t>https://www.brilliantearth.com/Zadie-Channel-Set-Lab-Diamond-Contour-Ring-(1/4-ct.-tw.)-Rose-Gold-BE2D3689LC/</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1211,19 +1211,19 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/7F/BE2D3689LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/CA/BE2D3689LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/16/BE2D3689LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/43/BE2D3689LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/5B/BE2D3689LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/4C/BE2D3689LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>embed.imajize.com/454244730?v=1739866026</t>
+          <t>embed.imajize.com/694640752?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Curved-Versailles-Lab-Diamond-Ring-White-Gold-BE2D7422LC/</t>
+          <t>https://www.brilliantearth.com/Curved-Versailles-Lab-Diamond-Ring-Rose-Gold-BE2D7422LC/</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1233,19 +1233,19 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/AC/BE2D7422_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/02/BE2D7422_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/VK/BE2D7422_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/87/BE2D7422_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/F5/BE2D7422_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/05/BE2D7422_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/4D/BE2D7422_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/4E/BE2D7422_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/CD/BE2D7422_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>embed.imajize.com/3018965?v=1739866026</t>
+          <t>embed.imajize.com/3883496?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Nathalie-Emerald-Cut-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-White-Gold-BE2D3426LC/</t>
+          <t>https://www.brilliantearth.com/Nathalie-Emerald-Cut-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D3426LC/</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1255,19 +1255,19 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/05/BE2D3426LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/S7/Perfect_Collection_-_Imagery_Crops_1x1-4_copy.jpg, https://image.brilliantearth.com/media/product_images/RI/Perfect_Collection_-_Imagery_Crops_1x1-8_copy.jpg, https://image.brilliantearth.com/media/product_new_images/AE/BE2D3426LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/30/BE2D3426LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/7C/BE2D3426LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/S7/Perfect_Collection_-_Imagery_Crops_1x1-4_copy.jpg, https://image.brilliantearth.com/media/product_images/RI/Perfect_Collection_-_Imagery_Crops_1x1-8_copy.jpg, https://image.brilliantearth.com/media/product_new_images/B3/BE2D3426LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/F8/BE2D3426LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>embed.imajize.com/622735190?v=1739866026</t>
+          <t>embed.imajize.com/909341398?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Flair-Lab-Diamond-Ring-(2/5-ct.-tw.)-White-Gold-BE2D1940LC/</t>
+          <t>https://www.brilliantearth.com/Flair-Lab-Diamond-Ring-(2/5-ct.-tw.)-Rose-Gold-BE2D1940LC/</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1277,19 +1277,19 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/B9/BE2D1940_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/3A/BE2D1940_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/22/BE2D1940_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B4/BE2D1940_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/FE/BE2D1940_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/87/BE2D1940_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/D3/BE2D1940_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/21/BE2D1940_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>embed.imajize.com/2455103?v=1739866026</t>
+          <t>embed.imajize.com/7573213?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Elongated-Flair-Lab-Diamond-Ring-Gold-BE2D2320LC/</t>
+          <t>https://www.brilliantearth.com/Elongated-Flair-Lab-Diamond-Ring-Rose-Gold-BE2D2320LC/</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1299,19 +1299,19 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/3E/BE2320_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/FD/BE2320_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/TW/BE487343-yellow_BE5D251-yellow_BE2320-18KW_053.jpg, https://image.brilliantearth.com/media/product_new_images/99/BE2320_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/3S/BE2320_yellow_top_upward.jpg, https://image.brilliantearth.com/media/product_new_images/3F/BE2320_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/70/BE2320_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/3A/BE2320_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/LR/BE487343-rose_BE5D251-rose_BE2320-18KW_053.jpg, https://image.brilliantearth.com/media/product_new_images/C7/BE2320_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/JY/BE2320_rose_top_upward.jpg, https://image.brilliantearth.com/media/product_new_images/FD/BE2320_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9409465?v=1739866026</t>
+          <t>embed.imajize.com/1274781?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Lunette-Lab-Diamond-Ring-(1/5-ct.-tw.)-Gold-BE2D594LC/</t>
+          <t>https://www.brilliantearth.com/Lunette-Lab-Diamond-Ring-(1/5-ct.-tw.)-Rose-Gold-BE2D594LC/</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1321,19 +1321,19 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/03/BE2D594_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/15/BE2D594_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B2/BE2D594_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/16/BE2D594_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/2C/BE2D594_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B6/BE2D594_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>embed.imajize.com/254769662?v=1739866026</t>
+          <t>embed.imajize.com/748742221?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Flair-Lab-Diamond-Ring-(1/6-ct.-tw.)-White-Gold-BE2D1812LC/</t>
+          <t>https://www.brilliantearth.com/Flair-Lab-Diamond-Ring-(1/6-ct.-tw.)-Rose-Gold-BE2D1812LC/</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1343,19 +1343,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/61/BE2D1812_white_top.jpg, https://image.brilliantearth.com/media/product_images/83/BE2D1812-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/7N/BE2D1812_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/1D/BE2D1812_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/75/BE2D1812_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/B9/BE2D1812_rose_top.jpg, https://image.brilliantearth.com/media/product_images/9Y/BE2D1812-rose_2.jpg, https://image.brilliantearth.com/media/product_images/AE/BE2D1812_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/BC/BE2D1812_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/A2/BE2D1812_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>embed.imajize.com/5884757?v=1739866026</t>
+          <t>embed.imajize.com/9667867?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Chloe-Flush-Set-Emerald-Cut-Lab-Diamond-Ring-Gold-BE2D818LC/</t>
+          <t>https://www.brilliantearth.com/Chloe-Flush-Set-Emerald-Cut-Lab-Diamond-Ring-Rose-Gold-BE2D818LC/</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1365,19 +1365,19 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/83/BE2D818LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/B6/BE2D818LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/EE/BE2D818LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/D5/BE2D818LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/EA/BE2D818LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/74/BE2D818LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>embed.imajize.com/785472030?v=1739866026</t>
+          <t>embed.imajize.com/783107639?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Sienna-Eternity-Lab-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2M3420ETLC/</t>
+          <t>https://www.brilliantearth.com/Sienna-Eternity-Lab-Diamond-Ring-(7/8-ct.-tw.)-Rose-Gold-BE2M3420ETLC/</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1387,19 +1387,19 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/70/BE2M3420ET_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/C8/BE2M3420ETLC_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/KP/BE2M3420-BE2M3420ET-BE2M3420H.jpg, https://image.brilliantearth.com/media/product_new_images/F0/BE2M3420ET_white_side1.jpg, https://image.brilliantearth.com/media/product_images/DQ/BE2M3420ET_white_additional1.webp, https://image.brilliantearth.com/media/product_new_images/18/BE2M3420ET_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/31/BE2M3420ET_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/C5/BE2M3420ETLC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/RY/BE266E_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/01/BE2M3420ET_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/1D/BE2M3420ET_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>embed.imajize.com/3767952?v=1739866026</t>
+          <t>embed.imajize.com/7656271?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Elodie-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-White-Gold-BE2D1126LC/</t>
+          <t>https://www.brilliantearth.com/Elodie-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D1126LC/</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1409,19 +1409,19 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/71/BE2D1126LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/K1/BE2D1136LC_white_side2.jpg, https://image.brilliantearth.com/media/product_new_images/8D/BE2D1126LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3A/BE2D1126LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/74/BE2D1126LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/05/BE2D1136LC_rose_side2.jpg, https://image.brilliantearth.com/media/product_new_images/03/BE2D1126LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/F1/BE2D1126LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>embed.imajize.com/897147454?v=1739866026</t>
+          <t>embed.imajize.com/490254582?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Lunette-Lab-Diamond-Ring-(1/10-ct.-tw.)-Gold-BE2D062LC/</t>
+          <t>https://www.brilliantearth.com/Lunette-Lab-Diamond-Ring-(1/10-ct.-tw.)-Rose-Gold-BE2D062LC/</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1431,19 +1431,19 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/05/BE2D062_yellow_00.jpg, https://image.brilliantearth.com/media/product_images/1V/BE2D062-18KY_2.jpg, https://image.brilliantearth.com/media/product_images/VJ/BE1D225-18KY_3.jpg, https://image.brilliantearth.com/media/product_images/L2/BE2D062_yellow_02.jpg, https://image.brilliantearth.com/media/product_images/9Q/BE2D062_yellow_hand_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/HR/BE2D062_rose_00.jpg, https://image.brilliantearth.com/media/product_images/58/BE2D062-rose_2.jpg, https://image.brilliantearth.com/media/product_images/9I/BE1D225-rose-7_BE2D062-rose_3.jpg, https://image.brilliantearth.com/media/product_images/K9/BE2D062_rose_02.jpg, https://image.brilliantearth.com/media/product_images/M5/BE2D062_rose_hand_ms_zi.png</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>embed.imajize.com/5480432?v=1739866026</t>
+          <t>embed.imajize.com/1670437?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Aria-Contoured-Lab-Diamond-Ring-(1/6-ct.-tw.)-Gold-BE2D232LC/</t>
+          <t>https://www.brilliantearth.com/Aria-Contoured-Lab-Diamond-Ring-(1/6-ct.-tw.)-Rose-Gold-BE2D232LC/</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1453,19 +1453,19 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/5B/BE2D232_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/0C/BE2D232_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/28/BE2D232_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3C/BE2D232_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/5E/BE2D232_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/80/BE2D232_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/82/BE2D232_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/1A/BE2D232_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>embed.imajize.com/4144475?v=1739866026</t>
+          <t>embed.imajize.com/5712503?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Tabitha-Channel-Set-Baguette-Eternity-Lab-Diamond-Ring-Gold-BE2D119LC/</t>
+          <t>https://www.brilliantearth.com/Tabitha-Channel-Set-Baguette-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D119LC/</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1475,19 +1475,19 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/2F/BE2D119LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/A8/BE2D119LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/D4/BE2D119LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/53/BE2D119LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/1F/BE2D119LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3F/BE2D119LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>embed.imajize.com/210626128?v=1739866026</t>
+          <t>embed.imajize.com/296489128?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Oval-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2DOV200ELC/</t>
+          <t>https://www.brilliantearth.com/Oval-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2DOV200ELC/</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1497,19 +1497,19 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/N2/BE2DOV200E_white_top.jpg, https://image.brilliantearth.com/media/product_images/TX/BE2D200OVE-white_019.jpg, https://image.brilliantearth.com/media/product_images/A5/BE2D200OVE_white_additional1_1.jpg, https://image.brilliantearth.com/media/product_images/LM/BE2DOV200E_white_side1.jpg, https://image.brilliantearth.com/media/product_images/U4/BE2DOV200E_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/CU/BE2DOV200E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/P5/BE2D200OVE-rose_019.jpg, https://image.brilliantearth.com/media/product_images/RX/BE2D200OVE_rose_additional1_1.jpg, https://image.brilliantearth.com/media/product_images/ZB/BE2DOV200E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/BC/BE2DOV200E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>embed.imajize.com/216705019?v=1739866026</t>
+          <t>embed.imajize.com/873046103?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/East-West-Bezel-Oval-Eternity-Lab-Diamond-Ring-White-Gold-BE2D210BELC/</t>
+          <t>https://www.brilliantearth.com/East-West-Bezel-Oval-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D210BELC/</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1519,19 +1519,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/00/BE2D210BELC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/11/BE2D210BELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/0B/BE2D210BELC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/3C/BE2D210BELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/40/BE2D210BELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/AD/BE2D210BELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>embed.imajize.com/882596993?v=1739866026</t>
+          <t>embed.imajize.com/864736382?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(6-ct.-tw.)-White-Gold-BE2D309LC/</t>
+          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(6-ct.-tw.)-Rose-Gold-BE2D309LC/</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1541,19 +1541,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/5F/BE2D309LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/08/BE2D309LC-18KW_012.jpg, https://image.brilliantearth.com/media/product_new_images/3D/BE2D309LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E9/BE2D309LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/17/BE2D309LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/7R/BE2D309LC-rose_F_model.jpg, https://image.brilliantearth.com/media/product_new_images/2A/BE2D309LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/68/BE2D309LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>embed.imajize.com/560771496?v=1739866026</t>
+          <t>embed.imajize.com/627275330?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/East-West-Bezel-Pear-Eternity-Lab-Diamond-Ring-Gold-BE2D209BELC/</t>
+          <t>https://www.brilliantearth.com/East-West-Bezel-Pear-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D209BELC/</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1563,19 +1563,19 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/1E/BE2D209BELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/AA/BE2D209BELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/41/BE2D209BELC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/FB/BE2D209BELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/F2/BE2D209BELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/64/BE2D209BELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>embed.imajize.com/646708211?v=1739866026</t>
+          <t>embed.imajize.com/276189044?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Valencia-Lab-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2D1789LC/</t>
+          <t>https://www.brilliantearth.com/Valencia-Lab-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE2D1789LC/</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1585,19 +1585,19 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/F8/BE2D1789LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/G1/BE2D1789LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/9E/BE2D1789LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/F5/BE2D1789LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/PG/BE2D1789LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/30/BE2D1789LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>embed.imajize.com/835894374?v=1739866026</t>
+          <t>embed.imajize.com/124210025?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Bliss-Lab-Diamond-Ring-(1/5-ct.-tw.)-White-Gold-BE2FPD14LC/</t>
+          <t>https://www.brilliantearth.com/Bliss-Lab-Diamond-Ring-(1/5-ct.-tw.)-Rose-Gold-BE2FPD14LC/</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1607,19 +1607,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/39/BE2FPD14_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/85/BE2FPD14_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/GO/BE2FPD14-18KW_v2_3.jpg, https://image.brilliantearth.com/media/product_new_images/BE/BE2FPD14_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/82/BE2FPD14_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/E9/BE2FPD14_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/A2/BE2FPD14_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/CV/BE2FPD14-rose_BE304RD50-18KW_v2_3.jpg, https://image.brilliantearth.com/media/product_new_images/00/BE2FPD14_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E1/BE2FPD14_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9481254?v=1739866026</t>
+          <t>embed.imajize.com/9049198?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Elodie-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2D1127LC/</t>
+          <t>https://www.brilliantearth.com/Elodie-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2D1127LC/</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1629,19 +1629,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/FB/BE2D1127LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/61/BE2D1127LC_white_side1.jpg, https://image.brilliantearth.com/media/product_images/ON/BE2D1127LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/C3/BE2D1127LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/10/BE2D1127LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/RZ/BE2D1127LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>embed.imajize.com/545233689?v=1739866026</t>
+          <t>embed.imajize.com/236125321?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Whisper-Half-Coverage-Lab-Diamond-Ring-(1/10-ct.-tw.)-White-Gold-BE266LC/</t>
+          <t>https://www.brilliantearth.com/Whisper-Half-Coverage-Lab-Diamond-Ring-(1/10-ct.-tw.)-Rose-Gold-BE266LC/</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1651,19 +1651,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/01/BE266_white_top.jpg, https://image.brilliantearth.com/media/product_images/2X/BE266-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/FS/BE4D305-S_BE1D166-18KW_BE266-18KW_2.jpg, https://image.brilliantearth.com/media/product_new_images/C4/BE266_white_side1.jpg, https://image.brilliantearth.com/media/product_images/69/BE266_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/26/BE266_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/C9/BE266_rose_top.jpg, https://image.brilliantearth.com/media/product_images/60/BE266-rose_2.jpg, https://image.brilliantearth.com/media/product_images/10/BE266_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/E7/BE266_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/33/BE266_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>embed.imajize.com/3958095?v=1739866026</t>
+          <t>embed.imajize.com/1329299?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Bezel-Oval-Eternity-Lab-Diamond-Ring-White-Gold-BE2D238BELC/</t>
+          <t>https://www.brilliantearth.com/Bezel-Oval-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D238BELC/</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1673,19 +1673,19 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/BF/BE2D238BELC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/20/BE2D238BELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3D/BE2D238BELC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/FC/BE2D238BELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/0D/BE2D238BELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/FA/BE2D238BELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>embed.imajize.com/491437791?v=1739866026</t>
+          <t>embed.imajize.com/651924753?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Ballad-Half-Coverage-Lab-Diamond-Ring-(1/6-ct.-tw.)-White-Gold-BE2D1823LC/</t>
+          <t>https://www.brilliantearth.com/Ballad-Half-Coverage-Lab-Diamond-Ring-(1/6-ct.-tw.)-Rose-Gold-BE2D1823LC/</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1695,19 +1695,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/5F/BE2D1823_white_top.jpg, https://image.brilliantearth.com/media/product_images/KZ/BE2D1823-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/BN/BE2D1823E_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/75/BE2D1823_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/2A/BE2D1823_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/28/BE2D1823_rose_top.jpg, https://image.brilliantearth.com/media/product_images/OL/BE2D1823-rose_2.jpg, https://image.brilliantearth.com/media/product_images/U0/BE2D1823E_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/66/BE2D1823_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/6F/BE2D1823_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>embed.imajize.com/7288068?v=1739866026</t>
+          <t>embed.imajize.com/2526480?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Flair-Lab-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2D1938LC/</t>
+          <t>https://www.brilliantearth.com/Flair-Lab-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE2D1938LC/</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1717,19 +1717,19 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/85/BE2D1938_white_top.jpg, https://image.brilliantearth.com/media/product_images/2V/BE2D1938.jpeg, https://image.brilliantearth.com/media/product_images/NW/BE2D1938_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/00/BE2D1938_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/D7/BE2D1938_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/47/BE2D1938_rose_top.jpg, https://image.brilliantearth.com/media/product_images/DA/BE2D1938_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/QU/BE2D1938.jpg, https://image.brilliantearth.com/media/product_new_images/04/BE2D1938_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/DE/BE2D1938_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>embed.imajize.com/6632964?v=1739866026</t>
+          <t>embed.imajize.com/7852806?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Anthology-Three-Quarter-Coverage-Lab-Diamond-Ring-Gold-BE2D1026LC/</t>
+          <t>https://www.brilliantearth.com/Anthology-Three-Quarter-Coverage-Lab-Diamond-Ring-Rose-Gold-BE2D1026LC/</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -1739,19 +1739,19 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/26/BE2D1026_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/3W/BE2D1026-18KY_002.jpg, https://image.brilliantearth.com/media/product_images/NX/BE2D1026_yellow_side.jpg, https://image.brilliantearth.com/media/product_new_images/7A/BE2D1026_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/HA/BE2D1026_rose_top.jpg, https://image.brilliantearth.com/media/product_images/2F/BE2D1026-14KR_002.jpg, https://image.brilliantearth.com/media/product_images/48/BE2D1026_rose_side.jpg, https://image.brilliantearth.com/media/product_new_images/A0/BE2D1026_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>embed.imajize.com/4559681?v=1739866026</t>
+          <t>embed.imajize.com/4370611?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Bezel-Emerald-Cut-Eternity-Lab-Diamond-Ring-(2-1/2-ct.-tw.)-Gold-BE2DEB250ELC/</t>
+          <t>https://www.brilliantearth.com/Bezel-Emerald-Cut-Eternity-Lab-Diamond-Ring-(2-1/2-ct.-tw.)-Rose-Gold-BE2DEB250ELC/</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1761,19 +1761,19 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/5B/BE2DEB250ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/AF/BE2DEB250ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/CC/BE2DEB250ELC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/2F/BE2DEB250ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/D0/BE2DEB250ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/79/BE2DEB250ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>embed.imajize.com/942328904?v=1739866026</t>
+          <t>embed.imajize.com/513725650?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Luxe-Valencia-Eternity-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-White-Gold-BE2D654LC/</t>
+          <t>https://www.brilliantearth.com/Luxe-Valencia-Eternity-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-Rose-Gold-BE2D654LC/</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -1783,19 +1783,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/52/BE2D654LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/4A/BE2D654LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/79/BE2D654LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/FB/BE2D654LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/L4/BE2D654LC_rose_harmony.jpg, https://image.brilliantearth.com/media/product_images/7E/BE2D654LC_rose_harmony1.jpg, https://image.brilliantearth.com/media/product_new_images/CE/BE2D654LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/FQ/BE2D654LC_rose_harmony2.jpg, https://image.brilliantearth.com/media/product_new_images/12/BE2D654LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>embed.imajize.com/974055173?v=1739866026</t>
+          <t>embed.imajize.com/647516546?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Marseille-Half-Coverage-Lab-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2D2110LC/</t>
+          <t>https://www.brilliantearth.com/Marseille-Half-Coverage-Lab-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE2D2110LC/</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1805,19 +1805,19 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/ED/BE2D2110_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/7F/BE2D2110_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/PO/BE2D2110_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/32/BE2D2110_white_side1.jpg, https://image.brilliantearth.com/media/product_images/MJ/expires_oct2024_103022_SL_HP_Marseille_Collection_HERO.jpg, https://image.brilliantearth.com/media/product_new_images/1F/BE2D2110_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/A6/BE2D2110_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/19/BE2D2110_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/LI/BE2D2110_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/7A/BE2D2110_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/40/BE2D2110_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>embed.imajize.com/1344082?v=1739866026</t>
+          <t>embed.imajize.com/5833659?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Arista-Eternity-Lab-Diamond-Ring-White-Gold-BE2D130ELC/</t>
+          <t>https://www.brilliantearth.com/Arista-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D130ELC/</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1827,19 +1827,19 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/A8/BE2D130E_white_top.jpg, https://image.brilliantearth.com/media/product_images/X2/BE2D130E-white-S6_BE3404-white_BE4110916-14KY_001.jpg, https://image.brilliantearth.com/media/product_images/0E/BE2D130E_2.jpg, https://image.brilliantearth.com/media/product_new_images/99/BE2D130E_white_side1.jpg, https://image.brilliantearth.com/media/product_images/E8/BE2D130E_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/Y9/BE2D130E_white_hand_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/FB/BE2D130E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/K6/BE2D130E-rose-S6_BE3404-rose_BE4110916-14KY_001.jpg, https://image.brilliantearth.com/media/product_images/RI/BE2D130E_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/AF/BE2D130E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/9A/BE2D130E_rose_hand_ms_zi.png</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9421289?v=1739866026</t>
+          <t>embed.imajize.com/8633991?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Jardiniere-Eternity-Lab-Diamond-Ring-Gold-BE2D836LC/</t>
+          <t>https://www.brilliantearth.com/Jardiniere-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D836LC/</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1849,19 +1849,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/AE/BE2D836LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/6R/Holiday_Campaign_PDP_Crops-39_PDP_image_square.jpg, https://image.brilliantearth.com/media/product_new_images/96/BE2D836LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/D4/BE2D836LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/19/BE2D836LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/07/BE2D836LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B2/BE2D836LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>embed.imajize.com/595640272?v=1739866026</t>
+          <t>embed.imajize.com/566230200?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Sienna-Half-Coverage-Lab-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2M3420HLC/</t>
+          <t>https://www.brilliantearth.com/Sienna-Half-Coverage-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2M3420HLC/</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -1871,19 +1871,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/2C/BE2M3420HLC_white_top.jpg, https://image.brilliantearth.com/media/product_images/4O/BE2M3420H-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/46/BE2M3420H_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/D3/BE2M3420H_white_side1.jpg, https://image.brilliantearth.com/media/product_images/QH/BE2M3420-BE2M3420ET-BE2M3420H.jpeg, https://image.brilliantearth.com/media/product_new_images/7C/BE2M3420HLC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/58/BE2M3420HLC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/XM/BE2M3420H-rose_2.jpg, https://image.brilliantearth.com/media/product_images/LB/BE2M3420ET_rose_additional1_1.jpg, https://image.brilliantearth.com/media/product_new_images/FD/BE2M3420H_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/63/BE2M3420HLC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9058259?v=1739866026</t>
+          <t>embed.imajize.com/5798642?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Olivetta-Three-Quarter-Coverage-Lab-Diamond-Ring-White-Gold-BE2D15104LC/</t>
+          <t>https://www.brilliantearth.com/Olivetta-Three-Quarter-Coverage-Lab-Diamond-Ring-Rose-Gold-BE2D15104LC/</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -1893,19 +1893,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/0J/WG0.jpg, https://image.brilliantearth.com/media/product_images/P5/BE2D15103LC-white-N-S6_034.jpg, https://image.brilliantearth.com/media/product_images/R6/WG2.jpg, https://image.brilliantearth.com/media/product_images/D2/WG1_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/ET/RG0.jpg, https://image.brilliantearth.com/media/product_images/7U/BE2D15103LC-rose-N-S6_034.jpg, https://image.brilliantearth.com/media/product_images/HU/RG2.jpg, https://image.brilliantearth.com/media/product_images/HR/RG1_ms_zi.png</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>embed.imajize.com/3958156?v=1739866026</t>
+          <t>embed.imajize.com/4788556?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Round-Five-Stone-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-White-Gold-BE2D5ST150RDLC/</t>
+          <t>https://www.brilliantearth.com/Round-Five-Stone-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-Rose-Gold-BE2D5ST150RDLC/</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -1915,19 +1915,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/PA/BE2D5ST150RDLC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/5A/BE2D5ST150RDLC_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/T5/BE2D5ST150RD_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/N7/BE2D5ST150RD_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/54/BE2D5ST150RDLC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/4L/BE2D5ST150RDLC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/15/BE2D5ST150RDLC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/DA/BE2D5ST150RD_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/EB/BE2D5ST150RD_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/F6/BE2D5ST150RDLC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>embed.imajize.com/4736447?v=1739866026</t>
+          <t>embed.imajize.com/3289797?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Petite-Shared-Prong-Three-Quarter-Coverage-Lab-Diamond-Ring-(3/8-ct.-tw.)-White-Gold-BE2PD28R15LC/</t>
+          <t>https://www.brilliantearth.com/Petite-Shared-Prong-Three-Quarter-Coverage-Lab-Diamond-Ring-(3/8-ct.-tw.)-Rose-Gold-BE2PD28R15LC/</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -1937,19 +1937,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/3D/BE2PD28R15_white_top.jpg, https://image.brilliantearth.com/media/product_images/UH/BE2PD28R15-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/FI/BE2PD28R15_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/4D/BE2PD28R15_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/65/BE2PD28R15_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/F1/BE2PD28R15_rose_top.jpg, https://image.brilliantearth.com/media/product_images/9U/BE2PD28R15-18KR_023.jpg, https://image.brilliantearth.com/media/product_images/EU/BE2PD28R15_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/E0/BE2PD28R15_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/50/BE2PD28R15_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>embed.imajize.com/3251726?v=1739866026</t>
+          <t>embed.imajize.com/3442969?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Petite-Twisted-Vine-Lab-Diamond-Ring-(1/8-ct.-tw.)-White-Gold-BE2M254PLC/</t>
+          <t>https://www.brilliantearth.com/Petite-Twisted-Vine-Lab-Diamond-Ring-(1/8-ct.-tw.)-Rose-Gold-BE2M254PLC/</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -1959,19 +1959,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/38/BE2M254P_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/30/BE2M254P_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/JX/BE2M254P_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/D8/BE2M254P_white_side1.jpg, https://image.brilliantearth.com/media/product_images/6U/BE2M254P.jpeg, https://image.brilliantearth.com/media/product_new_images/FB/BE2M254P_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/EB/BE2M254P_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/18/BE2M254P_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/0A/BE2M254P_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/44/BE2M254P_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/AB/BE2M254P_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>embed.imajize.com/6178727?v=1739866026</t>
+          <t>embed.imajize.com/6247714?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Versailles-Eternity-Lab-Diamond-Ring-(3/4-ct.-tw.)-Gold-BE2D1792LC/</t>
+          <t>https://www.brilliantearth.com/Versailles-Eternity-Lab-Diamond-Ring-(3/4-ct.-tw.)-Rose-Gold-BE2D1792LC/</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -1981,19 +1981,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/96/BE2D1792_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/NE/BE2D1792-yellow_019.jpg, https://image.brilliantearth.com/media/product_new_images/E6/BE2D1792_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/64/BE2D1792_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/28/BE2D1792_rose_top.jpg, https://image.brilliantearth.com/media/product_images/RK/BE2D1792-rose_019.jpg, https://image.brilliantearth.com/media/product_new_images/83/BE2D1792_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/0E/BE2D1792_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8721821?v=1739866026</t>
+          <t>embed.imajize.com/3078997?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(1-1/3-ct.-tw.)-White-Gold-BE2SD24R144LC/</t>
+          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(1-1/3-ct.-tw.)-Rose-Gold-BE2SD24R144LC/</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2003,19 +2003,19 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/07/BE2SD24R144LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/C0/BE2SD24R144-18KW_032.jpg, https://image.brilliantearth.com/media/product_images/E1/BE2SD24R144_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/7E/BE2SD24R144LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/70/BE2SD24R144LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/DD/BE2SD24R144LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/4M/BE2SD24R144-rose_BE4M616-rose_032.jpg, https://image.brilliantearth.com/media/product_images/PQ/BE2SD24R144_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/76/BE2SD24R144LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/70/BE2SD24R144LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>embed.imajize.com/381778886?v=1739866026</t>
+          <t>embed.imajize.com/416984609?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Ulla-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D1136LC/</t>
+          <t>https://www.brilliantearth.com/Ulla-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Rose-Gold-BE2D1136LC/</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2030,14 +2030,14 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>embed.imajize.com/528593322?v=1739866026</t>
+          <t>embed.imajize.com/528593322?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/French-Pavé-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2M200ETLC/</t>
+          <t>https://www.brilliantearth.com/French-Pavé-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2M200ETLC/</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2047,19 +2047,19 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/ZL/_BE2M200ET_white_top.jpg, https://image.brilliantearth.com/media/product_images/UD/BE2M200ET-PT-S65_030.jpg, https://image.brilliantearth.com/media/product_images/5R/BE2M200ET_white_additional1_1.jpg, https://image.brilliantearth.com/media/product_images/OD/_BE2M200ET_white_side1.jpg, https://image.brilliantearth.com/media/product_images/QX/_BE2M200ET_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/PS/_BE2M200ET_rose_top.jpg, https://image.brilliantearth.com/media/product_images/4S/BE025_BE2M200ET-rose-S65_030.jpg, https://image.brilliantearth.com/media/product_images/HU/BE2M200ET_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/5Z/_BE2M200ET_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/FU/_BE2M200ET_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9038601?v=1739866026</t>
+          <t>embed.imajize.com/8486512?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Petite-Shared-Prong-Half-Coverage-Lab-Diamond-Ring-(1/4-ct.-tw.)-White-Gold-BE2PD25R25LC/</t>
+          <t>https://www.brilliantearth.com/Petite-Shared-Prong-Half-Coverage-Lab-Diamond-Ring-(1/4-ct.-tw.)-Rose-Gold-BE2PD25R25LC/</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2069,19 +2069,19 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/JN/BE2PD25R25_white_top.jpeg, https://image.brilliantearth.com/media/product_images/H6/BE2PD25R25-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/89/BE3AQ4212-S_BE1PD25R25-18KW_BE2PD25R25-18KW_2.jpg, https://image.brilliantearth.com/media/product_new_images/B8/BE2PD25R25_white_side1.jpg, https://image.brilliantearth.com/media/product_images/7E/BE2PD25R25_white_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/3A/BE2PD25R25LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/WD/BE2PD25R25_rose_top.jpeg, https://image.brilliantearth.com/media/product_images/JP/BE2PD25R25-rose_BE4LBT85-S_BE4D056S-S_2.jpg, https://image.brilliantearth.com/media/product_images/UC/BE2PD25R25_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/84/BE2PD25R25_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/F3/BE2PD25R25LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>embed.imajize.com/5572625?v=1739866026</t>
+          <t>embed.imajize.com/9108265?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Petite-Shared-Prong-Eternity-Lab-Diamond-Ring-(1/2-ct.-tw.)-Gold-BE2PD50R50LC/</t>
+          <t>https://www.brilliantearth.com/Petite-Shared-Prong-Eternity-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2PD50R50LC/</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2091,19 +2091,19 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/E8/BE2PD50R50_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/XQ/BE2PD50R50-18KY-S6_015.jpg, https://image.brilliantearth.com/media/product_images/VQ/BE2PD50R50_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/C9/BE2PD50R50_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/EA/BE2PD50R50_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/59/BE2PD50R50_rose_top.jpg, https://image.brilliantearth.com/media/product_images/6P/BE2PD50R50-rose-S6_015.jpg, https://image.brilliantearth.com/media/product_images/MH/BE2PD50R50_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/6B/BE2PD50R50_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/65/BE2PD50R50_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>embed.imajize.com/5557416?v=1739866026</t>
+          <t>embed.imajize.com/6445490?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Curved-Ballad-Lab-Diamond-Ring-(1/6-ct.-tw.)-Gold-BE2D3542PLC/</t>
+          <t>https://www.brilliantearth.com/Curved-Ballad-Lab-Diamond-Ring-(1/6-ct.-tw.)-Rose-Gold-BE2D3542PLC/</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2113,19 +2113,19 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/3D/BE2D3542P_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/06/BE2D3542P_yellow_F_model.jpg, https://image.brilliantearth.com/media/product_new_images/52/BE2D3542P_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/90/BE2D3542P_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/1D/BE2D3542P_rose_top.jpg, https://image.brilliantearth.com/media/product_images/FT/BE2D3542P_rose_F_model.jpg, https://image.brilliantearth.com/media/product_new_images/BB/BE2D3542P_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/DA/BE2D3542P_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9158580?v=1739866026</t>
+          <t>embed.imajize.com/3307680?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(6-ct.-tw.)-Gold-BE2DEM600ELC/</t>
+          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(6-ct.-tw.)-Rose-Gold-BE2DEM600ELC/</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2135,19 +2135,19 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/LO/BE2DEM600E_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/7C/BE2DEM600E_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/0R/BE2DEM600E_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/GU/BE2DEM600E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/D9/BE2DEM600E_rose_harmony.jpg, https://image.brilliantearth.com/media/product_images/PK/BE2DEM600E_rose_harmony1.jpg, https://image.brilliantearth.com/media/product_images/H6/BE2DEM600E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/VW/BE2DEM600E_rose_harmony2.jpg, https://image.brilliantearth.com/media/product_images/FX/BE2DEM600E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>embed.imajize.com/776573768?v=1739866026</t>
+          <t>embed.imajize.com/363652894?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Santorini-Eternity-Lab-Diamond-Ring-Gold-BE2D4613LC/</t>
+          <t>https://www.brilliantearth.com/Santorini-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D4613LC/</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2157,19 +2157,19 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/E3/BE2D4613_yellow_top.png, https://image.brilliantearth.com/media/product_images/TR/BE2D4613LC_yellow_F_model.jpg, https://image.brilliantearth.com/media/product_new_images/C6/BE2D4613_yellow_side1.png, https://image.brilliantearth.com/media/product_new_images/EE/BE2D4613_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/67/BE2D4613_rose_top.png, https://image.brilliantearth.com/media/product_images/Q2/BE2D4613LC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_new_images/AA/BE2D4613_rose_side1.png, https://image.brilliantearth.com/media/product_new_images/A5/BE2D4613_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>embed.imajize.com/249529076?v=1739866026</t>
+          <t>embed.imajize.com/445113097?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Heart-Shaped-Lab-Diamond-Bezel-Ring-White-Gold-BE2DHB3ELC/</t>
+          <t>https://www.brilliantearth.com/Heart-Shaped-Lab-Diamond-Bezel-Ring-Rose-Gold-BE2DHB3ELC/</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2179,19 +2179,19 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/76/BE2DHB3ELC_white_top.jpg, https://image.brilliantearth.com/media/product_images/UA/BE2DHB3ELC_white_F_model.jpg, https://image.brilliantearth.com/media/product_new_images/04/BE2DHB3ELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/DA/BE2DHB3ELC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/F9/BE2DHB3ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/5U/BE2DHB3ELC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_new_images/E7/BE2DHB3ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3C/BE2DHB3ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>embed.imajize.com/654638077?v=1739866026</t>
+          <t>embed.imajize.com/127657015?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Grand-Olivetta-Eternity-Lab-Diamond-Ring-Gold-BE2D9987LC/</t>
+          <t>https://www.brilliantearth.com/Grand-Olivetta-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D9987LC/</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2201,19 +2201,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/E9/BE2D9987_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/46/BE2D9987_yellow_F_model.jpg, https://image.brilliantearth.com/media/product_images/OT/BE2D9987_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/NR/BE2D9987_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/CX/BE2D9987_rose_top.jpg, https://image.brilliantearth.com/media/product_images/8O/BE2D9987_rose_F_model.jpg, https://image.brilliantearth.com/media/product_images/2X/BE2D9987_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/ZG/BE2D9987_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>embed.imajize.com/487545492?v=1739866026</t>
+          <t>embed.imajize.com/120883390?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Grand-Versailles-Eternity-Lab-Diamond-Ring-White-Gold-BE2D3391LC/</t>
+          <t>https://www.brilliantearth.com/Grand-Versailles-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D3391LC/</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2223,19 +2223,19 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/9A/BE2D3391LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/DG/BE2D3391LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BC/BE2D3391LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/1A/BE2D3391LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/O9/BE2D3391LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/D4/BE2D3391LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>embed.imajize.com/519252759?v=1739866026</t>
+          <t>embed.imajize.com/274644739?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Channel-Set-Round-Eternity-Lab-Diamond-Ring-Gold-BE2D217LC/</t>
+          <t>https://www.brilliantearth.com/Channel-Set-Round-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D217LC/</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2245,19 +2245,19 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/05/BE2D217LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/O2/BE2D217LC-18KY_021.jpg, https://image.brilliantearth.com/media/product_images/85/BE2D217LC_BE2D812LC.jpeg, https://image.brilliantearth.com/media/product_new_images/26/BE2D217LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/00/BE2D217LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/D2/BE2D217LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/7L/BE2D217LC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_images/VD/BE2D217LC_BE2D812LC_RG_850px.jpg, https://image.brilliantearth.com/media/product_new_images/B5/BE2D217LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/1D/BE2D217LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>embed.imajize.com/146900019?v=1739866026</t>
+          <t>embed.imajize.com/745641043?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Kelly-Baguette-Eternity-Lab-Diamond-Ring-Gold-BE2D812LC/</t>
+          <t>https://www.brilliantearth.com/Kelly-Baguette-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D812LC/</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2267,19 +2267,19 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/4C/BE2D812LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/A9/BE2D812LC-18KY_011.jpg, https://image.brilliantearth.com/media/product_images/XU/BE2D217LC_BE2D812LC.jpeg, https://image.brilliantearth.com/media/product_new_images/05/BE2D812LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E4/BE2D812LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/32/BE2D812LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/JO/BE2D812LC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_images/61/BE2D217LC_BE2D812LC_RG_850px.jpg, https://image.brilliantearth.com/media/product_new_images/F4/BE2D812LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/05/BE2D812LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>embed.imajize.com/138485889?v=1739866026</t>
+          <t>embed.imajize.com/704313546?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/London-Lab-Diamond-Ring-Gold-BE2120LC/</t>
+          <t>https://www.brilliantearth.com/London-Lab-Diamond-Ring-Rose-Gold-BE2120LC/</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2289,19 +2289,19 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/8A/BE2LC120_yellow_top.png, https://image.brilliantearth.com/media/product_new_images/D7/BE2120LC_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/3D/BE2LC120_yellow_side1.png, https://image.brilliantearth.com/media/product_images/8F/BE2LC120_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/B9/BE2LC120_rose_top.png, https://image.brilliantearth.com/media/product_new_images/31/BE2120LC_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/D2/BE2LC120_rose_side1.png, https://image.brilliantearth.com/media/product_images/Y3/BE2LC120_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>embed.imajize.com/4246995?v=1739866026</t>
+          <t>embed.imajize.com/4046543?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Olivetta-Eternity-Lab-Diamond-Ring-(1-1/10-ct.-tw.)-Gold-BE2DE15103LC/</t>
+          <t>https://www.brilliantearth.com/Olivetta-Eternity-Lab-Diamond-Ring-(1-1/10-ct.-tw.)-Rose-Gold-BE2DE15103LC/</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2311,19 +2311,19 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/EB/BE2DE15103LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/T9/BE2DE15103-18KY_2.jpg, https://image.brilliantearth.com/media/product_images/5S/BE2DE15103_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/24/BE2DE15103LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/06/BE2DE15103LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/RI/BE2DE15103-rose_2.jpg, https://image.brilliantearth.com/media/product_images/OW/BE2DE15103_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/CE/BE2DE15103LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>embed.imajize.com/4924997?v=1739866026</t>
+          <t>embed.imajize.com/4712436?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Naya-Eternity-Lab-Diamond-Ring-Gold-BE2D8726LC/</t>
+          <t>https://www.brilliantearth.com/Naya-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D8726LC/</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2333,19 +2333,19 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/41/BE2D8726LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/AF/BE2D8726LC_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/20/BE2D8726LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BF/BE2D8726LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/7E/BE2D8726LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/5E/BE2D8726LC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/5B/BE2D8726LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/61/BE2D8726LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>embed.imajize.com/5789684?v=1739866026</t>
+          <t>embed.imajize.com/8448040?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Oval-Eternity-Lab-Diamond-Ring-(4-ct.-tw.)-Gold-BE2DOV400ELC/</t>
+          <t>https://www.brilliantearth.com/Oval-Eternity-Lab-Diamond-Ring-(4-ct.-tw.)-Rose-Gold-BE2DOV400ELC/</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2355,7 +2355,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/4C/BE2DOV400ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/4V/BE2D400OVE_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/E7/BE2DOV400ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/32/BE2DOV400ELC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/D3/BE2DOV400ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/V5/BE2D400OVE_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/18/BE2DOV400ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BC/BE2DOV400ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
@@ -2363,7 +2363,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/French-Pavé-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-White-Gold-BE2M300ETLC/</t>
+          <t>https://www.brilliantearth.com/French-Pavé-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-Rose-Gold-BE2M300ETLC/</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2373,19 +2373,19 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/ZQ/BE2M300ETLC_18KW_top.jpg, https://image.brilliantearth.com/media/product_images/3S/BE2M300ET-18KW_011.webp, https://image.brilliantearth.com/media/product_images/CB/BE2M300ET-18KW-S6_006.jpg, https://image.brilliantearth.com/media/product_images/3M/BE2M300ETLC_white_side.jpg, https://image.brilliantearth.com/media/product_images/ZF/BE2M300ET_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/00/BE2M300ETLC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/19/BE2M300ETLC_14KR_top.jpg, https://image.brilliantearth.com/media/product_images/4J/BE2M300ET-rose_011.jpg, https://image.brilliantearth.com/media/product_images/O3/BE2M300ET-rose-S6_006.jpg, https://image.brilliantearth.com/media/product_images/SC/BE2M300ETLC_rose_side.jpg, https://image.brilliantearth.com/media/product_images/GW/BE2M300ET_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/E2/BE2M300ETLC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9354014?v=1739866026</t>
+          <t>embed.imajize.com/4347327?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/East-West-Bezel-Emerald-Cut-Eternity-Lab-Diamond-Ring-Gold-BE2D1646LC/</t>
+          <t>https://www.brilliantearth.com/East-West-Bezel-Emerald-Cut-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D1646LC/</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2395,19 +2395,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/8A/BE2D1646_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/HX/BE2D1646LC-18KY_014.jpg, https://image.brilliantearth.com/media/product_images/9C/BE2D1646_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/11/BE2D1646_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/UO/BE2D1646_rose_top.jpg, https://image.brilliantearth.com/media/product_images/PE/BE2D1646LC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_images/8P/BE2D1646_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/B4/BE2D1646_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>embed.imajize.com/665458257?v=1739866026</t>
+          <t>embed.imajize.com/219167232?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Sienna-Three-Quarter-Coverage-Lab-Diamond-Ring-(5/8-ct.-tw.)-Rose-Gold-BE2M3420LC/</t>
+          <t>https://www.brilliantearth.com/Sienna-Three-Quarter-Coverage-Lab-Diamond-Ring-(5/8-ct.-tw.)-Rose-Rose-Gold-BE2M3420LC/</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2422,14 +2422,14 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>embed.imajize.com/6657876?v=1739866026</t>
+          <t>embed.imajize.com/6657876?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Three-Row-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-White-Gold-BE2D360LC/</t>
+          <t>https://www.brilliantearth.com/Three-Row-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-Rose-Gold-BE2D360LC/</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2439,19 +2439,19 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/0F/BE2D360LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/6B/BE2D360LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/19/BE2D360LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/59/BE2D360LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/0A/BE2D360LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/AF/BE2D360LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>embed.imajize.com/536176158?v=1739866026</t>
+          <t>embed.imajize.com/363308033?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Frances-Eternity-Lab-Diamond-Ring-Gold-BE2D6388LC/</t>
+          <t>https://www.brilliantearth.com/Frances-Eternity-Lab-Diamond-Ring-Rose-Gold-BE2D6388LC/</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2461,19 +2461,19 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/2W/BE2D6388LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/I5/BE2D6388LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/9F/BE2D6388LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/ZK/BE2D6388LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/Q2/BE2D6388LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/8C/BE2D6388LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>embed.imajize.com/594509374?v=1739866026</t>
+          <t>embed.imajize.com/537850886?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Radiant-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2DRA200ELC/</t>
+          <t>https://www.brilliantearth.com/Radiant-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2DRA200ELC/</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2483,19 +2483,19 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/CR/BE2DRA200E_white_top.jpg, https://image.brilliantearth.com/media/product_images/66/BE2D200RAE_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/DM/BE2DRA200E_white_side1.jpg, https://image.brilliantearth.com/media/product_images/47/BE2DRA200E_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/K1/BE2DRA200E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/5E/BE2D200RAE_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/Z2/BE2DRA200E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/32/BE2DRA200E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>embed.imajize.com/931557702?v=1739866026</t>
+          <t>embed.imajize.com/627348165?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Five-Stone-Contour-Lab-Diamond-Ring-(1-ct.-tw.)-White-Gold-BE2D864LC/</t>
+          <t>https://www.brilliantearth.com/Five-Stone-Contour-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D864LC/</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2505,19 +2505,19 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/03/BE2D864LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/FM/BE2D864LC-18KW_012.jpg, https://image.brilliantearth.com/media/product_images/PR/Holiday_Campaign_PDP_Crops-14_PDP_image_square.jpg, https://image.brilliantearth.com/media/product_new_images/72/BE2D864LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/41/BE2D864LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/6C/BE2D864LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/JO/BE2D864LC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_new_images/B5/BE2D864LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/13/BE2D864LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>embed.imajize.com/456439268?v=1739866026</t>
+          <t>embed.imajize.com/823116770?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Heart-Shaped-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2DHRT200ELC/</t>
+          <t>https://www.brilliantearth.com/Heart-Shaped-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2DHRT200ELC/</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2527,19 +2527,19 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/0A/BE2DHRT200ELC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/04/BE2DHRT200ELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/1E/BE2DHRT200ELC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/EC/BE2DHRT200ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/26/BE2DHRT200ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/47/BE2DHRT200ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>embed.imajize.com/883568357?v=1739866026</t>
+          <t>embed.imajize.com/373250307?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/French-Pavé-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-White-Gold-BE2M100ETLC/</t>
+          <t>https://www.brilliantearth.com/French-Pavé-Eternity-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2M100ETLC/</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2549,19 +2549,19 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/72/BE2M100ETLC_white_top.jpg, https://image.brilliantearth.com/media/product_images/AI/BE2M100ET-18KW-S6_024.jpg, https://image.brilliantearth.com/media/product_images/UQ/BE2M100ET_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/XV/BE2M100ET_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/33/BE2M100ETLC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/91/BE2M100ETLC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/PT/BE2M100ET-rose-S6_024.jpg, https://image.brilliantearth.com/media/product_images/DC/BE2M100ET_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/84/BE2M100ET_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E1/BE2M100ETLC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9889133?v=1739866026</t>
+          <t>embed.imajize.com/8510810?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Stacia-Lab-Diamond-Wedding-Ring-Gold-BE2D11310LC/</t>
+          <t>https://www.brilliantearth.com/Stacia-Lab-Diamond-Wedding-Ring-Rose-Gold-BE2D11310LC/</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2571,19 +2571,19 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/R7/BE2D11310_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/A9/BE2D11310LC_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/QT/BE2D11310_yellow_side.jpg, https://image.brilliantearth.com/media/product_images/0O/BE2D11310_yellow_hand_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/2D/BE2D11310_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/E2/BE2D11310LC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/1J/BE2D11310_rose_side.jpg, https://image.brilliantearth.com/media/product_images/EN/BE2D11310_rose_hand_zi.png</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>embed.imajize.com/143381892?v=1739866026</t>
+          <t>embed.imajize.com/571262161?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Anthology-Half-Coverage-Lab-Diamond-Ring-(2/3-ct.-tw.)-White-Gold-BE2D1025LC/</t>
+          <t>https://www.brilliantearth.com/Anthology-Half-Coverage-Lab-Diamond-Ring-(2/3-ct.-tw.)-Rose-Gold-BE2D1025LC/</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2593,19 +2593,19 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/RE/BE2D1025_white_top.jpg, https://image.brilliantearth.com/media/product_images/GT/BE2D1025-18KW_2.jpg, https://image.brilliantearth.com/media/product_images/TP/BE2D1025_white_additional1.jpeg, https://image.brilliantearth.com/media/product_images/SV/BE2D1025_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/5D/BE2D1025LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/W0/BE2D1025_rose_top.jpg, https://image.brilliantearth.com/media/product_images/27/BE2D1025-rose_2.jpg, https://image.brilliantearth.com/media/product_images/O7/BE2D1025_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/Q1/BE2D1025_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BF/BE2D1025LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>embed.imajize.com/5418422?v=1739866026</t>
+          <t>embed.imajize.com/3602783?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Luxe-Lunette-Lab-Diamond-Ring-(1/3-ct.-tw.)-White-Gold-BE2D6532LC/</t>
+          <t>https://www.brilliantearth.com/Luxe-Lunette-Lab-Diamond-Ring-(1/3-ct.-tw.)-Rose-Gold-BE2D6532LC/</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -2615,19 +2615,19 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/F8/BE2D6532LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/GP/BE2D6532LC-18KW_009.jpg, https://image.brilliantearth.com/media/product_images/7F/BE2D6532_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E1/BE2D6532LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/AA/BE2D6532LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/5T/BE2D6532LC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_images/G7/BE2D6532_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/F2/BE2D6532LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9743926?v=1739866026</t>
+          <t>embed.imajize.com/8559659?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Ellipse-Oval-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-Gold-BE2D8395LC/</t>
+          <t>https://www.brilliantearth.com/Ellipse-Oval-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-Rose-Gold-BE2D8395LC/</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -2637,19 +2637,19 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/20/BE2D8395LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/3B/BE2D8395LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/3E/BE2D8395LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/38/BE2D8395LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/D3/BE2D8395LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/51/BE2D8395LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>embed.imajize.com/791988861?v=1739866026</t>
+          <t>embed.imajize.com/212311819?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(4-ct.-tw.)-White-Gold-BE2DEM400ELC/</t>
+          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(4-ct.-tw.)-Rose-Gold-BE2DEM400ELC/</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -2659,19 +2659,19 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/Q4/BE2DEM400E_white_top.jpg, https://image.brilliantearth.com/media/product_images/UO/BE2D3727_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/RT/BE2DEM400E_white_side1.jpg, https://image.brilliantearth.com/media/product_images/XB/BE2DEM400E_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/GI/BE2DEM400E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/ZO/BE2D3727_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/B0/BE2DEM400E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/U0/BE2DEM400E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8821196?v=1739866026</t>
+          <t>embed.imajize.com/7882438?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Channel-Set-Baguette-Lab-Diamond-Ring-(1-ct.-tw.)-Gold-BE2D17CBLC/</t>
+          <t>https://www.brilliantearth.com/Channel-Set-Baguette-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D17CBLC/</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -2681,19 +2681,19 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/CD/BE2D17CB_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/BC/BE2D17CBLC_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/6D/BE2D17CB_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/B4/BE2D17CB_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/77/BE2D17CB_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/C7/BE2D17CB_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/BE/BE2D17CBLC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/4K/BE2D17CB_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/36/BE2D17CB_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/A7/BE2D17CB_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>embed.imajize.com/3702929?v=1739866026</t>
+          <t>embed.imajize.com/8086659?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Frances-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-Gold-BE2D6378LC/</t>
+          <t>https://www.brilliantearth.com/Frances-Lab-Diamond-Ring-(1-1/2-ct.-tw.)-Rose-Gold-BE2D6378LC/</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -2703,19 +2703,19 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/C4/BE2D6378LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/0C/BE2D6378LC_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/5H/BE2D6378LC-18KY_032.jpg, https://image.brilliantearth.com/media/product_new_images/78/BE2D6378LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/6F/BE2D6378LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/D4/BE2D6378LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/43/BE2D6378LC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/69/BE2D6378LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/50/BE2D6378LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>embed.imajize.com/558081793?v=1739866026</t>
+          <t>embed.imajize.com/701158347?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Ellora-Three-Quarter-Coverage-Lab-Diamond-Ring-(1-2/5-ct.-tw.)-White-Gold-BE2D8721PLC/</t>
+          <t>https://www.brilliantearth.com/Ellora-Three-Quarter-Coverage-Lab-Diamond-Ring-(1-2/5-ct.-tw.)-Rose-Gold-BE2D8721PLC/</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2725,19 +2725,19 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/SH/BE2D8721P_white_top.jpg, https://image.brilliantearth.com/media/product_images/1V/BE2D8721P-18KW_023.jpg, https://image.brilliantearth.com/media/product_images/YA/BE2D8721P_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/AP/BE2D8721P_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BB/BE2D8721PLC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/6H/BE2D8721P_rose_top.jpg, https://image.brilliantearth.com/media/product_images/X5/BE2D8721P-rose_BE5D909-18KW_023.jpg, https://image.brilliantearth.com/media/product_images/2M/BE2D8721P_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/VI/BE2D8721P_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/FF/BE2D8721PLC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>embed.imajize.com/7306013?v=1739866026</t>
+          <t>embed.imajize.com/1059235?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-White-Gold-BE2DEM300ELC/</t>
+          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-Rose-Gold-BE2DEM300ELC/</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2747,19 +2747,19 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/TP/BE2DEM300E_white_top.jpg, https://image.brilliantearth.com/media/product_images/YJ/BE2D3326_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/XG/BE2DEM300E_white_side1.jpg, https://image.brilliantearth.com/media/product_images/UA/BE2DEM300E_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/EF/BE2DEM300E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/M7/BE2D3326_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/87/BE2DEM300E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/QC/BE2DEM300E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>embed.imajize.com/465828215?v=1739866026</t>
+          <t>embed.imajize.com/566345360?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Gemma-Baguette-Lab-Diamond-Ring-(1/2-ct.-tw.)-Gold-BE2D084BLC/</t>
+          <t>https://www.brilliantearth.com/Gemma-Baguette-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D084BLC/</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -2769,19 +2769,19 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/YE/BE2D084B_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/7L/BE2D084B-18KY_070.jpg, https://image.brilliantearth.com/media/product_images/2G/BE2D084B_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/KS/BE2D084B_yellow_side.jpg, https://image.brilliantearth.com/media/product_images/9Z/BE2D084B_yellow_hand_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/W7/BE2D084B_rose_top.jpg, https://image.brilliantearth.com/media/product_images/V4/BE2D084B-18KR_070.jpg, https://image.brilliantearth.com/media/product_images/C5/BE2D084B_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/DK/BE2D084B_rose_side.jpg, https://image.brilliantearth.com/media/product_images/XN/BE2D084B_rose_hand_ms_zi.png</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>embed.imajize.com/1225476?v=1739866026</t>
+          <t>embed.imajize.com/2387605?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Heart-Shaped-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-White-Gold-BE2DHRT300ELC/</t>
+          <t>https://www.brilliantearth.com/Heart-Shaped-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-Rose-Gold-BE2DHRT300ELC/</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -2791,19 +2791,19 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/15/BE2DHRT300ELC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/98/BE2DHRT300ELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/1A/BE2DHRT300ELC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/56/BE2DHRT300ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/18/BE2DHRT300ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/AA/BE2DHRT300ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>embed.imajize.com/937465717?v=1739866026</t>
+          <t>embed.imajize.com/134808244?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Jardiniere-Lab-Diamond-Ring-Gold-BE2D835LC/</t>
+          <t>https://www.brilliantearth.com/Jardiniere-Lab-Diamond-Ring-Rose-Gold-BE2D835LC/</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -2813,19 +2813,19 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/CD/BE2D835_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/PJ/BE2D835-18KY_2.jpg, https://image.brilliantearth.com/media/product_images/76/BE2D835-18KY_3.jpg, https://image.brilliantearth.com/media/product_new_images/52/BE2D835_yellow_side1.jpg, https://image.brilliantearth.com/media/product_images/48/BE2D835_yellow_additional1.jpeg, https://image.brilliantearth.com/media/product_new_images/E5/BE2D835_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/GA/BE2D835_rose_top.jpg, https://image.brilliantearth.com/media/product_images/8Q/BE2D835-rose_2.jpg, https://image.brilliantearth.com/media/product_images/1W/BE2D835-rose_3.jpg, https://image.brilliantearth.com/media/product_new_images/28/BE2D835_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/HJ/BE2D835_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/44/BE2D835_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>embed.imajize.com/6117522?v=1739866026</t>
+          <t>embed.imajize.com/6391173?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2DEM200ELC/</t>
+          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2DEM200ELC/</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -2835,19 +2835,19 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/DP/BE2DEM200E_white_top.jpg, https://image.brilliantearth.com/media/product_images/5S/BE2D2721LC-PT_024.jpg, https://image.brilliantearth.com/media/product_images/IO/BE2D2721-18KW_049_1.jpg, https://image.brilliantearth.com/media/product_images/QG/BE2DEM200E_white_side1.jpg, https://image.brilliantearth.com/media/product_images/M4/BE2DEM200E_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/EF/BE2DEM200E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/1Q/BE2D2721LC-14KR_024.jpg, https://image.brilliantearth.com/media/product_images/ES/BE2D2721-rose_BE4M616-rose_049.jpg, https://image.brilliantearth.com/media/product_images/75/BE2DEM200E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/IH/BE2DEM200E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>embed.imajize.com/960480427?v=1739866026</t>
+          <t>embed.imajize.com/747853036?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Marseille-Three-Quarter-Coverage-Lab-Diamond-Ring-(1/2-ct.-tw.)-Gold-BE2D2774LC/</t>
+          <t>https://www.brilliantearth.com/Marseille-Three-Quarter-Coverage-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D2774LC/</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -2857,19 +2857,19 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/70/BE2D2774_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/23/BE2D2774-yellow_2.jpg, https://image.brilliantearth.com/media/product_images/H9/BE2D2774-yellow.jpg, https://image.brilliantearth.com/media/product_images/QF/BE2D2774_yellow_side.jpg, https://image.brilliantearth.com/media/product_images/MO/BE2D2774_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/CD/BE2D2774_rose_top.jpg, https://image.brilliantearth.com/media/product_images/Q5/BE2D2774-rose_2.jpg, https://image.brilliantearth.com/media/product_images/IR/BE2D2774-rose.jpg, https://image.brilliantearth.com/media/product_images/PO/BE2D2774_rose_side.jpg, https://image.brilliantearth.com/media/product_images/SF/BE2D2774_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9688818?v=1739866026</t>
+          <t>embed.imajize.com/1391317?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Grand-Versailles-Lab-Diamond-Ring-(2-1/4-ct.-tw.)-White-Gold-BE2D4390LC/</t>
+          <t>https://www.brilliantearth.com/Grand-Versailles-Lab-Diamond-Ring-(2-1/4-ct.-tw.)-Rose-Gold-BE2D4390LC/</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -2879,19 +2879,19 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/4C/BE2D4390LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/56/BE2D4390LC_white_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/AF/BE2D4390LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/32/BE2D4390LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/89/BE2D4390LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/F8/BE2D4390LC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_new_images/28/BE2D4390LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/77/BE2D4390LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8403560?v=1739866026</t>
+          <t>embed.imajize.com/3034093?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(4-ct.-tw.)-White-Gold-BE2SD14R4LC/</t>
+          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(4-ct.-tw.)-Rose-Gold-BE2SD14R4LC/</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -2901,19 +2901,19 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/9F/BE2SD14R4LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/71/BE2SD14R4-18KW-S6_029.jpg, https://image.brilliantearth.com/media/product_images/3R/BE2SD14R4_white_additional1.webp, https://image.brilliantearth.com/media/product_images/TO/BE2SD14R4LC_white_side.jpg, https://image.brilliantearth.com/media/product_new_images/8E/BE2SD14R4LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/46/BE2SD14R4LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/H5/BE2SD14R4-rose-S6_029.jpg, https://image.brilliantearth.com/media/product_images/4Z/BE2SD14R4_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/ZQ/BE2SD14R4LC_rose_side.jpg, https://image.brilliantearth.com/media/product_new_images/74/BE2SD14R4LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>embed.imajize.com/4439029?v=1739866026</t>
+          <t>embed.imajize.com/9351799?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Pear-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-White-Gold-BE2D9988LC/</t>
+          <t>https://www.brilliantearth.com/Pear-Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2D9988LC/</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -2923,19 +2923,19 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/QP/WG0.jpg, https://image.brilliantearth.com/media/product_images/5N/WG2.jpg, https://image.brilliantearth.com/media/product_images/T6/WG1_hand_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/GZ/RG0.jpg, https://image.brilliantearth.com/media/product_images/ZO/RG2.jpg, https://image.brilliantearth.com/media/product_images/5I/RG1_hand_ms_zi.png</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8624631?v=1739866026</t>
+          <t>embed.imajize.com/8843904?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Radiant-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-White-Gold-BE2DRA300ELC/</t>
+          <t>https://www.brilliantearth.com/Radiant-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-Rose-Gold-BE2DRA300ELC/</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -2945,19 +2945,19 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/S7/BE2DRA300E_white_top.jpg, https://image.brilliantearth.com/media/product_images/4X/BE2D300RAELC-PT_017.jpg, https://image.brilliantearth.com/media/product_images/AW/BE2DRA300E_white_side1.jpg, https://image.brilliantearth.com/media/product_images/UE/BE2DRA300E_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/M3/BE2DRA300E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/26/BE2D300RAELC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_images/C1/BE2DRA300E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/GK/BE2DRA300E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>embed.imajize.com/9168740?v=1739866026</t>
+          <t>embed.imajize.com/8367163?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(5-ct.-tw.)-White-Gold-BE2DEM500ELC/</t>
+          <t>https://www.brilliantearth.com/Emerald-Eternity-Lab-Diamond-Ring-(5-ct.-tw.)-Rose-Gold-BE2DEM500ELC/</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -2967,19 +2967,19 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/N7/BE2DEM500E_white_top.jpg, https://image.brilliantearth.com/media/product_images/LS/BE2D500EMELC-white_011.jpg, https://image.brilliantearth.com/media/product_images/A4/BE2D500EME_white_additional1_1.jpg, https://image.brilliantearth.com/media/product_images/FZ/BE2DEM500E.white_02.jpg, https://image.brilliantearth.com/media/product_images/0M/BE2DEM500E_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/8N/BE2DEM500E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/HV/BE2D500EMELC-rose_011.jpg, https://image.brilliantearth.com/media/product_images/2N/BE2D500EME_rose_additional1_1.jpg, https://image.brilliantearth.com/media/product_images/Y3/BE2DEM500E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/AT/BE2DEM500E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>embed.imajize.com/510448432?v=1739866026</t>
+          <t>embed.imajize.com/928074727?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Anthology-Eternity-Lab-Diamond-Ring-(1-1/3-ct.-tw.)-White-Gold-BE2D1025ELC/</t>
+          <t>https://www.brilliantearth.com/Anthology-Eternity-Lab-Diamond-Ring-(1-1/3-ct.-tw.)-Rose-Gold-BE2D1025ELC/</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -2989,19 +2989,19 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/01/BE2D1025E_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/6E/BE2D1025ELC_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/PM/BE2D1025E_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/VS/BE2D1025E_white_side.jpg, https://image.brilliantearth.com/media/product_images/6N/BE2D1025_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/XZ/BE2D1025E_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/F8/BE2D1025ELC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/O3/BE2D1025E_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/OE/BE2D1025E_rose_side.jpg, https://image.brilliantearth.com/media/product_images/8B/BE2D1025_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>embed.imajize.com/342379049?v=1739866026</t>
+          <t>embed.imajize.com/644152139?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Oval-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-White-Gold-BE2DOV300ELC/</t>
+          <t>https://www.brilliantearth.com/Oval-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-Rose-Gold-BE2DOV300ELC/</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3011,19 +3011,19 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/AY/BE2DOV300E_white_top.jpg, https://image.brilliantearth.com/media/product_images/2O/BE2D300OVELC-white_056.jpg, https://image.brilliantearth.com/media/product_images/DH/BE2D300OVE_white_additional1_1.jpg, https://image.brilliantearth.com/media/product_images/V6/BE2DOV300E_white_side1.jpg, https://image.brilliantearth.com/media/product_images/65/BE2DOV300E_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/7H/BE2DOV300E_rose_top.jpg, https://image.brilliantearth.com/media/product_images/K0/BE2D300OVELC-rose_056.jpg, https://image.brilliantearth.com/media/product_images/B8/BE2D300OVE_rose_additional1_1.jpg, https://image.brilliantearth.com/media/product_images/AG/BE2DOV300E_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/MK/BE2DOV300E_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>embed.imajize.com/629642679?v=1739866026</t>
+          <t>embed.imajize.com/561327087?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Gianna-Pavé-Lab-Diamond-Ring-(1-1/3-ct.-tw.)-White-Gold-BE2D5001LC/</t>
+          <t>https://www.brilliantearth.com/Gianna-Pavé-Lab-Diamond-Ring-(1-1/3-ct.-tw.)-Rose-Gold-BE2D5001LC/</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -3033,19 +3033,19 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/V8/BE2D5001_white_00.jpg, https://image.brilliantearth.com/media/product_images/D6/BE2D5001_white_02.jpg, https://image.brilliantearth.com/media/product_new_images/56/BE2D5001_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/DS/BE2D5001_rose_00.jpg, https://image.brilliantearth.com/media/product_images/FP/BE2D5001_rose_02.jpg, https://image.brilliantearth.com/media/product_new_images/9B/BE2D5001_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>embed.imajize.com/3769760?v=1739866026</t>
+          <t>embed.imajize.com/9872353?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Emerald-Cut-Lab-Diamond-Ring-Gold-BE2D783LC/</t>
+          <t>https://www.brilliantearth.com/Emerald-Cut-Lab-Diamond-Ring-Rose-Gold-BE2D783LC/</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3055,19 +3055,19 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/AA/BE2D783_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/C4/BE2D783LC-18KY_011.jpg, https://image.brilliantearth.com/media/product_images/UK/BE2D783_yellow_side.jpg, https://image.brilliantearth.com/media/product_new_images/78/BE2D783_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/8A/BE2D783_rose_top.jpg, https://image.brilliantearth.com/media/product_images/HD/BE2D783LC_rose_F_model.jpg, https://image.brilliantearth.com/media/product_images/AU/BE2D783_rose_side.jpg, https://image.brilliantearth.com/media/product_new_images/DD/BE2D783_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8910377?v=1739866026</t>
+          <t>embed.imajize.com/1191011?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(5-ct.-tw.)-White-Gold-BE2U30D43LC/</t>
+          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(5-ct.-tw.)-Rose-Gold-BE2U30D43LC/</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3077,19 +3077,19 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/30/BE2U30D43LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/JB/BE2U30D43-18KW-S65_047.jpg, https://image.brilliantearth.com/media/product_images/X8/BE2U30D43LC_white_side.jpg, https://image.brilliantearth.com/media/product_new_images/03/BE2U30D43LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/52/BE2U30D43LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/E6/BE2U30D43-rose-S65_047.jpg, https://image.brilliantearth.com/media/product_images/E6/BE2U30D43LC_rose_side.jpg, https://image.brilliantearth.com/media/product_new_images/9E/BE2U30D43LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8517052?v=1739866026</t>
+          <t>embed.imajize.com/5668707?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Trillion-Cut-Lab-Diamond-Ring-Gold-BE2D1537LC/</t>
+          <t>https://www.brilliantearth.com/Trillion-Cut-Lab-Diamond-Ring-Rose-Gold-BE2D1537LC/</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -3099,19 +3099,19 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/Q7/BE2D1537LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/B2/BE2D1537LC_yellow_side.jpg, https://image.brilliantearth.com/media/product_images/04/BE2D1537LC_yellow_hand_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/LB/BE2D1537LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/HM/BE2D1537LC_rose_side.jpg, https://image.brilliantearth.com/media/product_images/RN/BE2D1537LC_rose_hand_ms_zi.png</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>embed.imajize.com/5668938?v=1739866026</t>
+          <t>embed.imajize.com/9011984?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Riviera-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-Gold-BE2DR300ELC/</t>
+          <t>https://www.brilliantearth.com/Riviera-Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-Rose-Gold-BE2DR300ELC/</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -3121,19 +3121,19 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/78/BE2DR300ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/CY/Perfect_Collection_-_Imagery_Crops_1x1-13_copy.jpg, https://image.brilliantearth.com/media/product_new_images/33/BE2DR300ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/CD/BE2DR300ELC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/07/BE2DR300ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/1N/Perfect_Collection_-_Imagery_Crops_1x1-13_copy.jpg, https://image.brilliantearth.com/media/product_new_images/B5/BE2DR300ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/34/BE2DR300ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>embed.imajize.com/241977123?v=1739866026</t>
+          <t>embed.imajize.com/892903475?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Gold-BE2U10D3LC/</t>
+          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2U10D3LC/</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -3143,19 +3143,19 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/RY/BE2U10D3_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/C3/BE2U10D3_yellow_additional1.jpg, https://image.brilliantearth.com/media/product_images/0M/BE2U10D3LC_yellow_side.png, https://image.brilliantearth.com/media/product_new_images/42/BE2U10D3LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/5Z/BE2U10D3_rose_top.jpg, https://image.brilliantearth.com/media/product_images/HV/BE2U10D3_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/AV/BE2U10D3_rose_side.png, https://image.brilliantearth.com/media/product_new_images/7B/BE2U10D3LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8283512?v=1739866026</t>
+          <t>embed.imajize.com/6604007?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-Gold-BE2SD20R3LC/</t>
+          <t>https://www.brilliantearth.com/Eternity-Lab-Diamond-Ring-(3-ct.-tw.)-Rose-Gold-BE2SD20R3LC/</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -3165,19 +3165,19 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/95/BE2SD20R3LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_images/RD/BE2SD20R3-yellow-S6_020.jpg, https://image.brilliantearth.com/media/product_images/AV/BE2SD20R3LC_yellow_side.jpg, https://image.brilliantearth.com/media/product_new_images/27/BE2SD20R3LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/79/BE2SD20R3LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/S7/BE2SD20R3-rose-S6_020.jpg, https://image.brilliantearth.com/media/product_images/9J/BE2SD20R3LC_rose_side.jpg, https://image.brilliantearth.com/media/product_new_images/28/BE2SD20R3LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>embed.imajize.com/6169472?v=1739866026</t>
+          <t>embed.imajize.com/8783747?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Yellow-Lab-Diamond-Ring-(1/4-ct.-tw.)-Gold-BE2D318LC/</t>
+          <t>https://www.brilliantearth.com/Yellow-Lab-Diamond-Ring-(1/4-ct.-tw.)-Rose-Gold-BE2D318LC/</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3187,19 +3187,19 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/7A/BE2D318LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/1A/BE2D318LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/E4/BE2D318LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/9C/BE2D318LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/EA/BE2D318LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/BA/BE2D318LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>embed.imajize.com/914585612?v=1739866026</t>
+          <t>embed.imajize.com/843740417?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Riviera-Eternity-Lab-Diamond-Ring-(4-ct.-tw.)-White-Gold-BE2DR400ELC/</t>
+          <t>https://www.brilliantearth.com/Riviera-Eternity-Lab-Diamond-Ring-(4-ct.-tw.)-Rose-Gold-BE2DR400ELC/</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3209,19 +3209,19 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/AB/BE2DR400ELC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/33/BE2DR400ELC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/82/BE2DR400ELC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/67/BE2DR400ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/3B/BE2DR400ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/49/BE2DR400ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>embed.imajize.com/245348583?v=1739866026</t>
+          <t>embed.imajize.com/372945496?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Eternity-Yellow-Lab-Diamond-Ring-(2-ct.-tw.)-Gold-BE2D291ELC/</t>
+          <t>https://www.brilliantearth.com/Eternity-Yellow-Lab-Diamond-Ring-(2-ct.-tw.)-Rose-Gold-BE2D291ELC/</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3231,19 +3231,19 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/A7/BE2D291ELC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/6F/BE2D291ELC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/F4/BE2D291ELC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/D4/BE2D291ELC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/97/BE2D291ELC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/EA/BE2D291ELC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>embed.imajize.com/784150267?v=1739866026</t>
+          <t>embed.imajize.com/867871990?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/French-Pavé-Eternity-Lab-Diamond-Ring-(4-1/2-ct.-tw.)-White-Gold-BE2D0664LC/</t>
+          <t>https://www.brilliantearth.com/French-Pavé-Eternity-Lab-Diamond-Ring-(4-1/2-ct.-tw.)-Rose-Gold-BE2D0664LC/</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3253,19 +3253,19 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/HB/BE2D0664_white_top.jpg, https://image.brilliantearth.com/media/product_images/Z0/BE2D0664LC-18KW_013.jpg, https://image.brilliantearth.com/media/product_new_images/03/BE2D0664_white_side1.jpg, https://image.brilliantearth.com/media/product_images/5J/BE2D0664_white_hand_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/HA/BE2D0664_rose_top.jpg, https://image.brilliantearth.com/media/product_images/GA/BE2D0664LC-rose_F_model.jpg, https://image.brilliantearth.com/media/product_new_images/E8/BE2D0664_rose_side1.jpg, https://image.brilliantearth.com/media/product_images/UB/BE2D0664_rose_hand_ms_zi.png</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8916869?v=1739866026</t>
+          <t>embed.imajize.com/8691845?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Yellow-Lab-Diamond-Ring-(1/2-ct.-tw.)-White-Gold-BE2D585LC/</t>
+          <t>https://www.brilliantearth.com/Yellow-Lab-Diamond-Ring-(1/2-ct.-tw.)-Rose-Gold-BE2D585LC/</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -3275,19 +3275,19 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/A3/BE2D585LC_white_top.jpg, https://image.brilliantearth.com/media/product_new_images/95/BE2D585LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/22/BE2D585LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/35/BE2D585LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/11/BE2D585LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/7A/BE2D585LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>embed.imajize.com/630200619?v=1739866026</t>
+          <t>embed.imajize.com/445942314?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Seven-Stone-Trellis-Lab-Diamond-Ring-(7/8-ct.-tw.)-White-Gold-BE2D33T7STLC/</t>
+          <t>https://www.brilliantearth.com/Seven-Stone-Trellis-Lab-Diamond-Ring-(7/8-ct.-tw.)-Rose-Gold-BE2D33T7STLC/</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -3297,19 +3297,19 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_images/L7/BE2C733_white_top.jpg, https://image.brilliantearth.com/media/product_images/MP/BE2C5380_white_additional1.jpg, https://image.brilliantearth.com/media/product_images/1K/BE2C733_white_side.jpg, https://image.brilliantearth.com/media/product_images/7A/BE2C733_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_images/4U/BE2C733_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/B3/BE2D33T7STLC_rose_additional1.jpg, https://image.brilliantearth.com/media/product_images/PT/BE2C733_rose_side.jpg, https://image.brilliantearth.com/media/product_images/YZ/BE2C733_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>embed.imajize.com/4706910?v=1739866026</t>
+          <t>embed.imajize.com/1572151?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Yellow-Lab-Diamond-Ring-(1-ct.-tw.)-Gold-BE2D938LC/</t>
+          <t>https://www.brilliantearth.com/Yellow-Lab-Diamond-Ring-(1-ct.-tw.)-Rose-Gold-BE2D938LC/</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3319,19 +3319,19 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/7D/BE2D938LC_yellow_top.jpg, https://image.brilliantearth.com/media/product_new_images/59/BE2D938LC_yellow_side1.jpg, https://image.brilliantearth.com/media/product_new_images/50/BE2D938LC_yellow_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/D7/BE2D938LC_rose_top.jpg, https://image.brilliantearth.com/media/product_new_images/68/BE2D938LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/42/BE2D938LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>embed.imajize.com/782047239?v=1739866026</t>
+          <t>embed.imajize.com/836484200?v=1741166123</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>https://www.brilliantearth.com/Portia-Lab-Diamond-Ring-(1-1/3-ct.-tw.)-White-Gold-BE2D1628LC/</t>
+          <t>https://www.brilliantearth.com/Portia-Lab-Diamond-Ring-(1-1/3-ct.-tw.)-Rose-Gold-BE2D1628LC/</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3341,12 +3341,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>https://image.brilliantearth.com/media/product_new_images/3C/BE2D1628LC_white_top.jpg, https://image.brilliantearth.com/media/product_images/B7/BE2D1628LC-PT_016.jpg, https://image.brilliantearth.com/media/product_images/CH/BE2D1628LC_white_side1.jpg, https://image.brilliantearth.com/media/product_new_images/94/BE2D1628LC_white_ms_zi.png</t>
+          <t>https://image.brilliantearth.com/media/product_new_images/6C/BE2D1628LC_rose_top.jpg, https://image.brilliantearth.com/media/product_images/4E/BE2D1628LC-rose_F_model.jpg, https://image.brilliantearth.com/media/product_images/IW/BE2D1628LC_rose_side1.jpg, https://image.brilliantearth.com/media/product_new_images/D6/BE2D1628LC_rose_ms_zi.png</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>embed.imajize.com/8311725?v=1739866026</t>
+          <t>embed.imajize.com/1259499?v=1741166123</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scrape Grow Brillience ring data
</commit_message>
<xml_diff>
--- a/py_scraper/product_data.xlsx
+++ b/py_scraper/product_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D102"/>
+  <dimension ref="A1:D103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,21 +453,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/8-1-4-ctw-radiant-lab-grown-diamond-bridal-set-platinum/pid/BRDTXR08803T500PL2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>8 1/4 ctw Radiant Lab Grown Diamond Bridal Set</t>
-        </is>
-      </c>
+          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr"/>
@@ -477,7 +473,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr"/>
@@ -487,7 +483,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B5" t="inlineStr"/>
@@ -497,17 +493,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1 1/5 ctw Princess Lab Grown Diamond Split Shank Halo Engagement Ring</t>
+        </is>
+      </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B7" t="inlineStr"/>
@@ -517,7 +517,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-6-7-8-ctw-emerald-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ7731XX-PL4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
@@ -527,7 +527,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-3-1-2-ctw-round-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ78940H-HW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B9" t="inlineStr"/>
@@ -537,7 +537,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/8-1-4-ctw-radiant-lab-grown-diamond-bridal-set-platinum/pid/BRDTXR08803T500PL2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B10" t="inlineStr"/>
@@ -547,7 +547,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-2-5-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-18k-white-gold/pid/RIGTX06766R500-HW1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-6-7-8-ctw-emerald-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ7731XX-PL4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B11" t="inlineStr"/>
@@ -557,7 +557,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-round-lab-grown-diamond-three-stone-ring-18k-white-gold/pid/RIGJRD0315-HW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b&amp;amp;in_stock=yes</t>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-3-1-2-ctw-round-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ78940H-HW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B12" t="inlineStr"/>
@@ -567,7 +567,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-oval-lab-grown-diamond-petite-solitaire-engagement-ring-14k-white-gold/pid/RGTXR05314O300-GW2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B13" t="inlineStr"/>
@@ -577,21 +577,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-2-5-ctw-oval-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR07400O300GW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b&amp;amp;in_stock=yes</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>4 2/5 ctw Oval Lab Grown Diamond Bridal Set</t>
-        </is>
-      </c>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/6-2-3-ctw-round-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR08527-GW2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -601,7 +597,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/versailles-ring-18k-white-gold/pid/RIG3STRA1050-HW6?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B16" t="inlineStr"/>
@@ -611,7 +607,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/8-2-3-ctw-pear-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/RIGTX04156D800-GY1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B17" t="inlineStr"/>
@@ -621,7 +617,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-1-2-ctw-emerald-lab-grown-diamond-three-stone-ring-platinum/pid/RIGJRD0254XX-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B18" t="inlineStr"/>
@@ -631,7 +627,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-toi-et-moi-pear-and-emerald-engagement-ring-14k-yellow-gold/pid/RIGTXR05973PE40GY1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b&amp;amp;in_stock=yes</t>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B19" t="inlineStr"/>
@@ -641,7 +637,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/9-ctw-pear-lab-grown-diamond-engagement-ring-with-split-prong-side-accents-platinum/pid/RIGRV04550D800-PL1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B20" t="inlineStr"/>
@@ -651,7 +647,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/athens-ring-18k-white-gold/pid/RIG3STEC950-HW6?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B21" t="inlineStr"/>
@@ -661,7 +657,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/brussels-ring-18k-white-gold/pid/RIG3STRDHM780-HW3?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B22" t="inlineStr"/>
@@ -671,7 +667,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-3-4-ctw-fancy-pink-cushion-lab-grown-diamond-three-stone-engagement-ring-platinum/pid/RIGTXR09165-PN-PL4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B23" t="inlineStr"/>
@@ -681,7 +677,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-5-1-2-ctw-round-lab-grown-diamond-bypass-engagement-ring-platinum/pid/RIGJRZ758806R5-PL1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B24" t="inlineStr"/>
@@ -691,7 +687,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-trellis-solitaire-engagement-ring-14k-white-gold/pid/RIG-JOR037-GW1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B25" t="inlineStr"/>
@@ -701,7 +697,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-3-8-ctw-cushion-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRD0257XX-HW1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B26" t="inlineStr"/>
@@ -711,7 +707,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-1-2-ctw-oval-lab-grown-diamond-braided-halo-engagement-ring-with-micro-pave-shank-platinum/pid/RIGTXR06229-OV3-PL3?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B27" t="inlineStr"/>
@@ -721,7 +717,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/7-1-3-ctw-cushion-lab-grown-diamond-eternity-engagement-ring-platinum/pid/RIG08073C50PL2-700?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B28" t="inlineStr"/>
@@ -731,7 +727,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-4-1-3-ctw-cushion-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ7836XX-C-HW4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B29" t="inlineStr"/>
@@ -741,7 +737,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-7-8-ctw-oval-lab-grown-diamond-engagement-ring-with-floating-marquise-side-accents-14k-white-gold/pid/RIG2638X2O150SOGW2?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B30" t="inlineStr"/>
@@ -751,21 +747,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-3-4-ctw-pear-lab-grown-diamond-side-stone-engagement-ring-18k-yellow-gold/pid/RIGKSR6203-GY3?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>5 3/4 ctw Pear Lab Grown Diamond Side Stone Engagement Ring</t>
-        </is>
-      </c>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-2-3-ctw-oval-lab-grown-diamond-engagement-ring-with-pear-side-accents-14k-yellow-gold/pid/RIG0615X3-O200SO-GY?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B32" t="inlineStr"/>
@@ -775,17 +767,25 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-1-2-ctw-round-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD02180H-PL1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
-      <c r="C33" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>1 1/5 ctw Princess Lab Grown Diamond Split Shank Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X2/medium/RIG0625X2-P075H1-GW_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X2/medium/RIG0625X2-P075H1-GW_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X2/medium/RIG0625X2-P075H1-GW_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X4/medium/RIG0625X4-P150H1-GW-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
+        </is>
+      </c>
       <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-1-3-ctw-oval-lab-grown-diamond-double-heart-shape-prong-split-shank-side-stone-engagement-ring-platinum/pid/RIGRVR04394O500PL2?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B34" t="inlineStr"/>
@@ -795,7 +795,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-3-4-ctw-elongated-cushion-lab-grown-diamond-side-stone-engagement-ring-18k-white-gold/pid/RIGTXR07755Z400HW1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B35" t="inlineStr"/>
@@ -805,7 +805,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-ctw-emerald-lab-grown-diamond-side-stone-engagement-ring-platinum/pid/RIGKSR6129-PL1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B36" t="inlineStr"/>
@@ -815,7 +815,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-5-8-ctw-oval-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/TXR04040-GY1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
         </is>
       </c>
       <c r="B37" t="inlineStr"/>
@@ -825,680 +825,1190 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/12x7mm-pear-cut-created-emerald-and-1-2-ctw-lab-grown-diamond-halo-engagement-ring-engagement-ring-14k-white-gold/pid/RIGTXR06627-EM-GW4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>1 ctw Round Lab Grown Diamond Double Twist Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0629X1/medium/RIG0629X1-R075SO-GW-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0629X1/medium/RIG0629X1-R075SO-GW-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0629X1R075SOGW4/medium/LGR0629X1R075SOGW4-new2-img.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/0629/medium/0629-Round-GB.jpg</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-4-ctw-emerald-lab-grown-diamond-engagement-ring-with-tapered-baguette-side-accents-14k-white-gold/pid/RIG0617X3-E200SO-GW?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
-      <c r="C39" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Radiant Lab Grown Diamond Station Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X3/medium/RIG1860X3-T200SO-GW-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X3/medium/RIG1860X3-T200SO-GW-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X1/medium/RIG1860X1-T075SO-GW-1-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X3/medium/RIG1860X3-Radiant-GW.jpg</t>
+        </is>
+      </c>
       <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-3-4-ctw-oval-lab-grown-diamond-hidden-halo-bridal-set-platinum/pid/BRDTXR06232O200PL2?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>5 ctw Emerald Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD020837/medium/RIGJRD020837-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD020837/medium/RIGJRD020837-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD020837/medium/RIGJRD020837-PL_5-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-radiant-lab-grown-diamond-solitaire-engagement-ring-platinum/pid/RIGJRO1322-PL_5?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr"/>
-      <c r="C41" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2 ctw Round Lab Grown Diamond Graduated Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0641X2/medium/RIG0641X2-R150SO-GW_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0641X2/medium/RIG0641X2-R150SO-GW_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0641X2/medium/RIG0641X2-R150SO-GW-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0589X3/medium/LGR0589X3-R200-shape.jpg</t>
+        </is>
+      </c>
       <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-1-3-ctw-princess-lab-grown-diamond-split-shank-engagement-ring-platinum/pid/LGR0625X3-P300SO-PL4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr"/>
-      <c r="C42" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-6-7-8-ctw-emerald-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ7731XX-PL4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Near-Colorless 6 7/8 ctw Emerald Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7731XX/medium/RIGJRZ7731XX-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7731XX/medium/RIGJRZ7731XX-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7731XX/medium/RIGJRZ7731XX-HW_5-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-7-8-ctw-cushion-lab-grown-diamond-graduated-halo-engagement-ring-14k-white-gold/pid/RIG0641X4C200H1GW2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr"/>
-      <c r="C43" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-3-1-2-ctw-round-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ78940H-HW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Near-Colorless 3 1/2 ctw Round Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ78940H/medium/RIGJRZ78940H-HW_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ78940H/medium/RIGJRZ78940H-HW_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ78940H/medium/RIGJRZ78940H-HW_5-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/11x9mm-created-emerald-and-1-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR06623-EM-GW4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr"/>
-      <c r="C44" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/8-1-4-ctw-radiant-lab-grown-diamond-bridal-set-platinum/pid/BRDTXR08803T500PL2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>8 1/4 ctw Radiant Lab Grown Diamond Bridal Set</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08803T500/medium/BRDTXR08803T500-WG-RD-WH-816-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08803T500/medium/BRDTXR08803T500-WG-RD-WH-816-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
       <c r="D44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-bezel-set-solitaire-engagement-ring-platinum/pid/RIGTXR06655EM500PL3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr"/>
-      <c r="C45" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-2-5-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-18k-white-gold/pid/RIGTX06766R500-HW1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 5 2/5 ctw Round Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06766R500/medium/RIGTXR06766R500-WG-RB-WH-543-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06766R500/medium/RIGTXR06766R500-WG-RB-WH-543-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTX06766R500/medium/RIGTX06766R500-GW6-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-2-3-ctw-multi-shape-lab-grown-diamond-vintage-inspired-art-deco-engagement-ring-platinum/pid/RIGRVR05013-PL4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr"/>
-      <c r="C46" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-ctw-round-lab-grown-diamond-three-stone-ring-18k-white-gold/pid/RIGJRD0315-HW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b&amp;amp;in_stock=yes</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>4 ctw Round Lab Grown Diamond Three-Stone Ring</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0315/medium/RIGJRD0315-HW4_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0315/medium/RIGJRD0315-HW4_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0315/medium/RIGJRD0315-HW4-new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/10x8-mm-created-emerald-and-1-3-8-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR06678-EM-GW4?algoliaQueryId=961725d3c54423b9205778064301ed8e&amp;amp;in_stock=yes</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr"/>
-      <c r="C47" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-ctw-oval-lab-grown-diamond-petite-solitaire-engagement-ring-14k-white-gold/pid/RGTXR05314O300-GW2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>3 ctw Oval Lab Grown Diamond Petite Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05314/medium/RIGTXR05314-WG-OV-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05314O300/medium/RIGTXR05314O300-GY4-1-NEW.jpg</t>
+        </is>
+      </c>
       <c r="D47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-2-3-ctw-oval-lab-grown-diamond-three-stone-engagement-ring-with-half-moon-sides-platinum/pid/RIGTXR06001OV30PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr"/>
-      <c r="C48" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-2-5-ctw-oval-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR07400O300GW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b&amp;amp;in_stock=yes</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>4 2/5 ctw Oval Lab Grown Diamond Bridal Set</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07400O300/medium/BRDTXR07400O300-WG-OV-WH-439-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07400O300/medium/BRDTXR07400O300-WG-OV-WH-439-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07400O300GW4/medium/BRDTXR07400O300GW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-3-4-ctw-cushion-lab-grown-diamond-split-shank-x-side-stone-engagement-ring-14k-rose-gold/pid/RIGRV08957C400-GP2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/6-2-3-ctw-round-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR08527-GW2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>6 2/3 ctw Round Lab Grown Diamond Bridal Set</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08527/medium/BRDTXR08527-WG-RB-WH-665-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08527/medium/BRDTXR08527-WG-RB-WH-665-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/6-1-4-ctw-oval-lab-grown-diamond-trapezoid-and-pear-side-stone-bridal-set-platinum/pid/BRDTXR08417O500PL4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr"/>
-      <c r="C50" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/8-2-3-ctw-pear-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/RIGTX04156D800-GY1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>8 2/3 ctw Pear Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04156D300/medium/RIGTXR04156D300-YG-PE-WH-352-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04156D300/medium/RIGTXR04156D300-YG-PE-WH-352-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
+        </is>
+      </c>
       <c r="D50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-toi-et-moi-pear-and-oval-engagement-ring-14k-white-gold/pid/RIGTXR05974PO30-GW4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr"/>
-      <c r="C51" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/5-1-2-ctw-emerald-lab-grown-diamond-three-stone-ring-platinum/pid/RIGJRD0254XX-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>5 1/2  ctw Emerald Lab Grown Diamond Three-Stone Ring</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0254XX/medium/RIGJRD0254XX-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0254XX/medium/RIGJRD0254XX-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0254/medium/RIGJRD0254-HW_5-new-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-10-ctw-oval-lab-grown-diamond-pave-prong-solitaire-engagement-ring-with-hidden-accents-14k-yellow-gold/pid/RIGTXR05578O200GY2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/4-ctw-toi-et-moi-pear-and-emerald-engagement-ring-14k-yellow-gold/pid/RIGTXR05973PE40GY1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b&amp;amp;in_stock=yes</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>2 1/10 ctw Oval Lab Grown Diamond Pave Prong Solitaire Engagement Ring with Hidden Accents</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr"/>
+          <t>4 ctw Toi Et Moi Pear and Emerald Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05973/medium/RIGTXR05973-YG-VR-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05973/medium/RIGTXR05973-YG-VR-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05973PE40/medium/RIGTXR05973PE40-GW4-new.jpg</t>
+        </is>
+      </c>
       <c r="D52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-7-8-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-platinum/pid/RIGTXR09619R300PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr"/>
-      <c r="C53" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/9-ctw-pear-lab-grown-diamond-engagement-ring-with-split-prong-side-accents-platinum/pid/RIGRV04550D800-PL1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>9 ctw Pear Lab Grown Diamond Engagement Ring with Split Prong Side Accents</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04550D800/medium/RIGRVR04550D800-WG-PE-WH-900-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04550D800/medium/RIGRVR04550D800-WG-PE-WH-900-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
+        </is>
+      </c>
       <c r="D53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-cushion-lab-grown-diamond-v-prong-halo-engagement-ring-14k-white-gold/pid/RIG0639X4C200H1GW2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr"/>
-      <c r="C54" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-3-4-ctw-fancy-pink-cushion-lab-grown-diamond-three-stone-engagement-ring-platinum/pid/RIGTXR09165-PN-PL4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>3 3/4 ctw Fancy Pink Cushion Lab Grown Diamond Three Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09165P/medium/RIGTXR09165P-WG-CU-WH-375-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09165P/medium/RIGTXR09165P-WG-CU-WH-375-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09165/medium/RIGTXR09165-YL-BL-PN%20alt%20image.jpg</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-emerald-lab-grown-diamond-solitaire-engagement-ring-platinum/pid/RIGTXR09875E400PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-5-1-2-ctw-round-lab-grown-diamond-bypass-engagement-ring-platinum/pid/RIGJRZ758806R5-PL1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 5 1/2 ctw Round Lab Grown Diamond Bypass Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ758806/medium/RIGJRZ758806-WG-RB-WH-556-M0-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ758806/medium/RIGJRZ758806-WG-RB-WH-556-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ758806R7/medium/RIGJRZ758806R7-HW6-new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/13-4mm-cushion-cut-created-emerald-and-2-ctw-pear-lab-grown-diamond-three-stone-engagement-ring-14k-yellow-gold/pid/RIGTXR08896-EM-GY4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-trellis-solitaire-engagement-ring-14k-white-gold/pid/RIG-JOR037-GW1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2 ctw Round Lab Grown Diamond Trellis Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJOR037/medium/RIGJOR037-WG-RB-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJOR037/medium/RIGJOR037-WG-RB-WH-200-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJOR037/medium/RIGJOR037-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-twist-solitaire-engagement-ring-14k-white-gold/pid/RIGTXR05112-GW4-3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr"/>
-      <c r="C57" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-3-8-ctw-cushion-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRD0257XX-HW1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 5 3/8 ctw Cushion Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0257XX/medium/RIGJRD0257XX-HW_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0257XX/medium/RIGJRD0257XX-HW_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0257XX/medium/RIGJRD0257XX-HW_5-new-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-1-2-ctw-cushion-lab-grown-diamond-halo-engagement-ring-platinum/pid/RIGKSR6111N-PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr"/>
-      <c r="C58" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-1-2-ctw-oval-lab-grown-diamond-braided-halo-engagement-ring-with-micro-pave-shank-platinum/pid/RIGTXR06229-OV3-PL3?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 3 1/2 ctw Oval Lab Grown Diamond Braided Halo Engagement Ring with Micro Pave Shank</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06229/medium/RIGTXR06229-WG-OV-WH-350-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06229/medium/RIGTXR06229-WG-OV-WH-350-M1.jpg</t>
+        </is>
+      </c>
       <c r="D58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-1-4-ctw-oval-lab-grown-diamond-three-stone-bridal-set-platinum/pid/BRDTXR08075O300PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/7-1-3-ctw-cushion-lab-grown-diamond-eternity-engagement-ring-platinum/pid/RIG08073C50PL2-700?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>7 1/3 ctw Cushion Lab Grown Diamond Eternity Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08073C500/medium/RIGTXR08073C500-WG-CU-WH-740-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08073C500/medium/RIGTXR08073C500-WG-CU-WH-740-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-1-3-ctw-princess-lab-grown-diamond-hidden-halo-engagement-ring-18k-white-gold/pid/RIGKSR6164-GW3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr"/>
-      <c r="C60" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-4-1-3-ctw-cushion-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ7836XX-C-HW4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Near-Colorless 4 1/3 ctw Cushion Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7836XX%20/medium/RIGJRZ7836XX%20-WG-CU-WH-572-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7836XX%20/medium/RIGJRZ7836XX%20-WG-CU-WH-572-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGR629X1C050/medium/RIGR629X1C050-WG-CU-WH-075-M6.png</t>
+        </is>
+      </c>
       <c r="D60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-1-5-ctw-cushion-lab-grown-diamond-old-mine-cut-milgrain-split-floral-shank-side-stone-engagement-ring-platinum/pid/RIGRVR06510-PL2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr"/>
-      <c r="C61" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/1-7-8-ctw-oval-lab-grown-diamond-engagement-ring-with-floating-marquise-side-accents-14k-white-gold/pid/RIG2638X2O150SOGW2?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>1 7/8 ctw Oval Lab Grown Diamond Engagement Ring with Floating Marquise Side Accents</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR02638O200SOX3/medium/TXR02638O200SOX3-WG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR02638O200SOX3/medium/TXR02638O200SOX3-WG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG2638X3O250SO/medium/RIG2638X3O250SO-LW-new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR2638X20150S0GW4/medium/LGR2638X20150S0GW4-GW1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR2638X20150S0GW4/medium/LGR2638X20150S0GW4-GW2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-4-ctw-emerald-lab-grown-diamond-baguette-sides-engagement-ring-14k-white-gold/pid/RIGR617X3E20-GW3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr"/>
-      <c r="C62" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/5-3-4-ctw-pear-lab-grown-diamond-side-stone-engagement-ring-18k-yellow-gold/pid/RIGKSR6203-GY3?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>5 3/4 ctw Pear Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6203/medium/RIGKSR6203-YG-PE-WH-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6203/medium/RIGKSR6203-YG-PE-WH-500-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
+        </is>
+      </c>
       <c r="D62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-royal-crown-engagement-ring-14k-white-gold/pid/RIG0621X3-T200SO-GW?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr"/>
-      <c r="C63" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-2-3-ctw-oval-lab-grown-diamond-engagement-ring-with-pear-side-accents-14k-yellow-gold/pid/RIG0615X3-O200SO-GY?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2 2/3 ctw Oval Lab Grown Diamond Engagement Ring with Pear Side Accents</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00615O200SOX3/medium/TXR00615O200SOX3-YG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00615O200SOX3/medium/TXR00615O200SOX3-YG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0615X3/medium/RIG0615X3-O200SO-GW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-1-2-ctw-round-lab-grown-diamond-three-stone-engagement-ring-with-side-diamonds-platinum/pid/RIGAJ01024R300-PL2?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr"/>
-      <c r="C64" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-1-2-ctw-round-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD02180H-PL1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 5 1/2 ctw Round Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02180H%20/medium/RIGJRD02180H%20-WG-VR-WH-549-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02180H%20/medium/RIGJRD02180H%20-WG-VR-WH-549-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02180H/medium/RIGJRD02180H-HW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-1-2-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-platinum/pid/RIGTXR06690R300PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr"/>
-      <c r="C65" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/5-1-3-ctw-oval-lab-grown-diamond-double-heart-shape-prong-split-shank-side-stone-engagement-ring-platinum/pid/RIGRVR04394O500PL2?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>5 1/3 ctw Oval Lab Grown Diamond Double Heart Shape Prong Split Shank Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04394O500/medium/RIGRVR04394O500-WG-OV-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04394O500/medium/RIGRVR04394O500-WG-OV-500-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-5-8-ctw-round-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD0230XX-PL3?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-3-4-ctw-elongated-cushion-lab-grown-diamond-side-stone-engagement-ring-18k-white-gold/pid/RIGTXR07755Z400HW1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 4 3/4 ctw Elongated Cushion Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07755%20(EC%204.0%20SO)/medium/RIGTXR07755%20(EC%204.0%20SO)-WG-ECU-WH-475-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07755%20(EC%204.0%20SO)/medium/RIGTXR07755%20(EC%204.0%20SO)-WG-ECU-WH-475-M1.jpg</t>
+        </is>
+      </c>
       <c r="D66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-3-4-ctw-cushion-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD02104Q-PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-ctw-emerald-lab-grown-diamond-side-stone-engagement-ring-platinum/pid/RIGKSR6129-PL1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>3 3/4 ctw Cushion Lab Grown Diamond Engagement Ring</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr"/>
+          <t>Badgley Mischka Colorless 5 ctw Emerald Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6129/medium/RIGKSR6129-WG-EM-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6129/medium/RIGKSR6129-WG-EM-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-1-3-ctw-radiant-lab-grown-diamond-hidden-halo-bridal-set-platinum/pid/BRDTXR07490-PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr"/>
-      <c r="C68" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-5-8-ctw-oval-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/TXR04040-GY1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>4 5/8 ctw Oval Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04040/medium/RIGTXR04040-GY3_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04040/medium/RIGTXR04040-GY3_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04040/medium/RIGTXR04040-GW3-1-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-oval-lab-grown-diamond-three-stone-ring-18k-white-gold/pid/RIGJRD0242XX-PL18?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr"/>
-      <c r="C69" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/12x7mm-pear-cut-created-emerald-and-1-2-ctw-lab-grown-diamond-halo-engagement-ring-engagement-ring-14k-white-gold/pid/RIGTXR06627-EM-GW4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>12x7mm Pear Cut Created Emerald and 1/2 ctw Lab Grown Diamond Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06627/medium/RIGTXR06627-EM-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06627/medium/RIGTXR06627-EM-GW4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06627/medium/RIGTXR06627-EM-GW4-new.jpg</t>
+        </is>
+      </c>
       <c r="D69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-and-7-2-mm-round-shape-created-sapphire-three-stone-engagement-ring-platinum/pid/RIGR07347-RDSP-PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr"/>
-      <c r="C70" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-1-4-ctw-emerald-lab-grown-diamond-engagement-ring-with-tapered-baguette-side-accents-14k-white-gold/pid/RIG0617X3-E200SO-GW?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2 1/4 ctw Emerald Lab Grown Diamond Engagement Ring with Tapered Baguette Side Accents</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0617X3/medium/RIG0617X3-E200SO-GW-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0617X3/medium/RIG0617X3-E200SO-GW-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0617X3E200/medium/LGR0617X3E200-shape.jpg</t>
+        </is>
+      </c>
       <c r="D70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/16-0x11-25-mm-radiant-cut-created-ruby-and-6-ctw-trapezoid-lab-grown-diamond-engagement-ring-with-side-accents-platinum/pid/RIGTXR08893-RU-PL4?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr"/>
-      <c r="C71" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-3-4-ctw-oval-lab-grown-diamond-hidden-halo-bridal-set-platinum/pid/BRDTXR06232O200PL2?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2 3/4 ctw Oval Lab Grown Diamond Hidden Halo Bridal Set</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06232/medium/RIGTXR06232-WG-OV-WH-276-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06232/medium/RIGTXR06232-WG-OV-WH-276-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR06232O200GW1/medium/BRDTXR06232O200GW1-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-cushion-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD02094Q-HP1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr"/>
-      <c r="C72" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-ctw-radiant-lab-grown-diamond-solitaire-engagement-ring-platinum/pid/RIGJRO1322-PL_5?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>3 ctw Radiant Lab Grown Diamond Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRO1322/medium/RIGJRO1322-WG-RD1-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRO1322/medium/RIGJRO1322-WG-RD-WH-300-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
       <c r="D72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-7-8-ctw-cushion-lab-grown-diamond-fancy-yellow-halo-engagement-ring-14k-two-tone-white-and-yellow-gold/pid/RIGTXR05868-YL-GW4?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-1-3-ctw-princess-lab-grown-diamond-split-shank-engagement-ring-platinum/pid/LGR0625X3-P300SO-PL4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>3 1/3 ctw Princess Lab Grown Diamond Split Shank Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X3P300SO/medium/RIG0625X3P300SO-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X3P300SO/medium/RIG0625X3P300SO-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0589X3/medium/LGR0589X3-P300SO-FIN.jpg</t>
+        </is>
+      </c>
       <c r="D73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/9x7mm-created-emerald-and-2-3-8-pear-cut-lab-grown-diamond-two-stone-engagement-ring-platinum/pid/RIGTXR06625-EM-PL4?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr"/>
-      <c r="C74" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-7-8-ctw-cushion-lab-grown-diamond-graduated-halo-engagement-ring-14k-white-gold/pid/RIG0641X4C200H1GW2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2 7/8 ctw Cushion Lab Grown Diamond Graduated Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00641C200H1X5/medium/TXR00641C200H1X5-WG-CU-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00641C200H1X5/medium/TXR00641C200H1X5-WG-CU-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-3-8-ctw-radiant-lab-grown-diamond-side-stone-engagement-ring-14k-white-gold/pid/RIGTXR07701T300GW1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/11x9mm-created-emerald-and-1-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR06623-EM-GW4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>11x9mm Created Emerald and 1 ctw Lab Grown Diamond Three-Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06623/medium/RIGTXR06623-EM-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06623/medium/RIGTXR06623-EM-GW4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06623/medium/RIGTXR06623-EM-GW4-new.jpg</t>
+        </is>
+      </c>
       <c r="D75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-5-6-ctw-radiant-lab-grown-diamond-fancy-yellow-with-side-emerald-cuts-three-stone-engagement-ring-14k-two-tone-white-and-yellow-gold/pid/RIGTXR05886-YL-GW4?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr"/>
-      <c r="C76" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-bezel-set-solitaire-engagement-ring-platinum/pid/RIGTXR06655EM500PL3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>5 ctw Emerald Lab Grown Diamond Bezel Set Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06655/medium/RIGTXR06655-WG-EM-WH-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06655/medium/RIGTXR06655-WG-EM-WH-500-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-1-2-ctw-oval-lab-grown-diamond-double-scalloped-halo-engagement-ring-platinum/pid/RIGTXR06195O300PL2?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/2-2-3-ctw-multi-shape-lab-grown-diamond-vintage-inspired-art-deco-engagement-ring-platinum/pid/RIGRVR05013-PL4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>5 1/2 ctw Oval Lab Grown Diamond Double Scalloped Halo Engagement Ring</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr"/>
+          <t>2 2/3 ctw Multi-Shape Lab Grown Diamond Vintage Inspired Art Deco Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05013/medium/RIGRVR05013-WG-265N-VR-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05013/medium/RIGRVR05013-WG-265N-VR-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05013/medium/RIGRVR05013-GW1-NEW.jpg</t>
+        </is>
+      </c>
       <c r="D77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-emerald-lab-grown-diamond-wide-shank-solitaire-engagement-ring-14k-white-gold/pid/RIGTXR08593E300GW1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr"/>
-      <c r="C78" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/10x8-mm-created-emerald-and-1-3-8-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR06678-EM-GW4?algoliaQueryId=961725d3c54423b9205778064301ed8e&amp;amp;in_stock=yes</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>10x8 mm Created Emerald and 1 3/8 ctw Lab Grown Diamond Three-Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06678/medium/RIGTXR06678-EM-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06678/medium/RIGTXR06678-EM-GW4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06678/medium/RIGTXR06678-EM-GW4-1-NEW.jpg</t>
+        </is>
+      </c>
       <c r="D78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-1-8-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/RVR00048R300GY1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr"/>
-      <c r="C79" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-2-3-ctw-oval-lab-grown-diamond-three-stone-engagement-ring-with-half-moon-sides-platinum/pid/RIGTXR06001OV30PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>4 2/3 ctw Oval Lab Grown Diamond Three-Stone Engagement Ring with Half Moon sides</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06001/medium/RIGTXR06001-WG-OV-WH-441-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06001/medium/RIGTXR06001-WG-OV-WH-441-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-1-3-ctw-oval-lab-grown-diamond-split-shank-engagement-ring-18k-yellow-gold/pid/RIGJRF76530E-PL_5?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr"/>
-      <c r="C80" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-3-4-ctw-cushion-lab-grown-diamond-split-shank-x-side-stone-engagement-ring-14k-rose-gold/pid/RIGRV08957C400-GP2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>4 3/4 ctw Cushion Lab Grown Diamond Split Shank X  Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR08957C400/medium/RIGRVR08957C400-RG-CU-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR08957C400/medium/RIGRVR08957C400-RG-CU-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-princess-lab-grown-diamond-and-5-5x3-3x2-2-mm-trapezoid-created-sapphire-three-stone-ring-14k-yellow-gold/pid/RIGTXR07696SP-PR400-GY4?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr"/>
-      <c r="C81" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/6-1-4-ctw-oval-lab-grown-diamond-trapezoid-and-pear-side-stone-bridal-set-platinum/pid/BRDTXR08417O500PL4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>6 1/4 ctw Oval Lab Grown Diamond Trapezoid and Pear Side Stone Bridal Set</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08417O500/medium/BRDTXR08417O500-WG-OV-WH-625-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08417O500/medium/BRDTXR08417O500-WG-OV-WH-625-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-ctw-asscher-lab-grown-diamond-solitaire-engagement-ring-with-round-and-baguette-side-accents/pid/RIGTXR06225-HP1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr"/>
-      <c r="C82" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-ctw-toi-et-moi-pear-and-oval-engagement-ring-14k-white-gold/pid/RIGTXR05974PO30-GW4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>3 ctw Toi Et Moi Pear and Oval Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05974/medium/RIGTXR05974-WG-VR-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05974/medium/RIGTXR05974-WG-VR-WH-300-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGDTXR05974PO30GW%20/medium/LGDTXR05974PO30GW%20-%201.jpg</t>
+        </is>
+      </c>
       <c r="D82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-round-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ78340E-HP_5?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr"/>
-      <c r="C83" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-1-10-ctw-oval-lab-grown-diamond-pave-prong-solitaire-engagement-ring-with-hidden-accents-14k-yellow-gold/pid/RIGTXR05578O200GY2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2 1/10 ctw Oval Lab Grown Diamond Pave Prong Solitaire Engagement Ring with Hidden Accents</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05578/medium/RIGTXR05578-YG-OV-WH-212-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05578/medium/RIGTXR05578-YG-OV-WH-212-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-8-ctw-princess-lab-grown-diamond-double-twist-halo-engagement-ring-14k-white-gold/pid/RIG0629X2-P075H1-GW?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr"/>
-      <c r="C84" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-7-8-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-platinum/pid/RIGTXR09619R300PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>3 7/8 ctw Round Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR09619/medium/TXR09619-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR09619/medium/TXR09619-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09619R300GW4/medium/RIGTXR09619R300GW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-ctw-round-lab-grown-diamond-halo-engagement-ring-18k-white-gold/pid/RIGJRZ760310-HW_5?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr"/>
-      <c r="C85" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-cushion-lab-grown-diamond-v-prong-halo-engagement-ring-14k-white-gold/pid/RIG0639X4C200H1GW2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Cushion Lab Grown Diamond V-Prong Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00639C200H1X5/medium/TXR00639C200H1X5-WG-CU-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00639C200H1X5/medium/TXR00639C200H1X5-WG-CU-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-round-lab-grown-diamond-knife-edge-solitaire-engagement-ring-14k-white-gold/pid/RIGTX09876R400-GW2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr"/>
-      <c r="C86" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-ctw-emerald-lab-grown-diamond-solitaire-engagement-ring-platinum/pid/RIGTXR09875E400PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>4 ctw Emerald Lab Grown Diamond Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09875E400/medium/RIGTXR09875E400-WG-EM-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09875E400/medium/RIGTXR09875E400-WG-EM-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-1-8-ctw-round-lab-grown-diamond-micro-pave-bridal-set-platinum/pid/BRDTXR08071R300PL2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
+          <t>https://www.grownbrilliance.com/13-4mm-cushion-cut-created-emerald-and-2-ctw-pear-lab-grown-diamond-three-stone-engagement-ring-14k-yellow-gold/pid/RIGTXR08896-EM-GY4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>4 1/8 ctw Round Lab Grown Diamond Micro Pave Bridal Set</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr"/>
+          <t>13.4mm Cushion Cut Created Emerald and 2 ctw Pear Lab Grown Diamond Three Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08896/medium/RIGTXR08896-EM-GY4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08896/medium/RIGTXR08896-EM-GY4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08896/medium/RIGTXR08896-R0.jpg</t>
+        </is>
+      </c>
       <c r="D87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-1-2-ctw-princess-lab-grown-diamond-and-3-5mm-round-created-sapphire-side-stone-engagement-ring-14k-white-gold/pid/RIGTXR07695-GW1?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f&amp;amp;in_stock=yes</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr"/>
-      <c r="C88" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-twist-solitaire-engagement-ring-14k-white-gold/pid/RIGTXR05112-GW4-3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>3 ctw Round Lab Grown Diamond Twist Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05112/medium/RIGTXR05112-WG-RB-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05112/medium/RIGTXR05112-WG-RB-WH-300-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/10x8mm-radiant-cut-created-emerald-and-5-8-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR06621-EM-GW4?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-1-2-ctw-cushion-lab-grown-diamond-halo-engagement-ring-platinum/pid/RIGKSR6111N-PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 3 1/2 ctw Cushion Lab Grown Diamond Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6111/medium/RIGKSR6111-WG-CU-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6111/medium/RIGKSR6111-WG-CU-WH-300-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6184N/medium/RIGKSR6184N-HW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-cushion-lab-grown-diamond-old-mine-cut-split-shank-hidden-halo-engagement-ring-14k-white-gold/pid/RIGRVR06506-GW1?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr"/>
-      <c r="C90" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-1-4-ctw-oval-lab-grown-diamond-three-stone-bridal-set-platinum/pid/BRDTXR08075O300PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>4 1/4 ctw Oval Lab Grown Diamond Three-Stone Bridal Set</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08075O300/medium/BRDTXR08075O300-WG-OV-WH-426-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08075O300/medium/BRDTXR08075O300-WG-OV-WH-426-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-2-5-ctw-pear-lab-grown-diamond-ribbon-engagement-ring-14k-white-gold/pid/LGR1519X3D300SOGW2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr"/>
-      <c r="C91" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-1-3-ctw-princess-lab-grown-diamond-hidden-halo-engagement-ring-18k-white-gold/pid/RIGKSR6164-GW3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 4 1/3 ctw Princess Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6164/medium/RIGKSR6164-WG-PR-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6164/medium/RIGKSR6164-WG-PR-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
+        </is>
+      </c>
       <c r="D91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-3-4-ctw-oval-lab-grown-diamond-three-stone-halo-engagement-ring-14k-white-gold/pid/RIGRVR01595-GW2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
+          <t>https://www.grownbrilliance.com/5-1-5-ctw-cushion-lab-grown-diamond-old-mine-cut-milgrain-split-floral-shank-side-stone-engagement-ring-platinum/pid/RIGRVR06510-PL2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>3 3/4 ctw Oval Lab Grown Diamond Three Stone Halo Engagement Ring</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr"/>
+          <t>5 1/5 ctw Cushion Lab Grown Diamond Old Mine Cut Milgrain Split Floral Shank Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06510/medium/RIGRVR06510-WG-CU-491-M0_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06510/medium/RIGRVR06510-WG-CU-491-M1_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-3-4-ctw-cushion-lab-grown-diamond-ribbon-halo-engagement-ring-platinum/pid/RIG1519X4C200H1PL1?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr"/>
-      <c r="C93" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-1-4-ctw-emerald-lab-grown-diamond-baguette-sides-engagement-ring-14k-white-gold/pid/RIGR617X3E20-GW3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2 1/4 ctw Emerald Lab Grown Diamond Baguette Sides Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGR617X3E20/medium/RIGR617X3E20-WG-EM-WH-224-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGR617X3E20/medium/RIGR617X3E20-WG-EM-WH-224-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0617X3E200/medium/LGR0617X3E200-GW1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0617X3E200/medium/LGR0617X3E200-GW2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-7-8-ctw-oval-lab-grown-diamond-side-stone-solitaire-engagement-ring-platinum/pid/RIGTXR05540O3.0PL2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr"/>
-      <c r="C94" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-royal-crown-engagement-ring-14k-white-gold/pid/RIG0621X3-T200SO-GW?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Radiant Lab Grown Diamond Royal Crown Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00621T200SOX3/medium/TXR00621T200SOX3-WG-RD-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00621T200SOX3/medium/TXR00621T200SOX3-WG-RD-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
       <c r="D94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/6-3-4-ctw-fancy-yellow-radiant-lab-grown-diamond-with-trapezoid-three-stone-engagement-ring-14k-two-tone-white-yellow-gold/pid/RIGJOR6596-YL-GW4?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B95" t="inlineStr"/>
-      <c r="C95" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-1-2-ctw-round-lab-grown-diamond-three-stone-engagement-ring-with-side-diamonds-platinum/pid/RIGAJ01024R300-PL2?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>4 1/2 ctw Round Lab Grown Diamond Three Stone Engagement Ring with Side Diamonds</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01024R200/medium/RIGAJR01024R200-WG-RB-320-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01024R200/medium/RIGAJR01024R200-WG-RB-320-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-radiant-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/RVR00006T300GY2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B96" t="inlineStr"/>
-      <c r="C96" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-platinum/pid/RIGTXR06690R300PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Round Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG06690R300/medium/RIG06690R300-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG06690R300/medium/RIG06690R300-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-3-4-ctw-emerald-lab-grown-diamond-baguette-and-princess-side-stone-bridal-set-14k-white-gold/pid/BDTXR06230EM300GW2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B97" t="inlineStr"/>
-      <c r="C97" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-5-8-ctw-round-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD0230XX-PL3?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>4 5/8 ctw Round Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0230XX/medium/RIGJRD0230XX-WG-RB-WH-402-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0230XX/medium/RIGJRD0230XX-WG-RB-WH-402-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-ctw-emerald-lab-grown-diamond-celtic-knot-side-stone-engagement-ring-platinum/pid/RIGRVR00041E200PL1?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr"/>
-      <c r="C98" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-3-4-ctw-cushion-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD02104Q-PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>3 3/4 ctw Cushion Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02104Q/medium/RIGJRD02104Q-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02104Q/medium/RIGJRD02104Q-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02104Q/medium/RIGJRD02104Q-HW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-1-5-ctw-round-lab-grown-diamond-scalloped-classic-pave-solitaire-engagement-ring-with-side-stones-14k-white-gold/pid/RIGTXR05577R300GW2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B99" t="inlineStr"/>
-      <c r="C99" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-1-3-ctw-radiant-lab-grown-diamond-hidden-halo-bridal-set-platinum/pid/BRDTXR07490-PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>4 1/3 ctw Radiant Lab Grown Diamond Hidden Halo Bridal Set</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07490/medium/TXR07490-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07490/medium/TXR07490-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
       <c r="D99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-2-3-ctw-pear-lab-grown-diamond-french-pave-halo-engagement-ring-14k-white-gold/pid/RIGTXR06368D3.0GW2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
+          <t>https://www.grownbrilliance.com/5-ctw-oval-lab-grown-diamond-three-stone-ring-18k-white-gold/pid/RIGJRD0242XX-PL18?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>3 2/3 ctw Pear Lab Grown Diamond French Pave Halo Engagement Ring</t>
-        </is>
-      </c>
-      <c r="C100" t="inlineStr"/>
+          <t>5 ctw Oval Lab Grown Diamond Three-Stone Ring</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0242XX/medium/RIGJRD0242XX-WG-RB-WH-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0242XX/medium/RIGJRD0242XX-WG-RB-WH-500-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-1-5-ctw-emerald-lab-grown-diamond-side-stone-solitaire-engagement-ring-platinum/pid/RIGTXR05540E3.0PL2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
-        </is>
-      </c>
-      <c r="B101" t="inlineStr"/>
-      <c r="C101" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-and-7-2-mm-round-shape-created-sapphire-three-stone-engagement-ring-platinum/pid/RIGR07347-RDSP-PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>3 ctw Round Lab Grown Diamond and 7.2 mm Round Shape Created Sapphire Three-Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07347/medium/RIGTXR07347-RB-WG-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07347/medium/RIGTXR07347-RB-WG-WH-300-M1.jpg</t>
+        </is>
+      </c>
       <c r="D101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-1-3-ctw-radiant-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR07056-GW2?algoliaQueryId=37cb4077035a9f0479e20c829f2c2f8f</t>
+          <t>https://www.grownbrilliance.com/16-0x11-25-mm-radiant-cut-created-ruby-and-6-ctw-trapezoid-lab-grown-diamond-engagement-ring-with-side-accents-platinum/pid/RIGTXR08893-RU-PL4?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>4 1/3 ctw Radiant Lab Grown Diamond Bridal Set</t>
-        </is>
-      </c>
-      <c r="C102" t="inlineStr"/>
+          <t>16.0x11.25 mm Radiant Cut Created Ruby and 6 ctw Trapezoid Lab Grown Diamond Engagement Ring with Side Accents</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08893/medium/RIGTXR08893-RU-WG-RD-WH-598-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08893/medium/RIGTXR08893-RU-WG-RD-WH-598-M1.jpg</t>
+        </is>
+      </c>
       <c r="D102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-ctw-cushion-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD02094Q-HP1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>4 ctw Cushion Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02094Q/medium/RIGJRD02094Q-RG-RB-WH-396-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02094Q/medium/RIGJRD02094Q-RG-RB-WH-396-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update code for server migration
</commit_message>
<xml_diff>
--- a/py_scraper/product_data.xlsx
+++ b/py_scraper/product_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D103"/>
+  <dimension ref="A1:D233"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,331 +453,575 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-1-5-ctw-emerald-lab-grown-diamond-side-stone-solitaire-engagement-ring-platinum/pid/RIGTXR05540E3.0PL2?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>4 1/5 ctw Emerald Lab Grown Diamond Side Stone Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05540/medium/RIGTXR05540-WG-EM-WH-420-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05540/medium/RIGTXR05540-WG-EM-WH-420-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-1-3-ctw-radiant-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR07056-GW2?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>4 1/3 ctw Radiant Lab Grown Diamond Bridal Set</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07056/medium/BRDTXR07056-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07056/medium/BRDTXR07056-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-3-8-ctw-oval-lab-grown-diamond-double-hidden-halo-engagement-ring-platinum/pid/RIGTXR05543O300PL2?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3 3/8 ctw Oval Lab Grown Diamond Double Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05543/medium/RIGTXR05543-WG-OV-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05543/medium/RIGTXR05543-WG-OV-WH-300-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-7-8-ctw-round-lab-grown-diamond-french-pave-engagement-ring-platinum/pid/RIGT05118-PL4-R350?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3 7/8 ctw Round Lab Grown Diamond French Pave Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR05118R350/medium/TXR05118R350-WG-RB-WH-393-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR05118R350/medium/TXR05118R350-WG-RB-WH-393-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-engagement-ring-with-double-baguette-side-accents-platinum/pid/RIG0890X3T200SOPL1?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1 1/5 ctw Princess Lab Grown Diamond Split Shank Halo Engagement Ring</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>2 1/2 ctw Radiant Lab Grown Diamond Engagement Ring with Double Baguette Side Accents</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00890T200SOX3/medium/TXR00890T200SOX3-WG-RD-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00890T200SOX3/medium/TXR00890T200SOX3-WG-RD-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/4-ctw-cushion-lab-grown-diamond-double-prong-hidden-halo-engagement-ring-14k-two-tone-yellow-and-white-gold/pid/RIGRV04393C400GYW4?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>4 ctw Cushion Lab Grown Diamond Two Tone Double Prong Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04393C400/medium/RIGRVR04393C400-YW-CU-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04393C400/medium/RIGRVR04393C400-YW-CU-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-4-1-4-ctw-emerald-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ757240-PL12?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Near-Colorless 4 1/4 ctw Emerald Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ757240/medium/RIGJRZ757240-WG-RB-WH-429-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ757240/medium/RIGJRZ757240-WG-RB-WH-429-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ757240/medium/RIGJRZ757240-HW12-new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-fancy-blue-round-lab-grown-diamond-split-shank-side-stone-engagement-ring-14k-white-gold/pid/RIGTXR09163-BL-GW4?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Fancy Blue Round Lab Grown Diamond Split Shank Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09163B/medium/RIGTXR09163B-WG-EM-WH-350-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09163B/medium/RIGTXR09163B-WG-EM-WH-350-M1.jpg</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-7-8-ctw-oval-lab-grown-diamond-flower-petal-halo-engagement-ring-14k-yellow-gold/pid/RIG1613X4O200H1GY1?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2 7/8 ctw Oval Lab Grown Diamond Flower Petal Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR01613O200H1X5/medium/TXR01613O200H1X5-YG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR01613O200H1X5/medium/TXR01613O200H1X5-YG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-6-7-8-ctw-emerald-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ7731XX-PL4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-1-3-ctw-cushion-lab-grown-diamond-draping-hidden-halo-engagement-ring-platinum/pid/RIGTXR05668C300PL2?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>3 1/3 ctw Cushion Lab Grown Diamond Draping Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05668/medium/RIGTXR05668-WG-CU-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05668/medium/RIGTXR05668-WG-CU-WH-300-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-3-1-2-ctw-round-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ78940H-HW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-3-8-ctw-round-lab-grown-diamond-vine-engagement-ring-platinum/pid/RIG0887X3R200SOPL1?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2 3/8 ctw Round Lab Grown Diamond Vine Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00887R200SOX3/medium/TXR00887R200SOX3-WG-RB-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00887R200SOX3/medium/TXR00887R200SOX3-WG-RB-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-3-4-ctw-oval-lab-grown-diamond-engagement-ring-with-channel-set-side-accents-14k-white-gold/pid/RIG0635X3O250SOGW2?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2 3/4 ctw Oval Lab Grown Diamond Engagement Ring with Channel Set Side Accents</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00635O200SOX3/medium/TXR00635O200SOX3-WG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00635O200SOX3/medium/TXR00635O200SOX3-WG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-1-4-ctw-fancy-pink-pear-lab-grown-diamond-side-stone-engagement-ring-14k-rose-gold/pid/RIGTXR09152-PN-GP4?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>3 1/4 ctw Fancy Pink Pear Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09152P/medium/RIGTXR09152P-RG-PE-WH-328-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09152P/medium/RIGTXR09152P-RG-PE-WH-328-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09152/medium/RIGTXR09152-BL.jpg</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/1-1-2-ctw-princess-lab-grown-diamond-floral-solitaire-engagement-ring-14k-white-gold/pid/RIGTXR01782-GW2?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1 1/2 ctw Princess Lab Grown Diamond Floral Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR01782/medium/RIGTXR01782-WG-PR-WH-150-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR01782/medium/RIGTXR01782-WG-PR-WH-150-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-old-mine-cut-filigree-side-stone-engagement-ring-14k-yellow-gold/pid/RIGRVR06504-GY1?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2 ctw Round Lab Grown Diamond Old Mine Cut Filigree Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06504/medium/RIGRVR06504-YG-RB-219-M0_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06504/medium/RIGRVR06504-YG-RB-219-M1_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-round-lab-grown-diamond-side-stone-engagement-ring-14k-yellow-gold/pid/RIGAJR00806R300GY2?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Round Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR00806R300/medium/RIGAJR00806R300-YG-RB-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR00806R300/medium/RIGAJR00806R300-YG-RB-300-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr"/>
-      <c r="C18" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-1-4-ctw-oval-lab-grown-diamond-engagement-ring-18k-yellow-gold/pid/RIGJRZ76090Q-PL_5?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 3 1/4 ctw Oval Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76090Q/medium/RIGJRZ76090Q-WG-RB-WH-327-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76090Q/medium/RIGJRZ76090Q-WG-RB-WH-327-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
       <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr"/>
-      <c r="C19" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-5-8-ctw-cushion-lab-grown-diamond-crossover-halo-engagement-ring-14k-white-gold/pid/RIG0631X4C200H1GW1?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2 5/8 ctw Cushion Lab Grown Diamond Crossover Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00631C200H1X5/medium/TXR00631C200H1X5-WG-CU-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00631C200H1X5/medium/TXR00631C200H1X5-WG-CU-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-round-lab-grown-diamond-double-band-bridal-set-14k-white-gold/pid/RIGTXR06256RD300-GW4?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Round Lab Grown Diamond Double Band Bridal Set</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06256/medium/RIGTXR06256-WG-RB-WH-348-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06256/medium/RIGTXR06256-WG-RB-WH-348-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-2-7-8-ctw-emerald-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD02160T-HP_5?algoliaQueryId=7ad33818ec54fe63cf8e5383904b9671</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 2 7/8 ctw Emerald Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02160T/medium/RIGJRD02160T-RG-RB-WH-285-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02160T/medium/RIGJRD02160T-RG-RB-WH-285-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-ctw-emerald-lab-grown-diamond-crossover-solitaire-engagement-ring-14k-white-gold/pid/RIGTXR05124-GW4-EM3?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>3 ctw Emerald Lab Grown Diamond Crossover Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05124/medium/RIGTXR05124-WG-EM-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05124/medium/RIGTXR05124-WG-EM-WH-300-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
-      <c r="C23" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-1-8-ctw-round-lab-grown-diamond-three-stone-bridal-set-14k-yellow-gold/pid/BRDTXR08074R200GY2?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>3 1/8 ctw Round Lab Grown Diamond Three-Stone Bridal Set</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08074R200/medium/BRDTXR08074R200-YG-RB-WH-315-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08074R200/medium/BRDTXR08074R200-YG-RB-WH-315-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
-      <c r="C24" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/1-1-8-ctw-pear-lab-grown-diamond-marquise-vine-engagement-ring-14k-white-gold/pid/RIG0587X1-D075SO-GW?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>1 1/8 ctw Pear Lab Grown Diamond Marquise Vine Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00587D200SOX3/medium/TXR00587D200SOX3-WG-PE-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00587D200SOX3/medium/TXR00587D200SOX3-WG-PE-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
+        </is>
+      </c>
       <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-ctw-oval-lab-grown-diamond-and-6-0x3-8-mm-pear-shape-created-sapphire-side-stone-engagement-ring-14k-white-gold/pid/RIGTXR07342-OVSP-GW4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>3 ctw Oval Lab Grown Diamond and 6.0x3.8 mm Pear Shape Created Sapphire Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07342/medium/RIGTXR07342-OV-WG-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07342/medium/RIGTXR07342-OV-WG-WH-300-M1.jpg</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
-      <c r="C26" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-2-5-ctw-elongated-cushion-lab-grown-diamond-side-stone-engagement-ring-14k-white-gold/pid/RIGTXR08658Z300GW4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>3 2/5 ctw Elongated Cushion Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08658Z300/medium/RIGTXR08658Z300-WG-CU-WH-339-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08658Z300/medium/RIGTXR08658Z300-WG-CU-WH-339-M1.jpg</t>
+        </is>
+      </c>
       <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/1-1-2-ctw-round-lab-grown-diamond-cathedral-six-prong-solitaire-engagement-ring-platinum/pid/RIGTXR01745-PL4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>1 1/2 ctw Round Lab Grown Diamond Cathedral Six-Prong Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR01745/medium/RIGTXR01745-WG-RB-WH-150-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR01745/medium/RIGTXR01745-WG-RB-WH-150-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
-      <c r="C28" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-1-8-ctw-princess-lab-grown-diamond-arch-engagement-ring-platinum/pid/RIG0647X3P200SOPL2?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2 1/8 ctw Princess Lab Grown Diamond Arch Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00647P200SOX3/medium/TXR00647P200SOX3-WG-PR-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00647P200SOX3/medium/TXR00647P200SOX3-WG-PR-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
+        </is>
+      </c>
       <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
-      <c r="C29" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/1-1-2-ctw-pear-lab-grown-diamond-fancy-pink-with-prong-set-frame-halo-engagement-ring/pid/RIGTXR05878-PN-GR4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>1 1/2 ctw Pear Lab Grown Diamond Fancy Pink With Prong Set Frame Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05878/medium/RIGTXR05878-RG-PE-PN-141-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05878/medium/RIGTXR05878-RG-PE-PN-141-M1.jpg</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
-      <c r="C30" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/3-1-4-ctw-multi-shape-lab-grown-diamond-scatter-fancy-side-stone-engagement-ring-platinum/pid/RIGAJ00807R200-PL4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>3 1/4 ctw Multi-Shape Lab Grown Diamond Scatter Fancy Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJ00807R200/medium/RIGAJ00807R200-GW4-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJ00807R200/medium/RIGAJ00807R200-GW4-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
       <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
-      <c r="C31" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/9mm-cushion-cut-created-sapphire-and-5-8-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR06624-SP-GW4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>9mm Cushion Cut Created Sapphire and 5/8 ctw Lab Grown Diamond Three-Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06624/medium/RIGTXR06624-SP-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06624/medium/RIGTXR06624-SP-GW4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06624/medium/RIGTXR06624-SP-GW4-new.jpg</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
-      <c r="C32" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-2-3-ctw-emerald-lab-grown-diamond-double-shank-halo-engagement-ring-platinum/pid/RIGYR4354LEC-PL2?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2 2/3 ctw Emerald Lab Grown Diamond Double Shank Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR4354LEC/medium/RIGYR4354LEC-WG-EM-WH-267-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR4354LEC/medium/RIGYR4354LEC-WG-EM-WH-267-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/4-ctw-pear-lab-grown-diamond-split-prong-engagement-ring-with-large-halo-14k-white-gold/pid/RIGYR3743NE-GW4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1 1/5 ctw Princess Lab Grown Diamond Split Shank Halo Engagement Ring</t>
+          <t>4 ctw Pear Lab Grown Diamond Split Prong Engagement Ring With Large Halo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X2/medium/RIG0625X2-P075H1-GW_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X2/medium/RIG0625X2-P075H1-GW_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X2/medium/RIG0625X2-P075H1-GW_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X4/medium/RIG0625X4-P150H1-GW-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR3743NE/medium/RIGYR3743NE-WG-PE-WH-413-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR3743NE/medium/RIGYR3743NE-WG-PE-WH-413-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
@@ -785,57 +1029,89 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr"/>
-      <c r="C34" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-1-5-ctw-emerald-lab-grown-diamond-engagement-ring-with-marquise-shape-side-accents-platinum/pid/RIG0586X3E200SOPL1?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2 1/5 ctw Emerald Lab Grown Diamond Engagement Ring with Marquise Shape Side Accents</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00586E200SOX3/medium/TXR00586E200SOX3-WG-EM-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00586E200SOX3/medium/TXR00586E200SOX3-WG-EM-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr"/>
-      <c r="C35" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/2-ctw-radiant-lab-grown-diamond-bezel-set-wide-band-solitaire-engagement-ring-platinum/pid/RIGRVR02049-PL2?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2 ctw Radiant Lab Grown Diamond Bezel Set Wide Band Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02049/medium/RIGRVR02049-WG-RD-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02049/medium/RIGRVR02049-WG-RD-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
       <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr"/>
-      <c r="C36" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/1-1-2-ctw-radiant-lab-grown-diamond-fancy-yellow-floating-diamond-halo-engagement-ring-14k-two-tone-white-and-yellow-gold/pid/RIGTXR05882-YL-GW4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>1 1/2 ctw Radiant Lab Grown Diamond Fancy Yellow Floating Diamond Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05882/medium/RIGTXR05882-WG-RD-YL-147-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05882/medium/RIGTXR05882-WG-RD-YL-147-M1r.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGD/medium/LGD-TXR05882-YG-WG%20(2).jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGD/medium/LGD-TXR05882-YG-WG.jpg</t>
+        </is>
+      </c>
       <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
+          <t>https://www.grownbrilliance.com/9x7-mm-radiant-cut-created-sapphire-and-3-4-ctw-round-and-trapezoid-lab-grown-diamond-side-stone-engagement-ring-14k-white-gold/pid/RIGTXR06124-SP-GW4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>9X7 mm Radiant Cut Created Sapphire and 3/4 ctw Round and Trapezoid Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06124/medium/RIGTXR06124-WG-SP-RD-080-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06124/medium/RIGTXR06124-WG-SP-RD-080-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06124/medium/RIGTXR06124-R0.jpg</t>
+        </is>
+      </c>
       <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-ctw-cushion-lab-grown-diamond-woven-bridal-set-14k-white-gold/pid/BRDR06758CU1.5-GW1?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>1 ctw Round Lab Grown Diamond Double Twist Engagement Ring</t>
+          <t>2 ctw Cushion Lab Grown Diamond Woven Bridal Set</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0629X1/medium/RIG0629X1-R075SO-GW-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0629X1/medium/RIG0629X1-R075SO-GW-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0629X1R075SOGW4/medium/LGR0629X1R075SOGW4-new2-img.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/0629/medium/0629-Round-GB.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06758/medium/RIGTXR06758-WG-CU-WH-202-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06758/medium/RIGTXR06758-WG-CU-WH-202-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGDTXR06758C1.5GW4%20/medium/LGDTXR06758C1.5GW4%20-%201.jpg</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -843,17 +1119,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-1-4-ctw-oval-lab-grown-diamond-floating-marquise-halo-engagement-ring-platinum/pid/RIG2638X4O150H1PL2?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2 1/2 ctw Radiant Lab Grown Diamond Station Engagement Ring</t>
+          <t>2 1/4 ctw Oval Lab Grown Diamond Floating Marquise Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X3/medium/RIG1860X3-T200SO-GW-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X3/medium/RIG1860X3-T200SO-GW-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X1/medium/RIG1860X1-T075SO-GW-1-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X3/medium/RIG1860X3-Radiant-GW.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR02638O200H1X5/medium/TXR02638O200H1X5-WG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR02638O200H1X5/medium/TXR02638O200H1X5-WG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -861,17 +1137,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-2-5-ctw-fancy-blue-round-lab-grown-diamond-side-stone-engagement-ring-14k-white-gold/pid/RIGTXR09159-BL-GW4?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>5 ctw Emerald Lab Grown Diamond Engagement Ring</t>
+          <t>2 2/5 ctw Fancy Blue Round Lab Grown Diamond Side Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD020837/medium/RIGJRD020837-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD020837/medium/RIGJRD020837-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD020837/medium/RIGJRD020837-PL_5-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09159B/medium/RIGTXR09159B-WG-RB-WH-243-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09159B/medium/RIGTXR09159B-WG-RB-WH-243-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09159/medium/RIGTXR09159-PN-YL-BL.jpg</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -879,17 +1155,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-knot-halo-engagement-ring-14k-white-gold/pid/RIG0892X4-R200H1-GW?algoliaQueryId=30f3c9cea3149c7d240053d0bc60121b</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>2 ctw Round Lab Grown Diamond Graduated Engagement Ring</t>
+          <t>3 ctw Round Lab Grown Diamond Knot Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0641X2/medium/RIG0641X2-R150SO-GW_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0641X2/medium/RIG0641X2-R150SO-GW_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0641X2/medium/RIG0641X2-R150SO-GW-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0589X3/medium/LGR0589X3-R200-shape.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00892R200H1X5/medium/TXR00892R200H1X5-WG-RB-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00892R200H1X5/medium/TXR00892R200H1X5-WG-RB-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
@@ -897,17 +1173,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-6-7-8-ctw-emerald-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ7731XX-PL4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-1-3-ctw-pear-lab-grown-diamond-chevron-engagement-ring-with-side-accents-14k-white-gold/pid/RIGTXR06070233DGW2?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Badgley Mischka Near-Colorless 6 7/8 ctw Emerald Lab Grown Diamond Engagement Ring</t>
+          <t>2 1/3 ctw Pear Lab Grown Diamond Chevron Engagement Ring with Side Accents</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7731XX/medium/RIGJRZ7731XX-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7731XX/medium/RIGJRZ7731XX-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7731XX/medium/RIGJRZ7731XX-HW_5-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06070/medium/RIGTXR06070-WG-PE-WH-233-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06070/medium/RIGTXR06070-WG-PE-WH-233-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -915,17 +1191,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-3-1-2-ctw-round-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ78940H-HW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/11x9-mm-oval-cut-created-ruby-and-7-8-ctw-lab-grown-diamond-halo-engagement-ring-14k-white-gold/pid/RIGTXR06679-RU-GW4?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Badgley Mischka Near-Colorless 3 1/2 ctw Round Lab Grown Diamond Engagement Ring</t>
+          <t>11x9 mm Oval Cut Created Ruby and 7/8 ctw Lab Grown Diamond Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ78940H/medium/RIGJRZ78940H-HW_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ78940H/medium/RIGJRZ78940H-HW_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ78940H/medium/RIGJRZ78940H-HW_5-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06679/medium/RIGTXR06679-WG-OV-RU-086-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06679/medium/RIGTXR06679-WG-OV-RU-086-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06679/medium/RIGTXR06679-RU-GW4-new.jpg</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -933,17 +1209,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/8-1-4-ctw-radiant-lab-grown-diamond-bridal-set-platinum/pid/BRDTXR08803T500PL2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-1-4-ctw-emerald-lab-grown-diamond-double-halo-with-split-shank-halo-engagement-ring-14k-white-gold/pid/RIGTXR06196E150-GW3?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>8 1/4 ctw Radiant Lab Grown Diamond Bridal Set</t>
+          <t>2 1/4 ctw Emerald Lab Grown Diamond Double halo with Split Shank Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08803T500/medium/BRDTXR08803T500-WG-RD-WH-816-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08803T500/medium/BRDTXR08803T500-WG-RD-WH-816-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06196/medium/RIGTXR06196-WG-EM-229-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06196/medium/RIGTXR06196-WG-EM-229-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -951,17 +1227,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-2-5-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-18k-white-gold/pid/RIGTX06766R500-HW1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-oval-lab-grown-diamond-channel-set-halo-engagement-ring-platinum/pid/RIG0635X4-O200H1-LW?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Badgley Mischka Colorless 5 2/5 ctw Round Lab Grown Diamond Hidden Halo Engagement Ring</t>
+          <t>2 1/2 ctw Oval Lab Grown Diamond Channel Set Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06766R500/medium/RIGTXR06766R500-WG-RB-WH-543-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06766R500/medium/RIGTXR06766R500-WG-RB-WH-543-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTX06766R500/medium/RIGTX06766R500-GW6-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00635O200H1X5/medium/TXR00635O200H1X5-WG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00635O200H1X5/medium/TXR00635O200H1X5-WG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -969,17 +1245,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-round-lab-grown-diamond-three-stone-ring-18k-white-gold/pid/RIGJRD0315-HW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b&amp;amp;in_stock=yes</t>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-round-lab-grown-diamond-split-shank-double-square-halo-engagement-ring-14k-yellow-gold/pid/RIGTXR06197-GY4?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>4 ctw Round Lab Grown Diamond Three-Stone Ring</t>
+          <t>3 1/2 ctw Round Lab Grown Diamond Split Shank Double Square Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0315/medium/RIGJRD0315-HW4_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0315/medium/RIGJRD0315-HW4_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0315/medium/RIGJRD0315-HW4-new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06197/medium/RIGTXR06197-YG-RB-WH-350-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06197/medium/RIGTXR06197-YG-RB-WH-350-M1.jpg</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
@@ -987,17 +1263,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-oval-lab-grown-diamond-petite-solitaire-engagement-ring-14k-white-gold/pid/RGTXR05314O300-GW2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/3-1-4-ctw-oval-lab-grown-diamond-split-prong-halo-engagement-ring-14k-white-gold/pid/RIG0589X4-O200H1-GW?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>3 ctw Oval Lab Grown Diamond Petite Solitaire Engagement Ring</t>
+          <t>3 1/4 ctw Oval Lab Grown Diamond Split Prong Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05314/medium/RIGTXR05314-WG-OV-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05314O300/medium/RIGTXR05314O300-GY4-1-NEW.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00589O200H1X5/medium/TXR00589O200H1X5-WG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00589O200H1X5/medium/TXR00589O200H1X5-WG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1005,17 +1281,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-2-5-ctw-oval-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR07400O300GW4?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b&amp;amp;in_stock=yes</t>
+          <t>https://www.grownbrilliance.com/3-ctw-oval-lab-grown-diamond-channel-band-halo-bridal-set-14k-yellow-gold/pid/BRDTXR06231OV200-GY4?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>4 2/5 ctw Oval Lab Grown Diamond Bridal Set</t>
+          <t>3 ctw Oval Lab Grown Diamond Channel Band Halo Bridal Set</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07400O300/medium/BRDTXR07400O300-WG-OV-WH-439-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07400O300/medium/BRDTXR07400O300-WG-OV-WH-439-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07400O300GW4/medium/BRDTXR07400O300GW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06231/medium/RIGTXR06231-YG-OV-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06231/medium/RIGTXR06231-YG-OV-WH-300-M1.jpg</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1023,17 +1299,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/6-2-3-ctw-round-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR08527-GW2?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-ctw-oval-lab-grown-diamond-double-shank-trellis-solitaire-engagement-ring-14k-yellow-gold/pid/RIGYR3528KE-GY1?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>6 2/3 ctw Round Lab Grown Diamond Bridal Set</t>
+          <t>2 ctw Oval Lab Grown Diamond Double Shank Trellis Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08527/medium/BRDTXR08527-WG-RB-WH-665-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08527/medium/BRDTXR08527-WG-RB-WH-665-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR3528KE/medium/RIGYR3528KE-YG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR3528KE/medium/RIGYR3528KE-YG-OV-WH-200-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
@@ -1041,17 +1317,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/8-2-3-ctw-pear-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/RIGTX04156D800-GY1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-cathedral-solitaire-engagement-ring-platinum/pid/RIGTXR01870-PL1?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>8 2/3 ctw Pear Lab Grown Diamond Hidden Halo Engagement Ring</t>
+          <t>2 ctw Round Lab Grown Diamond Cathedral Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04156D300/medium/RIGTXR04156D300-YG-PE-WH-352-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04156D300/medium/RIGTXR04156D300-YG-PE-WH-352-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR01870/medium/RIGTXR01870-WG-RB-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR01870/medium/RIGTXR01870-WG-RB-WH-200-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1059,17 +1335,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-1-2-ctw-emerald-lab-grown-diamond-three-stone-ring-platinum/pid/RIGJRD0254XX-PL_5?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-ctw-emerald-lab-grown-diamond-6mm-bold-solitaire-engagement-ring-14k-yellow-gold/pid/RIGRVR02051-GY1?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>5 1/2  ctw Emerald Lab Grown Diamond Three-Stone Ring</t>
+          <t>2 ctw Emerald Lab Grown Diamond 6mm Bold Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0254XX/medium/RIGJRD0254XX-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0254XX/medium/RIGJRD0254XX-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0254/medium/RIGJRD0254-HW_5-new-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02051/medium/RIGRVR02051-YG-EM-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02051/medium/RIGRVR02051-YG-EM-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
@@ -1077,17 +1353,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-toi-et-moi-pear-and-emerald-engagement-ring-14k-yellow-gold/pid/RIGTXR05973PE40GY1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b&amp;amp;in_stock=yes</t>
+          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-old-mine-cut-halo-engagement-ring-in-milgrain-setting-14k-white-gold/pid/RIGRVR06503-GW4?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>4 ctw Toi Et Moi Pear and Emerald Engagement Ring</t>
+          <t>3 ctw Round Lab Grown Diamond Old Mine Cut Halo Engagement Ring in Milgrain Setting</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05973/medium/RIGTXR05973-YG-VR-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05973/medium/RIGTXR05973-YG-VR-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05973PE40/medium/RIGTXR05973PE40-GW4-new.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06503/medium/RIGRVR06503-WG-RB-300N-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06503/medium/RIGRVR06503-WG-RB-300N-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06503/medium/RIGRVR06503-GW4.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
@@ -1095,17 +1371,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/9-ctw-pear-lab-grown-diamond-engagement-ring-with-split-prong-side-accents-platinum/pid/RIGRV04550D800-PL1?algoliaQueryId=d55a5e87736cbe21a3157b130ffb2d8b</t>
+          <t>https://www.grownbrilliance.com/2-5-8-ctw-oval-lab-grown-diamond-double-row-halo-engagement-ring-14k-rose-gold/pid/RIG0623X4-O200H1-GS?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>9 ctw Pear Lab Grown Diamond Engagement Ring with Split Prong Side Accents</t>
+          <t>2 5/8 ctw Oval Lab Grown Diamond Double Row Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04550D800/medium/RIGRVR04550D800-WG-PE-WH-900-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04550D800/medium/RIGRVR04550D800-WG-PE-WH-900-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00623O200H1X5/medium/TXR00623O200H1X5-RG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00623O200H1X5/medium/TXR00623O200H1X5-RG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
@@ -1113,17 +1389,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-3-4-ctw-fancy-pink-cushion-lab-grown-diamond-three-stone-engagement-ring-platinum/pid/RIGTXR09165-PN-PL4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-5-8-ctw-emerald-lab-grown-diamond-bezel-set-with-trillion-three-stone-engagement-ring-14k-yellow-gold/pid/RIGRVR02050-GY4?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>3 3/4 ctw Fancy Pink Cushion Lab Grown Diamond Three Stone Engagement Ring</t>
+          <t>2 5/8 ctw Emerald Lab Grown Diamond Bezel Set With Trillion Three Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09165P/medium/RIGTXR09165P-WG-CU-WH-375-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09165P/medium/RIGTXR09165P-WG-CU-WH-375-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09165/medium/RIGTXR09165-YL-BL-PN%20alt%20image.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02050/medium/RIGRVR02050-YG-EM-WH-260-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02050/medium/RIGRVR02050-YG-EM-WH-260-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
@@ -1131,17 +1407,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-5-1-2-ctw-round-lab-grown-diamond-bypass-engagement-ring-platinum/pid/RIGJRZ758806R5-PL1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-1-3-ctw-princess-lab-grown-diamond-crossover-micro-pave-engagement-ringplatinum/pid/RIGTXR05130-PL4-PR2?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Badgley Mischka Colorless 5 1/2 ctw Round Lab Grown Diamond Bypass Engagement Ring</t>
+          <t>2 1/3 ctw Princess Lab Grown Diamond Crossover Micro Pave Engagement Ring</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ758806/medium/RIGJRZ758806-WG-RB-WH-556-M0-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ758806/medium/RIGJRZ758806-WG-RB-WH-556-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ758806R7/medium/RIGJRZ758806R7-HW6-new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05130/medium/RIGTXR05130-WG-PR-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05130/medium/RIGTXR05130-WG-PR-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
         </is>
       </c>
       <c r="D55" t="inlineStr"/>
@@ -1149,17 +1425,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-trellis-solitaire-engagement-ring-14k-white-gold/pid/RIG-JOR037-GW1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-ctw-marquise-lab-grown-diamond-petite-bow-engagement-ring-14k-yellow-gold/pid/RIG0891X2M150SOGY1?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>2 ctw Round Lab Grown Diamond Trellis Solitaire Engagement Ring</t>
+          <t>2 ctw Marquise Lab Grown Diamond Petite Bow Engagement Ring</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJOR037/medium/RIGJOR037-WG-RB-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJOR037/medium/RIGJOR037-WG-RB-WH-200-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJOR037/medium/RIGJOR037-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00891M200SOX3/medium/TXR00891M200SOX3-YG-MQ-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00891M200SOX3/medium/TXR00891M200SOX3-YG-MQ-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-MQ.jpg</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1167,17 +1443,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-3-8-ctw-cushion-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRD0257XX-HW1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-1-8-ctw-pear-lab-grown-diamond-intertwined-engagement-ring-platinum/pid/RIG0627X3D200SOPL2?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Badgley Mischka Colorless 5 3/8 ctw Cushion Lab Grown Diamond Engagement Ring</t>
+          <t>2 1/8 ctw Pear Lab Grown Diamond Intertwined Engagement Ring</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0257XX/medium/RIGJRD0257XX-HW_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0257XX/medium/RIGJRD0257XX-HW_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0257XX/medium/RIGJRD0257XX-HW_5-new-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00627D200SOX3/medium/TXR00627D200SOX3-WG-PE-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00627D200SOX3/medium/TXR00627D200SOX3-WG-PE-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
@@ -1185,17 +1461,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-1-2-ctw-oval-lab-grown-diamond-braided-halo-engagement-ring-with-micro-pave-shank-platinum/pid/RIGTXR06229-OV3-PL3?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-3-4-ctw-oval-lab-grown-diamond-floral-halo-engagement-ring-14k-white-gold/pid/RIGYR3670LE-GW4?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Badgley Mischka Colorless 3 1/2 ctw Oval Lab Grown Diamond Braided Halo Engagement Ring with Micro Pave Shank</t>
+          <t>2 3/4 ctw Oval Lab Grown Diamond Floral Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06229/medium/RIGTXR06229-WG-OV-WH-350-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06229/medium/RIGTXR06229-WG-OV-WH-350-M1.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR3670LE/medium/RIGYR3670LE-WG-OV-WH-280-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR3670LE/medium/RIGYR3670LE-WG-OV-WH-280-M1.jpg</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1203,17 +1479,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/7-1-3-ctw-cushion-lab-grown-diamond-eternity-engagement-ring-platinum/pid/RIG08073C50PL2-700?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-3-4-ctw-emerald-lab-grown-diamond-royal-crown-halo-engagement-ring-14k-white-gold/pid/RIG0621X4-E200H1-GW?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>7 1/3 ctw Cushion Lab Grown Diamond Eternity Engagement Ring</t>
+          <t>2 3/4 ctw Emerald Lab Grown Diamond Royal Crown Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08073C500/medium/RIGTXR08073C500-WG-CU-WH-740-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08073C500/medium/RIGTXR08073C500-WG-CU-WH-740-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00621E200H1X5/medium/TXR00621E200H1X5-WG-EM-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00621E200H1X5/medium/TXR00621E200H1X5-WG-EM-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1221,17 +1497,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-4-1-3-ctw-cushion-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ7836XX-C-HW4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-ctw-oval-lab-grown-diamond-and-7-2x5-1-mm-oval-created-sapphire-three-stone-hidden-halo-engagement-ring-14k-white-gold/pid/RIGTXR07350-OV200SPGW4?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Badgley Mischka Near-Colorless 4 1/3 ctw Cushion Lab Grown Diamond Engagement Ring</t>
+          <t>2 ctw Oval Lab Grown Diamond and 7.2x5.1 mm Oval Created Sapphire Three-Stone Hidden Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7836XX%20/medium/RIGJRZ7836XX%20-WG-CU-WH-572-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7836XX%20/medium/RIGJRZ7836XX%20-WG-CU-WH-572-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGR629X1C050/medium/RIGR629X1C050-WG-CU-WH-075-M6.png</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07350/medium/RIGTXR07350-OV-SP-WG-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07350/medium/RIGTXR07350-OV-SP-WG-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
@@ -1239,17 +1515,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/1-7-8-ctw-oval-lab-grown-diamond-engagement-ring-with-floating-marquise-side-accents-14k-white-gold/pid/RIG2638X2O150SOGW2?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-ctw-emerald-lab-grown-diamond-bold-bezel-solitaire-engagement-ring-14k-yellow-gold/pid/RIGRVR02047-GY4?algoliaQueryId=fb04ec293d453cb9cf42bc9be6443633</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>1 7/8 ctw Oval Lab Grown Diamond Engagement Ring with Floating Marquise Side Accents</t>
+          <t>2 ctw Emerald Lab Grown Diamond Bold Bezel Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR02638O200SOX3/medium/TXR02638O200SOX3-WG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR02638O200SOX3/medium/TXR02638O200SOX3-WG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG2638X3O250SO/medium/RIG2638X3O250SO-LW-new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR2638X20150S0GW4/medium/LGR2638X20150S0GW4-GW1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR2638X20150S0GW4/medium/LGR2638X20150S0GW4-GW2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02047/medium/RIGRVR02047-YG-EM-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02047/medium/RIGRVR02047-YG-EM-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -1257,17 +1533,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-3-4-ctw-pear-lab-grown-diamond-side-stone-engagement-ring-18k-yellow-gold/pid/RIGKSR6203-GY3?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-ctw-radiant-lab-grown-diamond-fancy-yellow-with-tapered-baguettes-three-stone-engagement-ring-14k-two-tone-white-and-yellow-gold/pid/RIGTXR05883-YL-GW4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>5 3/4 ctw Pear Lab Grown Diamond Side Stone Engagement Ring</t>
+          <t>2 ctw Radiant Lab Grown Diamond Fancy Yellow With Tapered Baguettes Three-Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6203/medium/RIGKSR6203-YG-PE-WH-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6203/medium/RIGKSR6203-YG-PE-WH-500-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05883/medium/RIGTXR05883-WG-RD-YL-195-M0r.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05883/medium/RIGTXR05883-WG-RD-YL-195-M1r.jpg</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1275,17 +1551,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-2-3-ctw-oval-lab-grown-diamond-engagement-ring-with-pear-side-accents-14k-yellow-gold/pid/RIG0615X3-O200SO-GY?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-ctw-emerald-lab-grown-diamond-celtic-twist-solitaire-engagement-ring-platinum/pid/RIGRVR00064E200PL2?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>2 2/3 ctw Oval Lab Grown Diamond Engagement Ring with Pear Side Accents</t>
+          <t>2 ctw Emerald Lab Grown Diamond Celtic Twist Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00615O200SOX3/medium/TXR00615O200SOX3-YG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00615O200SOX3/medium/TXR00615O200SOX3-YG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0615X3/medium/RIG0615X3-O200SO-GW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00064E200/medium/RIGRVR00064E200-WG-EM-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00064E200/medium/RIGRVR00064E200-WG-EM-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1293,17 +1569,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-1-2-ctw-round-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD02180H-PL1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-ctw-cushion-lab-grown-diamond-and-6-0x3-8-mm-pear-shape-created-sapphire-side-stone-engagement-ring-14k-white-gold/pid/RIGR07343-CUSP-GW1?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Badgley Mischka Colorless 5 1/2 ctw Round Lab Grown Diamond Engagement Ring</t>
+          <t>2 ctw Cushion Lab Grown Diamond and 6.0x3.8 mm Pear Shape Created Sapphire Side Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02180H%20/medium/RIGJRD02180H%20-WG-VR-WH-549-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02180H%20/medium/RIGJRD02180H%20-WG-VR-WH-549-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02180H/medium/RIGJRD02180H-HW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07343/medium/RIGTXR07343-CU-WG-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07343/medium/RIGTXR07343-CU-WG-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
@@ -1311,17 +1587,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-1-3-ctw-oval-lab-grown-diamond-double-heart-shape-prong-split-shank-side-stone-engagement-ring-platinum/pid/RIGRVR04394O500PL2?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/18-0x14-5mm-elongated-cushion-cut-created-sapphire-and-1-1-2-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-with-half-moon-sides-platinum/pid/RIGTXR08898-SP-PL4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>5 1/3 ctw Oval Lab Grown Diamond Double Heart Shape Prong Split Shank Side Stone Engagement Ring</t>
+          <t>18.0x14.5mm Elongated Cushion Cut Created Sapphire and 1 1/2 ctw Round Lab Grown Diamond Hidden Halo Engagement Ring with Half Moon Sides</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04394O500/medium/RIGRVR04394O500-WG-OV-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04394O500/medium/RIGRVR04394O500-WG-OV-500-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08898/medium/RIGTXR08898-SP-WG-CU-WH-150-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08898/medium/RIGTXR08898-SP-WG-CU-WH-150-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08898/medium/RIGTXR08898-R0.jpg</t>
         </is>
       </c>
       <c r="D65" t="inlineStr"/>
@@ -1329,17 +1605,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-3-4-ctw-elongated-cushion-lab-grown-diamond-side-stone-engagement-ring-18k-white-gold/pid/RIGTXR07755Z400HW1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-1-3-ctw-round-lab-grown-diamond-double-baguette-halo-engagement-ring-14k-yellow-gold/pid/RIG0890X4-R150H1-GY?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Badgley Mischka Colorless 4 3/4 ctw Elongated Cushion Lab Grown Diamond Side Stone Engagement Ring</t>
+          <t>2 1/3 ctw Round Lab Grown Diamond Double Baguette Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07755%20(EC%204.0%20SO)/medium/RIGTXR07755%20(EC%204.0%20SO)-WG-ECU-WH-475-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07755%20(EC%204.0%20SO)/medium/RIGTXR07755%20(EC%204.0%20SO)-WG-ECU-WH-475-M1.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00890R200H1X5/medium/TXR00890R200H1X5-YG-RB-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00890R200H1X5/medium/TXR00890R200H1X5-YG-RB-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1347,17 +1623,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-ctw-emerald-lab-grown-diamond-side-stone-engagement-ring-platinum/pid/RIGKSR6129-PL1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/9x7mm-oval-cut-created-ruby-and-1-1-2-ctw-pear-cut-lab-grown-diamond-two-stone-engagement-ring-platinum/pid/RIGTXR06626-RU-PL4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Badgley Mischka Colorless 5 ctw Emerald Lab Grown Diamond Side Stone Engagement Ring</t>
+          <t>9x7mm Oval Cut Created Ruby and 1 1/2 ctw Pear Cut Lab Grown Diamond Two Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6129/medium/RIGKSR6129-WG-EM-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6129/medium/RIGKSR6129-WG-EM-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06626/medium/RIGTXR06626-WG-VR-RU-153-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06626/medium/RIGTXR06626-WG-VR-RU-153-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06626/medium/RIGTXR06626-R0.jpg</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -1365,17 +1641,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-5-8-ctw-oval-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/TXR04040-GY1?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-1-3-ctw-oval-lab-grown-diamond-crossover-double-band-solitaire-engagement-ring-with-side-accents-platinum/pid/RIGYR3734LEC-PL4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>4 5/8 ctw Oval Lab Grown Diamond Hidden Halo Engagement Ring</t>
+          <t>2 1/3 ctw Oval Lab Grown Diamond Crossover Double Band Solitaire Engagement Ring with Side Accents</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04040/medium/RIGTXR04040-GY3_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04040/medium/RIGTXR04040-GY3_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04040/medium/RIGTXR04040-GW3-1-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR3734LEC/medium/RIGYR3734LEC-WG-OV-WH-230-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR3734LEC/medium/RIGYR3734LEC-WG-OV-WH-230-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -1383,17 +1659,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/12x7mm-pear-cut-created-emerald-and-1-2-ctw-lab-grown-diamond-halo-engagement-ring-engagement-ring-14k-white-gold/pid/RIGTXR06627-EM-GW4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/1-1-3-ctw-emerald-lab-grown-diamond-baguette-engagement-ringplatinum/pid/RIGTXR05136E1.0PL1?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>12x7mm Pear Cut Created Emerald and 1/2 ctw Lab Grown Diamond Halo Engagement Ring</t>
+          <t>1 1/3 ctw Emerald Lab Grown Diamond Baguette Engagement Ring</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06627/medium/RIGTXR06627-EM-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06627/medium/RIGTXR06627-EM-GW4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06627/medium/RIGTXR06627-EM-GW4-new.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05136/medium/RIGTXR05136-WG-EM-WH-100-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05136/medium/RIGTXR05136-WG-EM-WH-100-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
@@ -1401,17 +1677,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-4-ctw-emerald-lab-grown-diamond-engagement-ring-with-tapered-baguette-side-accents-14k-white-gold/pid/RIG0617X3-E200SO-GW?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/10x8-mm-oval-cut-created-emerald-and-5-8-ctw-oval-lab-grown-diamond-halo-engagement-ring-14k-yellow-gold/pid/RIGTXR06705-EM-GY4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>2 1/4 ctw Emerald Lab Grown Diamond Engagement Ring with Tapered Baguette Side Accents</t>
+          <t>10X8 mm Oval Cut Created Emerald and 5/8 ctw Oval Lab Grown Diamond Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0617X3/medium/RIG0617X3-E200SO-GW-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0617X3/medium/RIG0617X3-E200SO-GW-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0617X3E200/medium/LGR0617X3E200-shape.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06705/medium/RIGTXR06705-YG-EM-OV-617-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06705/medium/RIGTXR06705-YG-EM-OV-617-M1.jpg</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
@@ -1419,17 +1695,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-3-4-ctw-oval-lab-grown-diamond-hidden-halo-bridal-set-platinum/pid/BRDTXR06232O200PL2?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-3-8-ctw-round-lab-grown-diamond-double-row-engagement-ring-14k-yellow-gold/pid/RIG0623X3-R200SO-GY?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>2 3/4 ctw Oval Lab Grown Diamond Hidden Halo Bridal Set</t>
+          <t>2 3/8 ctw Round Lab Grown Diamond Double Row Engagement Ring</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06232/medium/RIGTXR06232-WG-OV-WH-276-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06232/medium/RIGTXR06232-WG-OV-WH-276-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR06232O200GW1/medium/BRDTXR06232O200GW1-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00623R200SOX3/medium/TXR00623R200SOX3-YG-RB-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00623R200SOX3/medium/TXR00623R200SOX3-YG-RB-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
@@ -1437,17 +1713,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-radiant-lab-grown-diamond-solitaire-engagement-ring-platinum/pid/RIGJRO1322-PL_5?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/2-1-5-ctw-oval-lab-grown-diamond-station-halo-engagement-ring-14k-rose-gold/pid/RIG1860X4-O150H1-GS?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>3 ctw Radiant Lab Grown Diamond Solitaire Engagement Ring</t>
+          <t>2 1/5 ctw Oval Lab Grown Diamond Station Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRO1322/medium/RIGJRO1322-WG-RD1-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRO1322/medium/RIGJRO1322-WG-RD-WH-300-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR01860O200H1X5/medium/TXR01860O200H1X5-RG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR01860O200H1X5/medium/TXR01860O200H1X5-RG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D72" t="inlineStr"/>
@@ -1455,17 +1731,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-1-3-ctw-princess-lab-grown-diamond-split-shank-engagement-ring-platinum/pid/LGR0625X3-P300SO-PL4?algoliaQueryId=4eba6a6d920558fa8dc3748625f4e603</t>
+          <t>https://www.grownbrilliance.com/boundless-star-ring-14k-white-gold/pid/BORIGAR02135YE-GW4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>3 1/3 ctw Princess Lab Grown Diamond Split Shank Engagement Ring</t>
+          <t>Boundless Star Ring</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X3P300SO/medium/RIG0625X3P300SO-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X3P300SO/medium/RIG0625X3P300SO-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0589X3/medium/LGR0589X3-P300SO-FIN.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAAR02135YE/medium/RIGAAR02135YE-WG-RB-150-M0-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAAR02135YE/medium/RIGAAR02135YE-WG-RB-150-M1-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BORIGAR02135YE/medium/BORIGAR02135YE-GW4-1.jpg</t>
         </is>
       </c>
       <c r="D73" t="inlineStr"/>
@@ -1473,17 +1749,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-7-8-ctw-cushion-lab-grown-diamond-graduated-halo-engagement-ring-14k-white-gold/pid/RIG0641X4C200H1GW2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/9-5-mm-heart-shaped-created-ruby-and-1-2-ctw-round-lab-grown-diamond-solitaire-engagement-ring-with-side-accents-14k-white-gold/pid/RIGTXR07245-RU-GW4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>2 7/8 ctw Cushion Lab Grown Diamond Graduated Halo Engagement Ring</t>
+          <t>9.5 mm Heart Shaped Created Ruby and 1/2 ctw Round Lab Grown Diamond Solitaire Engagement Ring with Side Accents</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00641C200H1X5/medium/TXR00641C200H1X5-WG-CU-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00641C200H1X5/medium/TXR00641C200H1X5-WG-CU-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07245/medium/RIGTXR07245-WG-HT-WH-350-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07245/medium/RIGTXR07245-WG-HT-WH-350-M1.jpg</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -1491,17 +1767,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/11x9mm-created-emerald-and-1-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR06623-EM-GW4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/2-1-4-ctw-oval-lab-grown-diamond-classic-solitaire-halo-engagement-ring-14k-rose-gold/pid/RIG2598X4-O200H1-GS?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>11x9mm Created Emerald and 1 ctw Lab Grown Diamond Three-Stone Engagement Ring</t>
+          <t>2 1/4 ctw Oval Lab Grown Diamond Classic Solitaire Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06623/medium/RIGTXR06623-EM-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06623/medium/RIGTXR06623-EM-GW4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06623/medium/RIGTXR06623-EM-GW4-new.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR02598O200H1X5/medium/TXR02598O200H1X5-RG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR02598O200H1X5/medium/TXR02598O200H1X5-RG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
@@ -1509,17 +1785,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-bezel-set-solitaire-engagement-ring-platinum/pid/RIGTXR06655EM500PL3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/19-5x13-9mm-oval-cut-created-sapphire-and-1-1-2-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/RIGTXR08897-SP-GY4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>5 ctw Emerald Lab Grown Diamond Bezel Set Solitaire Engagement Ring</t>
+          <t>19.5x13.9mm Oval Cut Created Sapphire and 1 1/2 ctw Round Lab Grown Diamond Hidden Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06655/medium/RIGTXR06655-WG-EM-WH-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06655/medium/RIGTXR06655-WG-EM-WH-500-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08897/medium/RIGTXR08897-SP-YG-OV-WH-150-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08897/medium/RIGTXR08897-SP-YG-OV-WH-150-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08897/medium/RIGTXR08897-R0.jpg</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
@@ -1527,17 +1803,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-2-3-ctw-multi-shape-lab-grown-diamond-vintage-inspired-art-deco-engagement-ring-platinum/pid/RIGRVR05013-PL4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/2-ctw-radiant-lab-grown-diamond-oval-side-stones-halo-engagement-ring-14k-yellow-gold/pid/RIG0893X4-T150H1-GY?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>2 2/3 ctw Multi-Shape Lab Grown Diamond Vintage Inspired Art Deco Engagement Ring</t>
+          <t>2 ctw Radiant Lab Grown Diamond Oval Side Stones Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05013/medium/RIGRVR05013-WG-265N-VR-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05013/medium/RIGRVR05013-WG-265N-VR-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05013/medium/RIGRVR05013-GW1-NEW.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00893T200H1X5/medium/TXR00893T200H1X5-YG-RD-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00893T200H1X5/medium/TXR00893T200H1X5-YG-RD-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -1545,17 +1821,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/10x8-mm-created-emerald-and-1-3-8-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR06678-EM-GW4?algoliaQueryId=961725d3c54423b9205778064301ed8e&amp;amp;in_stock=yes</t>
+          <t>https://www.grownbrilliance.com/10x8-mm-oval-cut-created-sapphire-and-7-8-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR06677-SP-GW4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>10x8 mm Created Emerald and 1 3/8 ctw Lab Grown Diamond Three-Stone Engagement Ring</t>
+          <t>10x8 mm Oval Cut Created Sapphire and 7/8 ctw Lab Grown Diamond Three-Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06678/medium/RIGTXR06678-EM-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06678/medium/RIGTXR06678-EM-GW4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06678/medium/RIGTXR06678-EM-GW4-1-NEW.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06677/medium/RIGTXR06677-SP-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06677/medium/RIGTXR06677-SP-GW4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06677/medium/RIGTXR06677-SP-GW4-new.jpg</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -1563,17 +1839,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-2-3-ctw-oval-lab-grown-diamond-three-stone-engagement-ring-with-half-moon-sides-platinum/pid/RIGTXR06001OV30PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/8-mm-cushion-cut-created-sapphire-and-1-1-3-ctw-round-and-pear-lab-grown-diamond-halo-engagement-ring-14k-yellow-gold/pid/RIGTXR06706-SP-GY4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>4 2/3 ctw Oval Lab Grown Diamond Three-Stone Engagement Ring with Half Moon sides</t>
+          <t>8 mm Cushion Cut Created Sapphire and 1 1/3 ctw Round and Pear Lab Grown Diamond Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06001/medium/RIGTXR06001-WG-OV-WH-441-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06001/medium/RIGTXR06001-WG-OV-WH-441-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06706/medium/RIGTXR06706-YG-SP-CU-134-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06706/medium/RIGTXR06706-YG-SP-CU-134-M1.jpg</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -1581,35 +1857,31 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-3-4-ctw-cushion-lab-grown-diamond-split-shank-x-side-stone-engagement-ring-14k-rose-gold/pid/RIGRV08957C400-GP2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/2-ctw-pear-lab-grown-diamond-fancy-yellow-with-prong-set-frame-halo-engagement-ring-14k-two-tone-white-and-yellow-gold/pid/RIGTXR05877-YL-GW4?algoliaQueryId=8a0bd6004417e27e6a319adf0a9057a9</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>4 3/4 ctw Cushion Lab Grown Diamond Split Shank X  Side Stone Engagement Ring</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR08957C400/medium/RIGRVR08957C400-RG-CU-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR08957C400/medium/RIGRVR08957C400-RG-CU-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
-        </is>
-      </c>
+          <t>2 ctw Pear Lab Grown Diamond Fancy Yellow With Prong Set Frame Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
       <c r="D80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/6-1-4-ctw-oval-lab-grown-diamond-trapezoid-and-pear-side-stone-bridal-set-platinum/pid/BRDTXR08417O500PL4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/1-1-2-ctw-pear-lab-grown-diamond-fancy-pink-split-shank-double-halo-engagement-ring/pid/RIGTXR05876-PN-GR4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>6 1/4 ctw Oval Lab Grown Diamond Trapezoid and Pear Side Stone Bridal Set</t>
+          <t>1 1/2 ctw Pear Lab Grown Diamond Fancy Pink Split Shank Double Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08417O500/medium/BRDTXR08417O500-WG-OV-WH-625-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08417O500/medium/BRDTXR08417O500-WG-OV-WH-625-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05876/medium/RIGTXR05876-RG-PE-PN-150-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05876/medium/RIGTXR05876-RG-PE-PN-150-M1.jpg</t>
         </is>
       </c>
       <c r="D81" t="inlineStr"/>
@@ -1617,17 +1889,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-toi-et-moi-pear-and-oval-engagement-ring-14k-white-gold/pid/RIGTXR05974PO30-GW4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/9x7-mm-radiant-cut-created-emerald-and-7-8-ctw-round-and-half-moon-lab-grown-diamond-side-stone-engagement-ring-14k-yellow-gold/pid/RIGTXR06125-EM-GY4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>3 ctw Toi Et Moi Pear and Oval Engagement Ring</t>
+          <t>9X7 mm Radiant Cut Created Emerald and 7/8 ctw Round and Half Moon Lab Grown Diamond Side Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05974/medium/RIGTXR05974-WG-VR-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05974/medium/RIGTXR05974-WG-VR-WH-300-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGDTXR05974PO30GW%20/medium/LGDTXR05974PO30GW%20-%201.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06125/medium/RIGTXR06125-YG-EM-RD-080-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06125/medium/RIGTXR06125-YG-EM-RD-080-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06125/medium/RIGTXR06125-R0.jpg</t>
         </is>
       </c>
       <c r="D82" t="inlineStr"/>
@@ -1635,17 +1907,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-10-ctw-oval-lab-grown-diamond-pave-prong-solitaire-engagement-ring-with-hidden-accents-14k-yellow-gold/pid/RIGTXR05578O200GY2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/11x9-mm-oval-cut-created-emerald-and-3-4-ctw-lab-grown-diamond-side-stone-engagement-ring-14k-white-gold/pid/RIGTXR06682-EM-GW4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>2 1/10 ctw Oval Lab Grown Diamond Pave Prong Solitaire Engagement Ring with Hidden Accents</t>
+          <t>11x9 mm Oval Cut Created Emerald and 3/4 ctw Lab Grown Diamond Side Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05578/medium/RIGTXR05578-YG-OV-WH-212-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05578/medium/RIGTXR05578-YG-OV-WH-212-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06680/medium/RIGTXR06680-WG-OV-ER-076-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06680/medium/RIGTXR06680-WG-OV-ER-076-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06681/medium/RIGTXR06681-R0.jpg</t>
         </is>
       </c>
       <c r="D83" t="inlineStr"/>
@@ -1653,17 +1925,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-7-8-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-platinum/pid/RIGTXR09619R300PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/1-2-5-ctw-cushion-lab-grown-diamond-luxe-celtic-side-stone-engagement-ring-14k-white-gold/pid/RIGRVR00043C100GW4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>3 7/8 ctw Round Lab Grown Diamond Hidden Halo Engagement Ring</t>
+          <t>1 2/5 ctw Cushion Lab Grown Diamond Luxe Celtic Side Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR09619/medium/TXR09619-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR09619/medium/TXR09619-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09619R300GW4/medium/RIGTXR09619R300GW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00043C100/medium/RIGRVR00043C100-WG-CU-WH-143-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00043C100/medium/RIGRVR00043C100-WG-CU-WH-143-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
         </is>
       </c>
       <c r="D84" t="inlineStr"/>
@@ -1671,17 +1943,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-cushion-lab-grown-diamond-v-prong-halo-engagement-ring-14k-white-gold/pid/RIG0639X4C200H1GW2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/10x8mm-ctw-oval-cut-created-ruby-and-1-2-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-yellow-gold/pid/RIGTXR06622-RU-GY4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>2 1/2 ctw Cushion Lab Grown Diamond V-Prong Halo Engagement Ring</t>
+          <t>10x8mm ctw Oval Cut Created Ruby and 1/2 ctw Lab Grown Diamond Three-Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00639C200H1X5/medium/TXR00639C200H1X5-WG-CU-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00639C200H1X5/medium/TXR00639C200H1X5-WG-CU-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06622/medium/RIGTXR06622-YG-OV-RU-050-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06622/medium/RIGTXR06622-YG-OV-RU-050-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06622/medium/RIGTXR06622-R0.jpg</t>
         </is>
       </c>
       <c r="D85" t="inlineStr"/>
@@ -1689,17 +1961,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-emerald-lab-grown-diamond-solitaire-engagement-ring-platinum/pid/RIGTXR09875E400PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/8-mm-emerald-cut-created-emerald-and-2-5-ctw-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGTXR07161-EM-GW4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>4 ctw Emerald Lab Grown Diamond Solitaire Engagement Ring</t>
+          <t>8 mm Emerald Cut Created Emerald and 2/5 ctw Lab Grown Diamond Three-Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09875E400/medium/RIGTXR09875E400-WG-EM-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09875E400/medium/RIGTXR09875E400-WG-EM-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07161/medium/RIGTXR07161-EM-GW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07161/medium/RIGTXR07161-EM-GW4-2.jpg</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
@@ -1707,17 +1979,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/13-4mm-cushion-cut-created-emerald-and-2-ctw-pear-lab-grown-diamond-three-stone-engagement-ring-14k-yellow-gold/pid/RIGTXR08896-EM-GY4?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/10x8mm-emerald-cut-created-sapphire-and-1-7-8-ctw-round-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGJOR5734-SP-GW4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>13.4mm Cushion Cut Created Emerald and 2 ctw Pear Lab Grown Diamond Three Stone Engagement Ring</t>
+          <t>10X8mm Emerald Cut Created Sapphire and 1 7/8 ctw Round Lab Grown Diamond Three-Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08896/medium/RIGTXR08896-EM-GY4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08896/medium/RIGTXR08896-EM-GY4-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08896/medium/RIGTXR08896-R0.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGD/medium/LGD-JOR5734-GW60SP-GB.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGD/medium/LGD-JOR5734-GW60SP-3-GB.jpg</t>
         </is>
       </c>
       <c r="D87" t="inlineStr"/>
@@ -1725,17 +1997,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-twist-solitaire-engagement-ring-14k-white-gold/pid/RIGTXR05112-GW4-3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/7-7x5-5-mm-oval-cut-created-sapphire-and-1-3-4-ctw-round-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGJOR5738-SP-GW4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>3 ctw Round Lab Grown Diamond Twist Solitaire Engagement Ring</t>
+          <t>7.7x5.5 mm Oval Cut Created Sapphire and 1 3/4 ctw Round Lab Grown Diamond Three-Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05112/medium/RIGTXR05112-WG-RB-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05112/medium/RIGTXR05112-WG-RB-WH-300-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGDJOR5738/medium/LGDJOR5738-GW60SP.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGDJOR5738GW60SP/medium/LGDJOR5738GW60SP-2.jpg</t>
         </is>
       </c>
       <c r="D88" t="inlineStr"/>
@@ -1743,17 +2015,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-1-2-ctw-cushion-lab-grown-diamond-halo-engagement-ring-platinum/pid/RIGKSR6111N-PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/1-2-ctw-emerald-lab-grown-diamond-petite-solitaire-engagement-ring-14k-yellow-gold/pid/RIGTXR05314E50-GY1?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Badgley Mischka Colorless 3 1/2 ctw Cushion Lab Grown Diamond Halo Engagement Ring</t>
+          <t>1/2 ctw Emerald Lab Grown Diamond Petite Solitaire Engagement Ring</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6111/medium/RIGKSR6111-WG-CU-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6111/medium/RIGKSR6111-WG-CU-WH-300-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6184N/medium/RIGKSR6184N-HW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05314E50/medium/RIGTXR05314E50-GY4_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05314E50/medium/RIGTXR05314E50-GY4_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR05314X1E050/medium/TXR05314X1E050-GY1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR05314X1E050/medium/TXR05314X1E050-GY2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D89" t="inlineStr"/>
@@ -1761,17 +2033,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-1-4-ctw-oval-lab-grown-diamond-three-stone-bridal-set-platinum/pid/BRDTXR08075O300PL1?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-3-4-ctw-radiant-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ7847XX-HW_5?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>4 1/4 ctw Oval Lab Grown Diamond Three-Stone Bridal Set</t>
+          <t>Badgley Mischka Colorless 3 3/4 ctw Radiant Lab Grown Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08075O300/medium/BRDTXR08075O300-WG-OV-WH-426-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08075O300/medium/BRDTXR08075O300-WG-OV-WH-426-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7847XX/medium/RIGJRZ7847XX-HW_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7847XX/medium/RIGJRZ7847XX-HW_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
         </is>
       </c>
       <c r="D90" t="inlineStr"/>
@@ -1779,17 +2051,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-1-3-ctw-princess-lab-grown-diamond-hidden-halo-engagement-ring-18k-white-gold/pid/RIGKSR6164-GW3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-4-1-2-ctw-oval-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ76040H-PL4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Badgley Mischka Colorless 4 1/3 ctw Princess Lab Grown Diamond Hidden Halo Engagement Ring</t>
+          <t>Badgley Mischka Near-Colorless 4 1/2 ctw Oval Lab Grown Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6164/medium/RIGKSR6164-WG-PR-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6164/medium/RIGKSR6164-WG-PR-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76040H%20/medium/RIGJRZ76040H%20-WG-VR-WH-440-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76040H%20/medium/RIGJRZ76040H%20-WG-VR-WH-440-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D91" t="inlineStr"/>
@@ -1797,17 +2069,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-1-5-ctw-cushion-lab-grown-diamond-old-mine-cut-milgrain-split-floral-shank-side-stone-engagement-ring-platinum/pid/RIGRVR06510-PL2?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-radiant-lab-grown-diamond-side-stone-engagement-ring-18k-white-gold/pid/RIGJRD0253XX-HW_5?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>5 1/5 ctw Cushion Lab Grown Diamond Old Mine Cut Milgrain Split Floral Shank Side Stone Engagement Ring</t>
+          <t>3 1/2 ctw Radiant Lab Grown Diamond Side Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06510/medium/RIGRVR06510-WG-CU-491-M0_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06510/medium/RIGRVR06510-WG-CU-491-M1_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0253XX/medium/RIGJRD0253XX-WG-RD1-WH-327-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0253XX/medium/RIGJRD0253XX-WG-RD1-WH-327-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
         </is>
       </c>
       <c r="D92" t="inlineStr"/>
@@ -1815,17 +2087,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-4-ctw-emerald-lab-grown-diamond-baguette-sides-engagement-ring-14k-white-gold/pid/RIGR617X3E20-GW3?algoliaQueryId=961725d3c54423b9205778064301ed8e</t>
+          <t>https://www.grownbrilliance.com/4-2-3-ctw-old-mine-cut-lab-grown-diamond-solitaire-engagement-ring-with-side-accents-platinum/pid/RIGTXR06813-PL4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>2 1/4 ctw Emerald Lab Grown Diamond Baguette Sides Engagement Ring</t>
+          <t>4 2/3 ctw Old Mine Cut Lab Grown Diamond Solitaire Engagement Ring with Side Accents</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGR617X3E20/medium/RIGR617X3E20-WG-EM-WH-224-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGR617X3E20/medium/RIGR617X3E20-WG-EM-WH-224-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0617X3E200/medium/LGR0617X3E200-GW1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0617X3E200/medium/LGR0617X3E200-GW2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06813/medium/RIGTXR06813-WG-CU-WH-443-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06813/medium/RIGTXR06813-WG-CU-WH-443-M1.jpg</t>
         </is>
       </c>
       <c r="D93" t="inlineStr"/>
@@ -1833,17 +2105,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-royal-crown-engagement-ring-14k-white-gold/pid/RIG0621X3-T200SO-GW?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-oval-lab-grown-diamond-prong-hidden-halo-engagement-ring-18k-white-gold/pid/RIGTXR05667-HW4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>2 1/2 ctw Radiant Lab Grown Diamond Royal Crown Engagement Ring</t>
+          <t>2 1/2 ctw Oval Lab Grown Diamond Prong Hidden Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00621T200SOX3/medium/TXR00621T200SOX3-WG-RD-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00621T200SOX3/medium/TXR00621T200SOX3-WG-RD-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05667/medium/RIGTXR05667-WG-VR-WH-250-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05667/medium/RIGTXR05667-WG-VR-WH-250-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D94" t="inlineStr"/>
@@ -1851,17 +2123,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-1-2-ctw-round-lab-grown-diamond-three-stone-engagement-ring-with-side-diamonds-platinum/pid/RIGAJ01024R300-PL2?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-2-5-ctw-cushion-lab-grown-diamond-large-halo-engagement-ring/pid/RIGTXR06222-PL3?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>4 1/2 ctw Round Lab Grown Diamond Three Stone Engagement Ring with Side Diamonds</t>
+          <t>Badgley Mischka Colorless 3 2/5 ctw Cushion Lab Grown Diamond Large Halo Engagement Ring</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01024R200/medium/RIGAJR01024R200-WG-RB-320-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01024R200/medium/RIGAJR01024R200-WG-RB-320-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06222/medium/RIGTXR06222-WG-CU-WH-340-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06222/medium/RIGTXR06222-WG-CU-WH-340-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGD/medium/LGD-TXR06222-PL3-HAND.jpg</t>
         </is>
       </c>
       <c r="D95" t="inlineStr"/>
@@ -1869,17 +2141,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-1-2-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-platinum/pid/RIGTXR06690R300PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/3-2-5-ctw-emerald-lab-grown-diamond-three-stone-engagement-ring-with-trillion-side-stones-14k-white-gold/pid/RIGTXR06002EM3.0-GW4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>3 1/2 ctw Round Lab Grown Diamond Hidden Halo Engagement Ring</t>
+          <t>3 2/5 ctw Emerald Lab Grown Diamond Three-Stone Engagement Ring with Trillion Side Stones</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG06690R300/medium/RIG06690R300-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG06690R300/medium/RIG06690R300-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06002/medium/RIGTXR06002-WG-EM-WH-356-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06002/medium/RIGTXR06002-WG-EM-WH-356-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D96" t="inlineStr"/>
@@ -1887,17 +2159,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-5-8-ctw-round-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD0230XX-PL3?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/2-ctw-oval-lab-grown-diamond-fancy-yellow-with-trillion-three-stone-engagement-ring-14k-two-tone-white-and-yellow-gold/pid/RIGTXR05873-YL-GW4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>4 5/8 ctw Round Lab Grown Diamond Engagement Ring</t>
+          <t>2 ctw Oval Lab Grown Diamond Fancy Yellow With Trillion Three-Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0230XX/medium/RIGJRD0230XX-WG-RB-WH-402-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0230XX/medium/RIGJRD0230XX-WG-RB-WH-402-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05873/medium/RIGTXR05873-WG-OV-YL-200-M0r.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05873/medium/RIGTXR05873-WG-OV-YL-200-M1r.jpg</t>
         </is>
       </c>
       <c r="D97" t="inlineStr"/>
@@ -1905,17 +2177,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-3-4-ctw-cushion-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD02104Q-PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/1-7-8-ctw-round-lab-grown-diamond-crossover-engagement-ring-14k-white-gold/pid/RIG0631X2-R150SO-GW?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>3 3/4 ctw Cushion Lab Grown Diamond Engagement Ring</t>
+          <t>1 7/8 ctw Round Lab Grown Diamond Crossover Engagement Ring</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02104Q/medium/RIGJRD02104Q-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02104Q/medium/RIGJRD02104Q-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02104Q/medium/RIGJRD02104Q-HW4-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00631R200SOX3/medium/TXR00631R200SOX3-WG-RB-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00631R200SOX3/medium/TXR00631R200SOX3-WG-RB-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
         </is>
       </c>
       <c r="D98" t="inlineStr"/>
@@ -1923,17 +2195,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-1-3-ctw-radiant-lab-grown-diamond-hidden-halo-bridal-set-platinum/pid/BRDTXR07490-PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/6-1-5-ctw-emerald-lab-grown-diamond-three-stone-engagement-ring-with-half-moon-sides-14k-white-gold/pid/RIGTXR06001EM5.0-GW4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>4 1/3 ctw Radiant Lab Grown Diamond Hidden Halo Bridal Set</t>
+          <t>6 1/5 ctw Emerald Lab Grown Diamond Three-Stone Engagement Ring with Half Moon sides</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07490/medium/TXR07490-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07490/medium/TXR07490-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06001/medium/RIGTXR06001-WG-EM-WH-589-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06001/medium/RIGTXR06001-WG-EM-WH-589-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
         </is>
       </c>
       <c r="D99" t="inlineStr"/>
@@ -1941,17 +2213,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/5-ctw-oval-lab-grown-diamond-three-stone-ring-18k-white-gold/pid/RIGJRD0242XX-PL18?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/5-ctw-oval-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD0259XX-PL4?algoliaQueryId=e33cee3d064616cd88aee9aea1c7902e</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>5 ctw Oval Lab Grown Diamond Three-Stone Ring</t>
+          <t>5 ctw Oval Lab Grown Diamond Engagement Ring</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0242XX/medium/RIGJRD0242XX-WG-RB-WH-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0242XX/medium/RIGJRD0242XX-WG-RB-WH-500-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0259XX%20/medium/RIGJRD0259XX%20-WG-VR-WH-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0259XX%20/medium/RIGJRD0259XX%20-WG-VR-WH-500-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D100" t="inlineStr"/>
@@ -1959,17 +2231,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-and-7-2-mm-round-shape-created-sapphire-three-stone-engagement-ring-platinum/pid/RIGR07347-RDSP-PL1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/1-3-4-ctw-round-lab-grown-diamond-vintage-inspired-old-mine-cut-engagement-ring-14k-yellow-gold/pid/RIGRV05552R100-GY4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>3 ctw Round Lab Grown Diamond and 7.2 mm Round Shape Created Sapphire Three-Stone Engagement Ring</t>
+          <t>1 3/4 ctw Round Lab Grown Diamond Vintage Inspired Old Mine Cut Engagement Ring</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07347/medium/RIGTXR07347-RB-WG-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07347/medium/RIGTXR07347-RB-WG-WH-300-M1.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05552R100/medium/RIGRVR05552R100-YG-175N-VR-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05552R100/medium/RIGRVR05552R100-YG-175N-VR-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRV05552R200/medium/RIGRV05552R200-GW4-NEW.jpg</t>
         </is>
       </c>
       <c r="D101" t="inlineStr"/>
@@ -1977,17 +2249,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/16-0x11-25-mm-radiant-cut-created-ruby-and-6-ctw-trapezoid-lab-grown-diamond-engagement-ring-with-side-accents-platinum/pid/RIGTXR08893-RU-PL4?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-cushion-lab-grown-diamond-old-mine-cut-filigree-with-baguettes-side-stone-engagement-ring-14k-white-gold/pid/RIGRVR06509-GW4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>16.0x11.25 mm Radiant Cut Created Ruby and 6 ctw Trapezoid Lab Grown Diamond Engagement Ring with Side Accents</t>
+          <t>3 1/2 ctw Cushion Lab Grown Diamond Old Mine Cut Filigree with Baguettes Side Stone Engagement Ring</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08893/medium/RIGTXR08893-RU-WG-RD-WH-598-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08893/medium/RIGTXR08893-RU-WG-RD-WH-598-M1.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06509/medium/RIGRVR06509-WG-CU-347-M0_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06509/medium/RIGRVR06509-WG-CU-347-M1_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06509/medium/RIGRVR06509-GW4.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
@@ -1995,20 +2267,2352 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>https://www.grownbrilliance.com/4-ctw-cushion-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRD02094Q-HP1?algoliaQueryId=128f3e2a20a017abe5de766c5fa68c77</t>
+          <t>https://www.grownbrilliance.com/1-1-2-ctw-oval-lab-grown-diamond-seven-stone-graduated-engagement-ring-14k-white-gold/pid/RIGRVR0082O100-GW4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>4 ctw Cushion Lab Grown Diamond Engagement Ring</t>
+          <t>1 1/2 ctw Oval Lab Grown Diamond Seven Stone Graduated Engagement Ring</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02094Q/medium/RIGJRD02094Q-RG-RB-WH-396-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02094Q/medium/RIGJRD02094Q-RG-RB-WH-396-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGR00882O100/medium/RIGR00882O100-WG-OV-WH-150-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGR00882O100/medium/RIGR00882O100-WG-OV-WH-150-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-fancy-pink-emerald-lab-grown-diamond-split-shank-side-stone-engagement-ring-platinum/pid/RIGTXR09156-PN-PL4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Fancy Pink Emerald Lab Grown Diamond Split Shank Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09156P/medium/RIGTXR09156P-WG-EM-WH-350-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09156P/medium/RIGTXR09156P-WG-EM-WH-350-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09156/medium/RIGTXR09156-PN-BL-YL.jpg</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-6-ctw-oval-lab-grown-diamond-halo-engagement-ring-14k-white-gold/pid/RIGTXR07513-GW4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>4 1/6 ctw Oval Lab Grown Diamond Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07513/medium/TXR07513-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07513/medium/TXR07513-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-6-ctw-round-lab-grown-diamond-solitaire-engagement-ring-with-round-and-baguette-side-accents/pid/RIGTXR06224-RD-PL3?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 6 ctw Round Lab Grown Diamond Solitaire Engagement Ring with Round and Baguette Side Accents</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06224/medium/RIGTXR06224-WG-RB-WH-593-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06224/medium/RIGTXR06224-WG-RB-WH-593-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-3-4-ctw-cushion-lab-grown-diamond-fancy-pink-with-trillion-three-stone-engagement-ring/pid/RIGTXR05867-PN-GY4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>1 3/4 ctw Cushion Lab Grown Diamond Fancy Pink With Trillion Three-Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05867/medium/RIGTXR05867-RG-CU-PN-174-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05867/medium/RIGTXR05867-RG-CU-PN-174-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-knot-engagement-ring-platinum/pid/RIG0892X2-R150SO-LW?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>2 ctw Round Lab Grown Diamond Knot Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00892R200SOX3/medium/TXR00892R200SOX3-WG-RB-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00892R200SOX3/medium/TXR00892R200SOX3-WG-RB-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-3-ctw-oval-lab-grown-diamond-swirl-halo-engagement-ring-14k-white-gold/pid/RIG1007X4-O150H1-GW?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>2 1/3 ctw Oval Lab Grown Diamond Swirl Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR01007O200H1X5/medium/TXR01007O200H1X5-WG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR01007O200H1X5/medium/TXR01007O200H1X5-WG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-marquise-shape-sides-halo-engagement-ring-14k-white-gold/pid/RIG0586X4-T200H1-GW?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Radiant Lab Grown Diamond Marquise Shape Sides Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00586T200H1X5/medium/TXR00586T200H1X5-WG-RD-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00586T200H1X5/medium/TXR00586T200H1X5-WG-RD-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-7-8-ctw-oval-lab-grown-diamond-channel-halo-engagement-ring-14k-white-gold/pid/RIG0637X4-O150H1-GW?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>1 7/8 ctw Oval Lab Grown Diamond Channel Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00637O200H1X5/medium/TXR00637O200H1X5-WG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00637O200H1X5/medium/TXR00637O200H1X5-WG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/9-ctw-fancy-pink-radiant-lab-grown-diamond-open-two-stone-engagement-ring-14k-two-tone-white-and-pink-gold/pid/RIGAJR01073PN-GWR4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>9 ctw Fancy Pink Radiant Lab Grown Diamond Open Two Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01073TP/medium/RIGAJR01073TP-RW-RD-900-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01073TP/medium/RIGAJR01073TP-RW-RD-900-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/boundless-love-ring-14k-white-gold/pid/BORIGAR01884JE-GW4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Boundless Love Ring</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAAR01884JE/medium/RIGAAR01884JE-WG-RB-150-M0-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAAR01884JE/medium/RIGAAR01884JE-WG-RB-150-M1-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BORIGAR01884JE/medium/BORIGAR01884JE-GW4-1.jpg</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-3-4-ctw-round-lab-grown-diamond-six-prong-channel-set-side-stone-engagement-ring-14k-white-gold/pid/RIGRV08548R150-GW4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>1 3/4 ctw Round Lab Grown Diamond Six Prong Channel Set Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR08548R150/medium/RIGRVR08548R150-WG-RD-150-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR08548R150/medium/RIGRVR08548R150-WG-RD-150-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-3-ctw-fancy-blue-oval-lab-grown-diamond-three-stone-engagement-ring-platinum/pid/RIGTXR09150-BL-PL4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>4 1/3 ctw Fancy Blue Oval Lab Grown Diamond Three Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09150B/medium/RIGTXR09150B-WG-OV-WH-430-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09150B/medium/RIGTXR09150B-WG-OV-WH-430-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09150/medium/RIGTXR09150-BL-PN-YL.jpg</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-7-8-ctw-fancy-pink-round-lab-grown-diamond-side-stone-engagement-ring-14k-white-gold/pid/RIGTXR09161-PN-GW4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>3 7/8 ctw Fancy Pink Round Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09161P/medium/RIGTXR09161P-WG-RB-WH-385-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09161P/medium/RIGTXR09161P-WG-RB-WH-385-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09161/medium/RIGTXR09161-PN-BL-YL.jpg</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-3-4-ctw-oval-fancy-blue-lab-grown-diamond-halo-engagement-ring-14k-white-gold/pid/RIGTXR05874-BL-GW4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>1 3/4 ctw Oval Fancy Blue Lab Grown Diamond Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05874BLU/medium/RIGTXR05874BLU-WG-OV-WH-176-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05874BLU/medium/RIGTXR05874BLU-WG-OV-WH-176-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-1-4-ctw-radiant-fancy-blue-lab-grown-diamond-halo-engagement-ring-14k-white-gold/pid/RIGTXR05881-BL-GW4?algoliaQueryId=c2281a98d6ca6caf6587edb6150ada79</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>1 1/4 ctw Radiant Fancy Blue Lab Grown Diamond Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05881BLU/medium/RIGTXR05881BLU-WG-RD-WH-125-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05881BLU/medium/RIGTXR05881BLU-WG-RD-WH-125-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-ctw-round-lab-grown-diamond-side-stone-engagement-ring-14k-yellow-gold/pid/RIGTXR08477-GY4?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>4 ctw Round Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08477/medium/RIGTXR08477-YG-RB-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08477/medium/RIGTXR08477-YG-RB-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-3-ctw-elongated-cushion-lab-grown-diamond-side-stone-engagement-ring-platinum/pid/RIGTXR07757Z200-PL6?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Near-Colorless 3 ctw Elongated Cushion Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07757(EC%202.0%20SO)/medium/RIGTXR07757(EC%202.0%20SO)-WG-ECU-WH-344-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07757(EC%202.0%20SO)/medium/RIGTXR07757(EC%202.0%20SO)-WG-ECU-WH-344-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-ctw-asscher-lab-grown-diamond-hidden-halo-bridal-set-platinum/pid/BRDTXR07445-PL3?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>4 ctw Asscher Lab Grown Diamond Hidden Halo Bridal Set</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07445/medium/TXR07445-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07445/medium/TXR07445-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-AS.jpg</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-3-4-ctw-emerald-lab-grown-diamond-solitaire-engagement-ring-with-graduated-side-accents-18k-platinum/pid/RIGTXR06786-PL3?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 3 3/4 ctw Emerald Lab Grown Diamond Solitaire Engagement Ring with Graduated Side Accents</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06786/medium/RIGTXR06786-WG-OV-WH-351-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06786/medium/RIGTXR06786-WG-OV-WH-351-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-ctw-emerald-lab-grown-diamond-and-5-0x4-2x3-0-mm-bullet-shape-created-sapphire-side-stone-engagement-ring-platinum/pid/RIGTXR07344-EMSP-PL4?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>3 ctw Emerald Lab Grown Diamond and 5.0x4.2x3.0 mm Bullet Shape Created Sapphire Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07344/medium/RIGTXR07344-EM-WG-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07344/medium/RIGTXR07344-EM-WG-WH-300-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-2-3-ctw-oval-lab-grown-diamond-side-stone-engagement-ring-platinum/pid/RIGKSR6170-PL3?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 5 2/3 ctw Oval Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6170/medium/RIGKSR6170-WG-OV-WH-500-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGKSR6170/medium/RIGKSR6170-WG-OV-WH-500-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-3-4-ctw-round-lab-grown-diamond-double-scalloped-halo-engagement-ring-platinum/pid/RIGTXR06195-PL4?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>3 3/4 ctw Round Lab Grown Diamond Double Scalloped Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06195/medium/RIGTXR06195-WG-RB-WH-374-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06195/medium/RIGTXR06195-WG-RB-WH-374-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-3-ctw-round-lab-grown-diamond-petite-pave-engagement-ring-with-side-accents-platinum/pid/RIGTXR05852RD3308-PL4?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>3 1/3 ctw Round Lab Grown Diamond Petite Pave Engagement Ring with Side Accents</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05852/medium/RIGTXR05852-WG-RB-WH-3308-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05852/medium/RIGTXR05852-WG-RB-WH-3308-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-7-8-ctw-oval-lab-grown-diamond-double-band-solitaire-engagement-ring-with-side-accents-14k-yellow-gold/pid/RIGYR4393LEC-GY4?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>2 7/8 ctw Oval Lab Grown Diamond Double Band Solitaire Engagement Ring with Side Accents</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR4393LEC/medium/RIGYR4393LEC-YG-OV-WH-281-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGYR4393LEC/medium/RIGYR4393LEC-YG-OV-WH-281-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-7-8-ctw-pear-lab-grown-diamond-fancy-pink-split-shank-solitaire-engagement-ring-with-side-accents/pid/RIGTXR05879-PN-GW4?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>1 7/8 ctw Pear Lab Grown Diamond Fancy Pink Split Shank Solitaire Engagement Ring with Side Accents</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05879/medium/RIGTXR05879-WG-PE-PN-183-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05879/medium/RIGTXR05879-WG-PE-PN-183-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-oval-lab-grown-diamond-fancy-pink-framed-halo-engagement-ring/pid/RIGTXR05870-PN-GW4?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Oval Lab Grown Diamond Fancy Pink Framed Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr"/>
+      <c r="D129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-3-8-ctw-emerald-lab-grown-diamond-double-prong-engagement-ring-18k-yellow-gold/pid/RIGJRZ76970E-PL_5?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 3 3/8 ctw Emerald Lab Grown Diamond Double Prong Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76970E/medium/RIGJRZ76970E-WG-RB-WH-338-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76970E/medium/RIGJRZ76970E-WG-RB-WH-338-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-1-2-ctw-round-lab-grown-diamond-engagement-ring-18k-yellow-gold/pid/RIGJRZ76960S-PL_5?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 5 1/2 ctw Round Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76960S/medium/RIGJRZ76960S-WG-RB-WH-560-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76960S/medium/RIGJRZ76960S-WG-RB-WH-560-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-1-2-ctw-round-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ76560E-PL_5?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 4 1/2 ctw Round Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76560E%20/medium/RIGJRZ76560E%20-WG-RB-WH-427-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76560E%20/medium/RIGJRZ76560E%20-WG-RB-WH-427-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-4-ctw-cushion-lab-grown-diamond-hidden-halo-engagement-ring-18k-yellow-gold/pid/RIGJRZ76330H-PL_5?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 4 ctw Cushion Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76330H/medium/RIGJRZ76330H-WG-RB-WH-414-M0-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76330H/medium/RIGJRZ76330H-WG-RB-WH-414-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76330H/medium/RIGJRZ76330H-HW27-M4.png, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-6-1-2-ctw-round-lab-grown-diamond-double-prong-engagement-ring-18k-yellow-gold/pid/RIGJRD02200Q-PL_5?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 6 1/2 ctw Round Lab Grown Diamond Double Prong Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02200Q/medium/RIGJRD02200Q-WG-RB-WH-628-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02200Q/medium/RIGJRD02200Q-WG-RB-WH-628-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-5-1-10-ctw-emerald-lab-grown-diamond-double-prong-engagement-ring-18k-rose-gold/pid/RIGJRD02210Q-PL11?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Near-Colorless 5 1/10 ctw Emerald Lab Grown Diamond Double Prong Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02210Q/medium/RIGJRD02210Q-WG-RB-WH-511-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD02210Q/medium/RIGJRD02210Q-WG-RB-WH-511-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-1-3-ctw-round-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ76580S-HW_5?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 5 1/3 ctw Round Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76580S%20/medium/RIGJRZ76580S%20-WG-VR-WH-565-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76580S%20/medium/RIGJRZ76580S%20-WG-VR-WH-565-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-4-ctw-heart-lab-grown-diamond-pave-engagement-ring-14k-rose-gold/pid/RIG0889X2-H150SO-GS?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>2 1/4 ctw Heart Lab Grown Diamond Pave Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00889H200SOX3/medium/TXR00889H200SOX3-RG-HT-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00889H200SOX3/medium/TXR00889H200SOX3-RG-HT-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-HE.jpg</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-ctw-emerald-lab-grown-diamond-pave-halo-engagement-ring-14k-white-gold/pid/RIG0889X4-E200H1-GW?algoliaQueryId=d9d350048211773493f5aa7688aae96b</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>3 ctw Emerald Lab Grown Diamond Pave Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00889E200H1X5/medium/TXR00889E200H1X5-WG-EM-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00889E200H1X5/medium/TXR00889E200H1X5-WG-EM-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-5-ctw-princess-lab-grown-diamond-petite-bow-halo-engagement-ring-14k-white-gold/pid/RIG0891X4-P150H1-GW?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2 1/5 ctw Princess Lab Grown Diamond Petite Bow Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00891P200H1X5/medium/TXR00891P200H1X5-WG-PR-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00891P200H1X5/medium/TXR00891P200H1X5-WG-PR-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-2-ctw-fancy-yellow-oval-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGJOR7031-YL-GW4?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>4 1/2 ctw Fancy Yellow Oval Lab Grown Diamond Three-Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGDJOR7031O390/medium/LGDJOR7031O390-GT87.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGDJOR7031O390GT87/medium/LGDJOR7031O390GT87-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJOR7031/medium/RIGJOR7031-YL-GW4-new.jpg</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-8-ctw-round-lab-grown-diamond-old-mine-cut-art-deco-side-stone-engagement-ring-platinum/pid/RIGRVR06498-PL1?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>4 1/8 ctw Round Lab Grown Diamond Old Mine Cut Art Deco Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06498/medium/RIGRVR06498-WG-RB-410N-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06498/medium/RIGRVR06498-WG-RB-410N-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06498/medium/RIGRVR06498-PL4.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-10-ctw-round-lab-grown-diamond-eternity-solitaire-engagement-ring-platinum/pid/RIGR05633R20PL1700?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>4 1/10 ctw Round Lab Grown Diamond Eternity Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05633/medium/RIGTXR05633-WG-RB-WH-414-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05633/medium/RIGTXR05633-WG-RB-WH-414-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05633RB2.0/medium/RIGTXR05633RB2.0-GW4-4.50-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-round-lab-grown-diamond-old-mine-cut-filigree-side-stone-engagement-ring-14k-white-gold/pid/RIGRVR06499-GW2?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Round Lab Grown Diamond Old Mine Cut Filigree Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06499/medium/RIGRVR06499-WG-RB-350N-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06499/medium/RIGRVR06499-WG-RB-350N-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-5-8-ctw-cushion-lab-grown-diamond-old-mine-cut-side-stone-engagement-ring-in-french-pave-setting-14k-yellow-gold/pid/RIGRVR06508-GY4?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>3 5/8 ctw Cushion Lab Grown Diamond Old Mine Cut Side Stone Engagement Ring in French Pave Setting</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06508/medium/RIGRVR06508-YG-CU-368-M0_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06508/medium/RIGRVR06508-YG-CU-368-M1_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-round-lab-grown-diamond-old-mine-cut-in-micro-pave-setting-side-stone-engagement-ring-14k-white-gold/pid/RIGRVR06501-GW4?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Round Lab Grown Diamond Old Mine Cut in Micro Pave Setting Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06501/medium/RIGRVR06501-WG-RB-360N-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06501/medium/RIGRVR06501-WG-RB-360R-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/6-7-8-ctw-oval-lab-grown-diamond-three-stone-engagement-ring-with-trillion-side-stones-platinum/pid/RIGTXR06002O5.0PL2?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>6 7/8 ctw Oval Lab Grown Diamond Three-Stone Engagement Ring with Trillion side stones</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06002/medium/RIGTXR06002-WG-OV-WH-683-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06002/medium/RIGTXR06002-WG-OV-WH-683-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-3-ctw-oval-lab-grown-diamond-engagement-ring-with-oval-side-accents-platinum/pid/RIG0893X3O200SOPL2?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>2 1/3 ctw Oval Lab Grown Diamond Engagement Ring with Oval Side Accents</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00893O200SOX3/medium/TXR00893O200SOX3-WG-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00893O200SOX3/medium/TXR00893O200SOX3-WG-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-3-4-ctw-fancy-blue-oval-lab-grown-diamond-side-stone-engagement-ring-14k-yellow-gold/pid/RIGTXR09151-BL-GY4?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>2 3/4 ctw Fancy Blue Oval Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09151B/medium/RIGTXR09151B-YG-OV-WH-275-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09151B/medium/RIGTXR09151B-YG-OV-WH-275-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09151/medium/RIGTXR09151-BL-YL-PN%20alt%20image.jpg</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-fancy-pink-pear-lab-grown-diamond-three-stone-engagement-ring-platinum/pid/RIGTXR09154-PN-PL4?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Fancy Pink Pear Lab Grown Diamond Three Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09154P/medium/RIGTXR09154P-WG-PE-WH-250-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09154P/medium/RIGTXR09154P-WG-PE-WH-250-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09154/medium/RIGTXR09154-BL-YL-PN.jpg</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-3-4-ctw-fancy-yellow-emerald-lab-grown-diamond-split-shank-side-stone-engagement-ring-platinum/pid/RIGTXR09155-YL-PL4?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>2 3/4 ctw Fancy Yellow Emerald Lab Grown Diamond Split Shank Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09155Y/medium/RIGTXR09155Y-WG-EM-WH-277-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09155Y/medium/RIGTXR09155Y-WG-EM-WH-277-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09155/medium/RIGTXR09155-BL-YL-PN.jpg</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-solitaire-engagement-ring-14k-white-gold/pid/RGTXR06203RB1.0GW2?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>1 ctw Round Lab Grown Diamond Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06203/medium/RIGTXR06203-WG-RB-WH-100-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06203/medium/RIGTXR06203-WG-RB-WH-100-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-2-5-ctw-fancy-yellow-pear-lab-grown-diamond-split-shank-side-stone-engagement-ring-platinum/pid/RIGTXR09162-YL-PL4?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>2 2/5 ctw Fancy Yellow Pear Lab Grown Diamond Split Shank Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09162Y/medium/RIGTXR09162Y-WG-PE-WH-240-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09162Y/medium/RIGTXR09162Y-WG-PE-WH-240-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09162/medium/RIGTXR09162-BL-YL-PN.jpg</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/10-1-5-ctw-oval-lab-grown-diamond-eternity-side-stone-engagement-ring-platinum/pid/RIGTXR06852-500OEPL4-4.75?algoliaQueryId=89486efaee9e0e22a190e26f158e16a2</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>10 1/5 ctw Oval Lab Grown Diamond Eternity Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06852/medium/RIGTXR06852-WG-OV-WH-980-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06852/medium/RIGTXR06852-WG-OV-WH-980-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-6-ctw-emerald-lab-grown-diamond-side-stone-engagement-ring-platinum/pid/RIGTXR07510-PL4?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>3 1/6 ctw Emerald Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07510/medium/TXR07510-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR07510/medium/TXR07510-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/11x9-mm-cushion-cut-created-sapphire-and-1-1-4-ctw-baguette-lab-grown-diamond-side-stone-engagement-ring-platinum/pid/RIGTXR07346-SP-PL4?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>11x9 mm Cushion Cut Created Sapphire and 1 1/4 ctw Baguette Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07346/medium/RIGTXR07346-CU-SP-WG-WH-124-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07346/medium/RIGTXR07346-CU-SP-WG-WH-124-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/6-1-5-ctw-old-mine-cut-lab-grown-diamond-hidden-halo-engagement-ring-14k-white-gold/pid/RIGTXR06811-GW4?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>6 1/5 ctw Old Mine Cut Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06811/medium/RIGTXR06811-WG-CU-WH-639-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06811/medium/RIGTXR06811-WG-CU-WH-639-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-3-4-ctw-emerald-lab-grown-diamond-channel-band-halo-engagement-ring-18k-yellow-gold/pid/RIGJRZ760707-PL_5?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 3 3/4 ctw Emerald Lab Grown Diamond Channel Band Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ760707/medium/RIGJRZ760707-WG-RB-WH-380-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ760707/medium/RIGJRZ760707-WG-RB-WH-380-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76050H/medium/RIGJRZ76050H-HW_5-shape.jpg</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-3-7-8-ctw-cushion-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ76190E-PL4?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Near-Colorless 3 7/8 ctw Cushion Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76190E%20/medium/RIGJRZ76190E%20-WG-VR-WH-406-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ76190E%20/medium/RIGJRZ76190E%20-WG-VR-WH-406-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-emerald-lab-grown-diamond-framed-engagement-ring-18k-rose-gold/pid/RIGJRZ75713E-PL19?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Emerald Lab Grown Diamond Framed Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ75713E/medium/RIGJRZ75713E-WG-RB-WH-353-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ75713E/medium/RIGJRZ75713E-WG-RB-WH-353-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-tapered-baguette-halo-engagement-ring-14k-white-gold/pid/RIG0617X4-T200H1-GW?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Radiant Lab Grown Diamond Tapered Baguette Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00617T200H1X5/medium/TXR00617T200H1X5-WG-RD-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00617T200H1X5/medium/TXR00617T200H1X5-WG-RD-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-2-3-ctw-radiant-lab-grown-diamond-vine-halo-engagement-ring-14k-white-gold/pid/RIG0887X4-T200H1-GW?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>2 2/3 ctw Radiant Lab Grown Diamond Vine Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00887T200H1X5/medium/TXR00887T200H1X5-WG-RD-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/TXR00887T200H1X5/medium/TXR00887T200H1X5-WG-RD-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-oval-lab-grown-diamond-halo-engagement-ring-14k-white-gold/pid/RIGAJR02421-GW1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Oval Lab Grown Diamond Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/AJR02421/medium/AJR02421-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/AJR02421/medium/AJR02421-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/5-1-5-ctw-princess-lab-grown-diamond-three-stone-engagement-ring-14k-white-gold/pid/RIGRVR09419-GW1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>5 1/5 ctw Princess Lab Grown Diamond Three-Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09419/medium/RVR09419-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09419/medium/RVR09419-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/6-1-3-ctw-round-emerald-lab-grown-diamond-eternity-engagement-ring-14k-white-gold/pid/RIGRVR05525GW1-900?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>6 1/3 ctw Round &amp; Emerald Lab Grown Diamond Eternity Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05525/medium/RIGRVR05525-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05525/medium/RIGRVR05525-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/7-1-8-ctw-round-lab-grown-diamond-eternity-engagement-ring-platinum/pid/RIGRVR09619PL1-800?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>7 1/8 ctw Round Lab Grown Diamond Eternity Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09619/medium/RVR09619-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09619/medium/RVR09619-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-4-ctw-radiant-lab-grown-diamond-side-stone-engagement-ring-14k-white-gold/pid/RIGRVR6186-GW1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>3 1/4 ctw Radiant Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06186/medium/RIGRVR06186-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06186/medium/RIGRVR06186-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-10-ctw-pear-lab-grown-diamond-and-1-20-mm-round-created-sapphire-side-stone-engagement-ring-14k-white-gold/pid/RIGRVR02610-GW1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>2 1/10 ctw Pear Lab Grown Diamond and 1.20 mm Round Created Sapphire Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02610/medium/RIGRVR02610-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR02610/medium/RIGRVR02610-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-5-ctw-oval-lab-grown-diamond-side-stone-engagement-ring-14k-yellow-gold/pid/RIGRVR01554-GY1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>4 1/5 ctw Oval Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR01554/medium/RIGRVR01554-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR01554/medium/RIGRVR01554-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-ctw-cushion-lab-grown-diamond-solitaire-engagement-ring-14k-yellow-gold/pid/RIGTXR08515-GW1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>3 ctw Cushion Lab Grown Diamond Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08515/medium/RIGTXR08515-YG-M0-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08515/medium/RIGTXR08515-YG-M1-1.jpg</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-60x2-20-mm-created-pear-shape-emerald-and-2-1-5-ctw-pear-lab-grown-diamond-side-stone-engagement-ring18k-white-gold/pid/RIGRVR04183-HW1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>3.60x2.20 mm Created Pear Shape Emerald and 2 1/5 ctw Pear Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04183/medium/RIGRVR04183-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04183/medium/RIGRVR04183-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-round-lab-grown-diamond-and-1-20-mm-marquise-created-emerald-side-stone-engagement-ring-14k-yellow-gold/pid/RIGRVR07781-GY1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Round Lab Grown Diamond and 1.20 mm Marquise Created Emerald Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR07781/medium/RIGRVR07781-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR07781/medium/RIGRVR07781-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-2-5-ctw-dutch-marquise-lab-grown-diamond-side-stone-engagement-ring-14k-yellow-gold/pid/RIGAJR02294-GY1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>2 2/5 ctw Dutch Marquise Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/AJR02294/medium/AJR02294-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/AJR02294/medium/AJR02294-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-ctw-dutch-marquise-lab-grown-diamond-side-stone-engagement-ring-14k-white-gold/pid/RIGAJR01567-GW1?algoliaQueryId=101f3c002f7b9b9ff310f398a631b859</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>3 ctw Dutch Marquise Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/R10/medium/R10-AJR01567-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/R10/medium/R10-AJR01567-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-1-5-ctw-princess-lab-grown-diamond-split-shank-halo-engagement-ring-14k-white-gold/pid/RIG0625X2-P075H1-GW?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>1 1/5 ctw Princess Lab Grown Diamond Split Shank Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X2/medium/RIG0625X2-P075H1-GW_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X2/medium/RIG0625X2-P075H1-GW_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X4/medium/RIG0625X4-P150H1-GW-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-ctw-round-lab-grown-diamond-double-twist-engagement-ring-14k-white-gold/pid/RIG0629X1-R075SO-GW?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>1 ctw Round Lab Grown Diamond Double Twist Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0629X1/medium/RIG0629X1-R075SO-GW-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0629X1/medium/RIG0629X1-R075SO-GW-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0629X1R075SOGW4/medium/LGR0629X1R075SOGW4-new2-img.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/0629/medium/0629-Round-GB.jpg</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-radiant-lab-grown-diamond-station-engagement-ring-14k-white-gold/pid/RIG1860X3-T200SO-GW?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Radiant Lab Grown Diamond Station Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X3/medium/RIG1860X3-T200SO-GW-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X3/medium/RIG1860X3-T200SO-GW-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X1/medium/RIG1860X1-T075SO-GW-1-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG1860X3/medium/RIG1860X3-Radiant-GW.jpg</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-engagement-ring-platinum/pid/RIGJRD020837-PL_5?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>5 ctw Emerald Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD020837/medium/RIGJRD020837-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD020837/medium/RIGJRD020837-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD020837/medium/RIGJRD020837-PL_5-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-2-5-ctw-oval-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR07400O300GW4?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>4 2/5 ctw Oval Lab Grown Diamond Bridal Set</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07400O300/medium/BRDTXR07400O300-WG-OV-WH-439-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07400O300/medium/BRDTXR07400O300-WG-OV-WH-439-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR07400O300GW4/medium/BRDTXR07400O300GW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-6-7-8-ctw-emerald-lab-grown-diamond-engagement-ring-18k-rose-gold/pid/RIGJRZ7731XX-PL4?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Near-Colorless 6 7/8 ctw Emerald Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7731XX/medium/RIGJRZ7731XX-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7731XX/medium/RIGJRZ7731XX-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ7731XX/medium/RIGJRZ7731XX-HW_5-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-near-colorless-3-1-2-ctw-round-lab-grown-diamond-engagement-ring-18k-white-gold/pid/RIGJRZ78940H-HW4?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Near-Colorless 3 1/2 ctw Round Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ78940H/medium/RIGJRZ78940H-HW_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ78940H/medium/RIGJRZ78940H-HW_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRZ78940H/medium/RIGJRZ78940H-HW_5-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-graduated-engagement-ring-14k-white-gold/pid/RIG0641X2-R150SO-GW?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>2 ctw Round Lab Grown Diamond Graduated Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0641X2/medium/RIG0641X2-R150SO-GW_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0641X2/medium/RIG0641X2-R150SO-GW_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0641X2/medium/RIG0641X2-R150SO-GW-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/LGR0589X3/medium/LGR0589X3-R200-shape.jpg</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/8-1-4-ctw-radiant-lab-grown-diamond-bridal-set-platinum/pid/BRDTXR08803T500PL2?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>8 1/4 ctw Radiant Lab Grown Diamond Bridal Set</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08803T500/medium/BRDTXR08803T500-WG-RD-WH-816-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08803T500/medium/BRDTXR08803T500-WG-RD-WH-816-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RA.jpg</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-5-2-5-ctw-round-lab-grown-diamond-hidden-halo-engagement-ring-18k-white-gold/pid/RIGTX06766R500-HW1?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 5 2/5 ctw Round Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06766R500/medium/RIGTXR06766R500-WG-RB-WH-543-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06766R500/medium/RIGTXR06766R500-WG-RB-WH-543-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTX06766R500/medium/RIGTX06766R500-GW6-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-ctw-round-lab-grown-diamond-three-stone-ring-18k-white-gold/pid/RIGJRD0315-HW4?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>4 ctw Round Lab Grown Diamond Three-Stone Ring</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0315/medium/RIGJRD0315-HW4_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0315/medium/RIGJRD0315-HW4_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0315/medium/RIGJRD0315-HW4-new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-ctw-oval-lab-grown-diamond-petite-solitaire-engagement-ring-14k-white-gold/pid/RGTXR05314O300-GW2?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>3 ctw Oval Lab Grown Diamond Petite Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05314/medium/RIGTXR05314-WG-OV-WH-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05314O300/medium/RIGTXR05314O300-GY4-1-NEW.jpg</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/6-2-3-ctw-round-lab-grown-diamond-bridal-set-14k-white-gold/pid/BRDTXR08527-GW2?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>6 2/3 ctw Round Lab Grown Diamond Bridal Set</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08527/medium/BRDTXR08527-WG-RB-WH-665-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BRDTXR08527/medium/BRDTXR08527-WG-RB-WH-665-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/8-2-3-ctw-pear-lab-grown-diamond-hidden-halo-engagement-ring-14k-yellow-gold/pid/RIGTX04156D800-GY1?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>8 2/3 ctw Pear Lab Grown Diamond Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04156D300/medium/RIGTXR04156D300-YG-PE-WH-352-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR04156D300/medium/RIGTXR04156D300-YG-PE-WH-352-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr"/>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/5-1-2-ctw-emerald-lab-grown-diamond-three-stone-ring-platinum/pid/RIGJRD0254XX-PL_5?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>5 1/2  ctw Emerald Lab Grown Diamond Three-Stone Ring</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0254XX/medium/RIGJRD0254XX-PL_5_1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0254XX/medium/RIGJRD0254XX-PL_5_2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGJRD0254/medium/RIGJRD0254-HW_5-new-IMG.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr"/>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-ctw-toi-et-moi-pear-and-emerald-engagement-ring-14k-yellow-gold/pid/RIGTXR05973PE40GY1?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>4 ctw Toi Et Moi Pear and Emerald Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05973/medium/RIGTXR05973-YG-VR-WH-400-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05973/medium/RIGTXR05973-YG-VR-WH-400-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05973PE40/medium/RIGTXR05973PE40-GW4-new.jpg</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr"/>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/9-ctw-pear-lab-grown-diamond-engagement-ring-with-split-prong-side-accents-platinum/pid/RIGRV04550D800-PL1?algoliaQueryId=7f3db39354dee3af8538a3c641f2139d</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>9 ctw Pear Lab Grown Diamond Engagement Ring with Split Prong Side Accents</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04550D800/medium/RIGRVR04550D800-WG-PE-WH-900-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR04550D800/medium/RIGRVR04550D800-WG-PE-WH-900-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PE.jpg</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr"/>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-2-ctw-round-lab-grown-diamond-engagement-ring-platinum/pid/RIGRVR01656-PL2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>4 1/2 ctw Round Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR01656/medium/RIGRVR01656-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR01656/medium/RIGRVR01656-WG-M3.jpg</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr"/>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-7-8-ctw-round-lab-grown-diamond-engagement-ring-14k-rose-gold/pid/RIGRVR00790-GP2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>1 7/8 ctw Round Lab Grown Diamond Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00790/medium/RIGRVR00790-RG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00790/medium/RIGRVR00790-RG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr"/>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-3-8-ctw-lab-grown-diamond-round-shape-engagement-ring-14k-yellow-gold/pid/RIGRVR00485-GY2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>3 3/8 ctw Lab Grown Diamond Round Shape Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00485/medium/RIGRVR00485-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00485/medium/RIGRVR00485-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr"/>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-3-4-ctw-emerald-lab-grown-diamond-two-stone-solitaire-engagement-ring-14k-yellow-gold/pid/RIGTXR09509-GY2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>2 3/4 ctw Emerald Lab Grown Diamond Two Stone Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09509/medium/RIGTXR09509-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR09509/medium/RIGTXR09509-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr"/>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-three-stone-engagement-ring-14k-yellow-gold/pid/RIGRVR09438-GY2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>5 ctw Emerald Lab Grown Diamond Three Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09438/medium/RVR09438-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09438/medium/RVR09438-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr"/>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/5-ctw-emerald-lab-grown-diamond-solitaire-engagement-ring-18k-white-gold/pid/RIGRVR09411-HW2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>5 ctw Emerald Lab Grown Diamond Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09411/medium/RVR09411-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09411/medium/RVR09411-WG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr"/>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-2-ctw-emerald-lab-grown-diamond-side-stone-engagement-ring-14k-yellow-gold/pid/RIGRVR09259-GY2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>4 1/2 ctw Emerald Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09259/medium/RVR09259-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RVR09259/medium/RVR09259-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr"/>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-elongated-cushion-lab-grown-diamond-side-stone-engagement-ring-14k-white-gold/pid/RIGRVR08158-GW2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Elongated Cushion Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR08158/medium/RIGRVR08158-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR08158/medium/RIGRVR08158-WG-M3.jpg</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-2-ctw-oval-lab-grown-diamond-solitaire-engagement-ring-14k-two-tone-white-yellow-gold/pid/RIGRVR07654-GWY2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>3 1/2 ctw Oval Lab Grown Diamond Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR07654/medium/RIGRVR07654-WY-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR07654/medium/RIGRVR07654-WY-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr"/>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-5-ctw-oval-lab-grown-diamond-side-stone-engagement-ring-14k-two-tone-white-yellow-gold/pid/RIGRVR07433-GWY2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>3 1/5 ctw Oval Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR07433/medium/RIGRVR07433-WY-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR07433/medium/RIGRVR07433-WY-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr"/>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-ctw-oval-lab-grown-diamond-solitaire-engagement-ring-14k-yellow-gold/pid/RIGRVR06791-GY2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>2 ctw Oval Lab Grown Diamond  Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06791/medium/RIGRVR06791-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06791/medium/RIGRVR06791-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr"/>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-2-5-ctw-oval-lab-grown-diamond-side-stone-engagement-ring-14k-yellow-gold/pid/RIGRVR01393-GY2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>2 2/5 ctw Oval Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR01393/medium/RIGRVR01393-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR01393/medium/RIGRVR01393-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr"/>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-ctw-marquise-lab-grown-diamond-side-stone-engagement-ring-18k-white-gold/pid/RIGRVR00786-HW2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>4 ctw Marquise Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00786/medium/RIGRVR00786-WG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00786/medium/RIGRVR00786-WG-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00786/medium/RIGRVR00786-WG-M3.jpg</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr"/>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-marquise-lab-grown-diamond-bezel-setting-solitaire-engagement-ring-14k-yellow-gold/pid/RIGAJR02001-GY2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Marquise Lab Grown Diamond Bezel Setting Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/AJR02001/medium/AJR02001-YG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/AJR02001/medium/AJR02001-YG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/10-ctw-round-lab-grown-diamond-solitaire-engagement-ring-14k-rose-gold/pid/RIGAJR00204-GP2?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>10 ctw Round Lab Grown Diamond Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/AJR00204/medium/AJR00204-RG-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/AJR00204/medium/AJR00204-RG-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr"/>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/8-1-6-ctw-lab-grown-diamond-solitaire-engagement-ring-18k-white-gold/pid/RIGR001BL558HW3-ST?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>8 1/6 ctw Lab Grown Diamond Solitaire Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr"/>
+      <c r="D206" t="inlineStr"/>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-2-3-ctw-emerald-lab-grown-diamond-nature-inspired-side-stone-engagement-ring-platinum/pid/RIGAJR01219-PL1?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>4 2/3 ctw Emerald Lab Grown Diamond Nature Inspired Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01219/medium/RIGAJR01219-WG-VR-460-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01219/medium/RIGAJR01219-WG-VR-460-M3.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/6-3-8-ctw-fancy-yellow-east-west-radiant-engagement-ring-with-princess-and-baguette-side-stones-14k-two-tone-white-and-yellow-gold/pid/RIGAJR01077YL-GWY4?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>6 3/8 ctw Fancy Yellow East West Radiant Engagement Ring with Princess and Baguette Side Stones</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01077TY/medium/RIGAJR01077TY-YW-VR-638-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01077TY/medium/RIGAJR01077TY-YW-VR-638-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/8-ctw-fancy-yellow-emerald-lab-grown-diamond-side-by-side-two-stone-engagement-ring-14k-two-tone-white-and-yellow-gold/pid/RIGAJ01074EYL-GWY4?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>8 ctw Fancy Yellow Emerald Lab Grown Diamond Side by Side Two Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01074EY/medium/RIGAJR01074EY-YW-EM-800-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01074EY/medium/RIGAJR01074EY-YW-EM-800-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/6-ctw-fancy-blue-pear-lab-grown-diamond-bypass-two-stone-engagement-ring-14k-white-gold/pid/RIGAJR01072BL-GW4?algoliaQueryId=4754dac7d40108a1c89d9e1e6a7c0bd5</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>6 ctw Fancy Blue Pear Lab Grown Diamond Bypass Two Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01072DB/medium/RIGAJR01072DB-WG-PE-600-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01072DB/medium/RIGAJR01072DB-WG-PE-600-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/8-ctw-fancy-blue-oval-lab-grown-diamond-double-band-side-stone-engagement-ring-14k-white-gold/pid/RIGAJR01079OBL-GW4?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>8 ctw Fancy Blue Oval Lab Grown Diamond Double Band Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01079OB/medium/RIGAJR01079OB-WG-VR-802-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01079OB/medium/RIGAJR01079OB-WG-VR-802-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/5-3-4-ctw-fancy-yellow-emerald-lab-grown-diamond-cobble-stone-baguette-engagement-ring-14k-two-tone-white-and-yellow-gold/pid/RIGAJ01078EYL-GWY4?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>5 3/4 ctw Fancy Yellow Emerald Lab Grown Diamond Cobble Stone Baguette Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01078EY/medium/RIGAJR01078EY-YW-VR-572-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01078EY/medium/RIGAJR01078EY-YW-VR-572-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-8-ctw-princess-lab-grown-diamond-pave-profile-side-stone-engagement-ring-platinum/pid/RIGAJ01023P300-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>4 1/8 ctw Princess Lab Grown Diamond Pave Profile Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01023P200/medium/RIGAJR01023P200-WG-PR-310-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01023P200/medium/RIGAJR01023P200-WG-PR-310-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-PR.jpg</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-2-ctw-oval-lab-grown-diamond-profile-side-stone-engagement-ring-platinum/pid/RIGAJ01022O300-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>4 1/2 ctw Oval Lab Grown Diamond Profile Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01022O300/medium/RIGAJR01022O300-WG-VR-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAJR01022O300/medium/RIGAJR01022O300-WG-VR-300-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-and-6-0x3-8-mm-pear-shape-created-emerald-side-stone-engagement-ring-platinum/pid/RIGTX07342CU-EMPL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>3 ctw Round Lab Grown Diamond and 6.0x3.8 mm Pear Shape Created Emerald Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07342EG/medium/RIGTXR07342EG-WG-VR-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07342EG/medium/RIGTXR07342EG-WG-VR-300-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-ctw-oval-lab-grown-diamond-and-7-2x5-1-mm-oval-created-emerald-three-stone-hidden-halo-engagement-ring-platinum/pid/RIG07350-OV2-EMPL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>2 ctw Oval Lab Grown Diamond and 7.2x5.1 mm Oval Created Emerald Three-Stone Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07350EG/medium/RIGTXR07350EG-WG-OV-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07350EG/medium/RIGTXR07350EG-WG-OV-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG07350/medium/RIG07350-OV2-EMGW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-ctw-round-lab-grown-diamond-and-7-2-mm-round-shape-created-emerald-three-stone-engagement-ring-platinum/pid/RIGTX07347RD-EMPL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>3 ctw Round Lab Grown Diamond and 7.2 mm Round Shape Created Emerald Three-Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07347EG/medium/RIGTXR07347EG-WG-RB-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07347EG/medium/RIGTXR07347EG-WG-RB-300-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-round-lab-grown-diamond-twist-shank-hidden-halo-engagement-ring-platinum/pid/RIGRVR05422R200PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Round Lab Grown Diamond Twist Shank Hidden Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05422R200/medium/RIGRVR05422R200-WG-RB-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05422R200/medium/RIGRVR05422R200-WG-RB-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-3-ctw-round-lab-grown-diamond-vintage-inspired-old-mine-cut-edwardian-style-knife-edge-engagement-ring-platinum/pid/RIGRV05672R200-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>2 1/3 ctw Round Lab Grown Diamond Vintage Inspired Old Mine Cut Edwardian Style Knife Edge Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05672R200/medium/RIGRVR05672R200-WG-230N-RB-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05672R200/medium/RIGRVR05672R200-WG-230N-RB-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRV05672R200/medium/RIGRV05672R200-GW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-1-2-ctw-round-lab-grown-diamond-vintage-inspired-old-mine-cut-edwardian-style-engagement-ring-platinum/pid/RIGRVR05660-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>2 1/2 ctw Round Lab Grown Diamond Vintage Inspired Old Mine Cut Edwardian Style Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05660/medium/RIGRVR05660-WG-250N-RB-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05660/medium/RIGRVR05660-WG-250N-RB-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05660/medium/RIGRVR05660-GW4-NEW.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/4-1-5-ctw-cushion-lab-grown-diamond-vintage-inspired-engagement-ring-platinum/pid/RIGRVR05018-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>4 1/5 ctw Cushion Lab Grown Diamond Vintage Inspired Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05018/medium/RIGRVR05018-WG-422N-VR-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR05018/medium/RIGRVR05018-WG-422N-VR-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-1-3-ctw-cushion-lab-grown-diamond-old-mine-cut-engagement-ring-with-side-step-baguettes-platinum/pid/RIGRVR06507-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>3 1/3 ctw Cushion Lab Grown Diamond Old Mine Cut Engagement Ring with Side Step Baguettes</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06507/medium/RIGRVR06507-WG-CU-338-M0_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06507/medium/RIGRVR06507-WG-CU-338-M1_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-ctw-cushion-lab-grown-diamond-old-mine-cut-halo-engagement-ring-platinum/pid/RIGRVR06505-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>3 ctw Cushion Lab Grown Diamond Old Mine Cut Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06505/medium/RIGRVR06505-WG-CU-300-M0_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06505/medium/RIGRVR06505-PL4.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06505/medium/RIGRVR06505-WG-CU-300-M1_new.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-CU.jpg</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-ctw-round-lab-grown-diamond-old-mine-cut-milgrain-halo-engagement-ring-platinum/pid/RIGRVR06502-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>2 ctw Round Lab Grown Diamond Old Mine Cut Milgrain Halo Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06502/medium/RIGRVR06502-WG-RB-216N-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06502/medium/RIGRVR06502-WG-RB-216N-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-2-3-ctw-round-lab-grown-diamond-old-mine-cut-engagement-ring-with-baguette-side-stones-platinum/pid/RIGRVR06500-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>3 2/3 ctw Round Lab Grown Diamond Old Mine Cut Engagement Ring with Baguette Side Stones</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06500/medium/RIGRVR06500-WG-RB-337N-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR06500/medium/RIGRVR06500-WG-RB-337N-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-RD.jpg</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/3-ctw-radiant-lab-grown-diamond-and-5-5x3-3x2-2-mm-trapezoid-created-emerald-three-stone-ring-platinum/pid/RIG07696EM-RA3-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>3 ctw Radiant Lab Grown Diamond and 5.5x3.3x2.2 mm Trapezoid Created Emerald Three-Stone Ring</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07696EG/medium/RIGTXR07696EG-WG-VR-300-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07696EG/medium/RIGTXR07696EG-WG-VR-300-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/5-3-4-ctw-elongated-cushion-lab-grown-diamond-side-stone-engagement-ring-platinum/pid/RIGTXR08656Z500PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>5 3/4 ctw Elongated Cushion Lab Grown Diamond Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08656Z500/medium/RIGTXR08656Z500-WG-CU-WH-569-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR08656Z500/medium/RIGTXR08656Z500-WG-CU-WH-569-M1.jpg</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/1-7-8-ctw-marquise-lab-grown-diamond-east-west-side-stone-engagement-ring-platinum/pid/RIGRVR00294-PL1?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>1 7/8 ctw Marquise Lab Grown Diamond East-West Side Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00294/medium/RIGRVR00294-WG-MQ-WH-192-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGRVR00294/medium/RIGRVR00294-WG-MQ-WH-192-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-MQ.jpg</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/boundless-trio-14k-white-gold/pid/BORIGAAR02547M-GW4?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Boundless Trio</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAAR02547M/medium/RIGAAR02547M-WG-RB-300-M0-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAAR02547M/medium/RIGAAR02547M-WG-RB-300-M1-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BORIGAAR02547M/medium/BORIGAAR02547M-GW4-1.jpg</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/boundless-bridal-duo-14k-white-gold/pid/BORIGAR01616QS-GW4?algoliaQueryId=b08c91b19d3c27f407010167382bb7b7</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Boundless Bridal Duo</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAAR01616QS/medium/RIGAAR01616QS-WG-RB-385-M0-1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGAAR01616QS/medium/RIGAAR01616QS-WG-RB-385-M1-2.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/BORIGAR01616QS/medium/BORIGAR01616QS-GW4-1.jpg</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-8-ctw-asscher-lab-grown-diamond-solitaire-engagement-ring-with-side-accents-platinum/pid/RIGTXR07092PL1?algoliaQueryId=68065bb4a294cbc975a72f30ef8e7bf8</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 8 ctw Asscher Lab Grown Diamond Solitaire Engagement Ring with Side Accents</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07092/medium/RIGTXR07092-WG-AS-WH-749-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR07092/medium/RIGTXR07092-WG-AS-WH-749-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-AS.jpg</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/badgley-mischka-colorless-3-3-4-ctw-emerald-lab-grown-diamond-halo-bypass-engagement-ring-platinum/pid/RIGTXR06526-PL1?algoliaQueryId=68065bb4a294cbc975a72f30ef8e7bf8</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Badgley Mischka Colorless 3 3/4 ctw Emerald Lab Grown Diamond Halo Bypass Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06526/medium/RIGTXR06526-WG-EM-WH-377-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR06526/medium/RIGTXR06526-WG-EM-WH-377-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-EM.jpg</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>https://www.grownbrilliance.com/2-ctw-oval-fancy-blue-lab-grown-diamond-framed-three-stone-engagement-ring-14k-two-tone-white-and-yellow-gold/pid/RIGTXR05872BL-GWY4?algoliaQueryId=68065bb4a294cbc975a72f30ef8e7bf8</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>2 ctw Oval Fancy Blue Lab Grown Diamond Framed Three Stone Engagement Ring</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05872BLU/medium/RIGTXR05872BLU-WY-OV-WH-200-M0.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIGTXR05872BLU/medium/RIGTXR05872BLU-WY-OV-WH-200-M1.jpg, https://media.grownbrilliance.com/a2c5372a-e16a-4ea3-b361-da9fdc89a59f/https://images.grownbrilliance.com/productimages/RIG0625X1/medium/RIG0625X1-C075SO-GW-OV.jpg</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>